<commit_message>
take off year and region from fluxGenerator class. Add Prospective class. Add Nitrogen content un GRAFS_data.xlsx
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\informatique\Donnees\GRAFS-E\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2263F683-4EDD-48C7-9D35-25E7E3599F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B3D338E-9EF1-4A98-B5B4-ECB7AC75B108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4800" yWindow="2840" windowWidth="14400" windowHeight="7360" activeTab="1" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Surf N org" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="87">
   <si>
     <t>Culture</t>
   </si>
@@ -294,13 +294,16 @@
   </si>
   <si>
     <t>N-N2O EM. slurry indoor</t>
+  </si>
+  <si>
+    <t>Nitrogen Content (%)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -313,6 +316,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -335,10 +343,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -653,13 +667,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{973E28D2-5D19-4409-920F-79B00DDA2ABC}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.7265625" customWidth="1"/>
+    <col min="4" max="4" width="19.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -669,64 +684,88 @@
       <c r="C1" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
         <v>0.12</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D2" s="3">
+        <v>1.95</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>39</v>
       </c>
       <c r="B3">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D3" s="3">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4">
         <v>0.13</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D4" s="3">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D5" s="3">
+        <v>2.08</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D6" s="3">
+        <v>1.52</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D7" s="3">
+        <v>1.07</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D8" s="3">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -736,48 +775,66 @@
       <c r="C9" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D9" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>9</v>
       </c>
       <c r="B10">
         <v>0.33</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D10" s="3">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11">
         <v>0.16</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D11" s="3">
+        <v>1.96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>11</v>
       </c>
       <c r="B12">
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D12" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>12</v>
       </c>
       <c r="B13">
         <v>0.56000000000000005</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D13" s="4">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>13</v>
       </c>
       <c r="B14">
         <v>0.35</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D14" s="3">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -787,8 +844,11 @@
       <c r="C15" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D15" s="3">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -798,173 +858,239 @@
       <c r="C16" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D16" s="3">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>16</v>
       </c>
       <c r="B17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D17" s="3">
+        <v>0.20799999999999999</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>40</v>
       </c>
       <c r="B18">
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D18" s="3">
+        <v>0.25600000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>17</v>
       </c>
       <c r="B19">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D19" s="3">
+        <v>0.23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>18</v>
       </c>
       <c r="B20">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D20" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>19</v>
       </c>
       <c r="B21">
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D21" s="3">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>20</v>
       </c>
       <c r="B22">
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D22" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>21</v>
       </c>
       <c r="B23">
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D23" s="3">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>22</v>
       </c>
       <c r="B24">
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D24" s="3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>23</v>
       </c>
       <c r="B25">
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D25" s="3">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>24</v>
       </c>
       <c r="B26">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D26" s="3">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>25</v>
       </c>
       <c r="B27">
         <v>0</v>
       </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D27" s="3">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>26</v>
       </c>
       <c r="B28">
         <v>0.38</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D28" s="3">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>27</v>
       </c>
       <c r="B29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D29" s="3">
+        <v>0.67</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>28</v>
       </c>
       <c r="B30">
         <v>0.08</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D30" s="3">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>30</v>
       </c>
       <c r="B31">
         <v>0.08</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D31" s="3">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>29</v>
       </c>
       <c r="B32">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D32" s="3">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>31</v>
       </c>
       <c r="B33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D33" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>32</v>
       </c>
       <c r="B34">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D34" s="3">
+        <v>0.36</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>33</v>
       </c>
       <c r="B35">
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D35" s="3">
+        <v>2.8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>34</v>
       </c>
       <c r="B36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D36" s="3">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>41</v>
       </c>
       <c r="B37">
         <v>0.25</v>
+      </c>
+      <c r="D37" s="3">
+        <v>2.0499999999999998</v>
       </c>
     </row>
   </sheetData>
@@ -1241,10 +1367,10 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="5.7265625" customWidth="1"/>
-    <col min="3" max="3" width="4.6328125" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" customWidth="1"/>
     <col min="4" max="4" width="5.7265625" customWidth="1"/>
-    <col min="5" max="5" width="3.90625" customWidth="1"/>
-    <col min="6" max="6" width="4.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.90625" customWidth="1"/>
+    <col min="6" max="6" width="14" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Change cultures to crops in area tab. Finish initial update on Cultures and Elevage class.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B3D338E-9EF1-4A98-B5B4-ECB7AC75B108}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4773AA81-69B3-49C0-B523-BDF538730BCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="Surf N org" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="89">
   <si>
     <t>Culture</t>
   </si>
@@ -56,9 +56,6 @@
     <t>Grain maize</t>
   </si>
   <si>
-    <t>Rice</t>
-  </si>
-  <si>
     <t>Other cereals</t>
   </si>
   <si>
@@ -297,6 +294,15 @@
   </si>
   <si>
     <t>Nitrogen Content (%)</t>
+  </si>
+  <si>
+    <t>% edible</t>
+  </si>
+  <si>
+    <t>% non edible</t>
+  </si>
+  <si>
+    <t>rice</t>
   </si>
 </sst>
 </file>
@@ -682,10 +688,10 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
@@ -701,7 +707,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B3">
         <v>0.03</v>
@@ -745,7 +751,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>88</v>
       </c>
       <c r="B7">
         <v>0.03</v>
@@ -756,7 +762,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8">
         <v>0.03</v>
@@ -767,13 +773,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9">
         <v>0.1</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D9" s="3">
         <v>0.5</v>
@@ -781,7 +787,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10">
         <v>0.33</v>
@@ -792,7 +798,7 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11">
         <v>0.16</v>
@@ -803,7 +809,7 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -814,7 +820,7 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13">
         <v>0.56000000000000005</v>
@@ -825,7 +831,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14">
         <v>0.35</v>
@@ -836,13 +842,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <v>0.45</v>
       </c>
       <c r="C15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D15" s="3">
         <v>3.6</v>
@@ -850,13 +856,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B16">
         <v>0</v>
       </c>
       <c r="C16" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D16" s="3">
         <v>3.6</v>
@@ -864,7 +870,7 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -875,7 +881,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -886,7 +892,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -897,7 +903,7 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -908,7 +914,7 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -919,7 +925,7 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -930,7 +936,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -941,7 +947,7 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -952,7 +958,7 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -963,7 +969,7 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B26">
         <v>0.82</v>
@@ -974,7 +980,7 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -985,7 +991,7 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B28">
         <v>0.38</v>
@@ -996,7 +1002,7 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -1007,7 +1013,7 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B30">
         <v>0.08</v>
@@ -1018,7 +1024,7 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31">
         <v>0.08</v>
@@ -1029,7 +1035,7 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B32">
         <v>0</v>
@@ -1040,7 +1046,7 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -1051,7 +1057,7 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B34">
         <v>0</v>
@@ -1062,7 +1068,7 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B35">
         <v>0</v>
@@ -1073,7 +1079,7 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B36">
         <v>0</v>
@@ -1084,7 +1090,7 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B37">
         <v>0.25</v>
@@ -1100,7 +1106,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12223D9-0A39-4CC4-B45B-34CE66BF62BA}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="22.36328125" customWidth="1"/>
@@ -1113,41 +1119,47 @@
     <col min="9" max="9" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H1" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J1" t="s">
+        <v>81</v>
+      </c>
+      <c r="K1" t="s">
+        <v>86</v>
+      </c>
+      <c r="L1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>42</v>
-      </c>
-      <c r="B1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1" t="s">
-        <v>84</v>
-      </c>
-      <c r="G1" t="s">
-        <v>83</v>
-      </c>
-      <c r="H1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I1" t="s">
-        <v>81</v>
-      </c>
-      <c r="J1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>43</v>
       </c>
       <c r="B2">
         <f>1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -1179,10 +1191,16 @@
         <f>G2*5</f>
         <v>0.1</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K2">
+        <v>2.2700000000000001E-2</v>
+      </c>
+      <c r="L2">
+        <v>2.7699999999999999E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3">
         <f>1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -1214,10 +1232,16 @@
         <f t="shared" ref="J3:J7" si="1">G3*5</f>
         <v>0.05</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K3">
+        <v>2.12E-2</v>
+      </c>
+      <c r="L3">
+        <v>2.5600000000000001E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B4">
         <f t="shared" ref="B4:B7" si="2">1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -1249,10 +1273,16 @@
         <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K4">
+        <v>2.12E-2</v>
+      </c>
+      <c r="L4">
+        <v>2.5600000000000001E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B5">
         <f t="shared" si="2"/>
@@ -1284,10 +1314,16 @@
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K5">
+        <v>2.8299999999999999E-2</v>
+      </c>
+      <c r="L5">
+        <v>1.95E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6">
         <f>1-(1-0.5)*(1-0.2)*(1-0.2)</f>
@@ -1319,10 +1355,16 @@
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K6">
+        <v>2.07E-2</v>
+      </c>
+      <c r="L6">
+        <v>2.8299999999999999E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B7">
         <f t="shared" si="2"/>
@@ -1353,6 +1395,12 @@
       <c r="J7">
         <f t="shared" si="1"/>
         <v>0.05</v>
+      </c>
+      <c r="K7">
+        <v>2.2700000000000001E-2</v>
+      </c>
+      <c r="L7">
+        <v>2.7699999999999999E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1375,31 +1423,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" t="s">
         <v>51</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>52</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>53</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>54</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" t="s">
         <v>56</v>
       </c>
-      <c r="G1" t="s">
-        <v>57</v>
-      </c>
       <c r="H1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I1" t="s">
         <v>77</v>
-      </c>
-      <c r="I1" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -1425,7 +1473,7 @@
         <v>54417</v>
       </c>
       <c r="H2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I2" s="1">
         <f>2*14/(2*14+16)*(0.01164*B2+0.00594*C2+0.00594*F2)/(B2+C2+F2)*100</f>
@@ -1455,7 +1503,7 @@
         <v>266265</v>
       </c>
       <c r="H3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I3" s="1">
         <f t="shared" ref="I3:I24" si="0">2*14/(2*14+16)*(0.01164*B3+0.00594*C3+0.00594*F3)/(B3+C3+F3)*100</f>
@@ -1485,7 +1533,7 @@
         <v>168251</v>
       </c>
       <c r="H4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I4" s="1">
         <f t="shared" si="0"/>
@@ -1515,7 +1563,7 @@
         <v>80548</v>
       </c>
       <c r="H5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I5" s="1">
         <f t="shared" si="0"/>
@@ -1545,7 +1593,7 @@
         <v>256528</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I6" s="1">
         <f t="shared" si="0"/>
@@ -1575,7 +1623,7 @@
         <v>74606</v>
       </c>
       <c r="H7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I7" s="1">
         <f t="shared" si="0"/>
@@ -1605,7 +1653,7 @@
         <v>96358</v>
       </c>
       <c r="H8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I8" s="1">
         <f t="shared" si="0"/>
@@ -1635,7 +1683,7 @@
         <v>87002</v>
       </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" si="0"/>
@@ -1665,7 +1713,7 @@
         <v>116150</v>
       </c>
       <c r="H10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I10" s="1">
         <f t="shared" si="0"/>
@@ -1695,7 +1743,7 @@
         <v>35716</v>
       </c>
       <c r="H11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I11" s="1">
         <f t="shared" si="0"/>
@@ -1725,7 +1773,7 @@
         <v>29157</v>
       </c>
       <c r="H12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I12" s="1">
         <f t="shared" si="0"/>
@@ -1755,7 +1803,7 @@
         <v>141243</v>
       </c>
       <c r="H13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I13" s="1">
         <f t="shared" si="0"/>
@@ -1785,7 +1833,7 @@
         <v>111801</v>
       </c>
       <c r="H14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I14" s="1">
         <f t="shared" si="0"/>
@@ -1815,7 +1863,7 @@
         <v>184174</v>
       </c>
       <c r="H15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I15" s="1">
         <f t="shared" si="0"/>
@@ -1845,7 +1893,7 @@
         <v>133267</v>
       </c>
       <c r="H16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I16" s="1">
         <f t="shared" si="0"/>
@@ -1875,7 +1923,7 @@
         <v>135672</v>
       </c>
       <c r="H17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I17" s="1">
         <f t="shared" si="0"/>
@@ -1905,7 +1953,7 @@
         <v>18541</v>
       </c>
       <c r="H18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I18" s="1">
         <f t="shared" si="0"/>
@@ -1935,7 +1983,7 @@
         <v>66736</v>
       </c>
       <c r="H19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I19" s="1">
         <f t="shared" si="0"/>
@@ -1965,7 +2013,7 @@
         <v>50349</v>
       </c>
       <c r="H20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I20" s="1">
         <f>2*14/(2*14+16)*(0.01164*B20+0.00594*C20+0.00594*F20)/(B20+C20+F20)*100</f>
@@ -1995,7 +2043,7 @@
         <v>31445</v>
       </c>
       <c r="H21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I21" s="1">
         <f t="shared" si="0"/>
@@ -2025,7 +2073,7 @@
         <v>21502</v>
       </c>
       <c r="H22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I22" s="1">
         <f t="shared" si="0"/>
@@ -2044,7 +2092,7 @@
       </c>
       <c r="F23" s="2"/>
       <c r="H23" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I23" s="1">
         <f t="shared" si="0"/>
@@ -2053,7 +2101,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B24">
         <v>924490</v>
@@ -2074,7 +2122,7 @@
         <v>2205890</v>
       </c>
       <c r="H24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I24" s="1">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
change other oil crops to oleaginous. Add global data columns in GRAFS_data. Add many early computation of df_elevage in create_elevage_dataframe. Correction of mismatch between slurry and manure FE coef.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4773AA81-69B3-49C0-B523-BDF538730BCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC15F38-4956-4666-A143-E5C6689C63A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="1" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
-    <sheet name="Surf N org" sheetId="1" r:id="rId1"/>
+    <sheet name="crops" sheetId="1" r:id="rId1"/>
     <sheet name="Volatilisation" sheetId="2" r:id="rId2"/>
     <sheet name="N_syn" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="100">
   <si>
     <t>Culture</t>
   </si>
@@ -303,13 +303,46 @@
   </si>
   <si>
     <t>rice</t>
+  </si>
+  <si>
+    <t>Seed input (kt seeds/kt Ymax)</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>N fixation coef (kgN/kgN)</t>
+  </si>
+  <si>
+    <t>cereals (excluding rice)</t>
+  </si>
+  <si>
+    <t>oleaginous</t>
+  </si>
+  <si>
+    <t>leguminous</t>
+  </si>
+  <si>
+    <t>roots</t>
+  </si>
+  <si>
+    <t>forages</t>
+  </si>
+  <si>
+    <t>grasslands</t>
+  </si>
+  <si>
+    <t>fruits and vegetables</t>
+  </si>
+  <si>
+    <t>%N dairy</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -325,6 +358,18 @@
     </font>
     <font>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -346,10 +391,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -359,9 +405,21 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Texte explicatif 6" xfId="1" xr:uid="{FA142338-8601-4E55-AA3D-600E38F000DF}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -673,14 +731,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{973E28D2-5D19-4409-920F-79B00DDA2ABC}">
-  <dimension ref="A1:D37"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.7265625" customWidth="1"/>
     <col min="4" max="4" width="19.6328125" customWidth="1"/>
+    <col min="5" max="5" width="14.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -693,8 +752,17 @@
       <c r="D1" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -704,8 +772,18 @@
       <c r="D2" s="3">
         <v>1.95</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E2" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G2" s="9">
+        <v>0</v>
+      </c>
+      <c r="H2" s="7"/>
+    </row>
+    <row r="3" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -715,8 +793,18 @@
       <c r="D3" s="3">
         <v>1.76</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E3" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G3" s="9">
+        <v>0</v>
+      </c>
+      <c r="H3" s="7"/>
+    </row>
+    <row r="4" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -726,8 +814,18 @@
       <c r="D4" s="3">
         <v>1.76</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E4" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G4" s="9">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7"/>
+    </row>
+    <row r="5" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -737,8 +835,18 @@
       <c r="D5" s="3">
         <v>2.08</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E5" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G5" s="9">
+        <v>0</v>
+      </c>
+      <c r="H5" s="7"/>
+    </row>
+    <row r="6" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -748,8 +856,18 @@
       <c r="D6" s="3">
         <v>1.52</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E6" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G6" s="9">
+        <v>0</v>
+      </c>
+      <c r="H6" s="7"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>88</v>
       </c>
@@ -759,8 +877,18 @@
       <c r="D7" s="3">
         <v>1.07</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E7" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>88</v>
+      </c>
+      <c r="G7" s="9">
+        <v>0</v>
+      </c>
+      <c r="H7" s="7"/>
+    </row>
+    <row r="8" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -770,8 +898,18 @@
       <c r="D8" s="3">
         <v>1.8</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E8" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" s="9">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -784,8 +922,18 @@
       <c r="D9" s="3">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E9" s="5">
+        <v>0</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G9" s="9">
+        <v>0</v>
+      </c>
+      <c r="H9" s="7"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -795,8 +943,18 @@
       <c r="D10" s="3">
         <v>3.5</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E10" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="G10" s="9">
+        <v>0</v>
+      </c>
+      <c r="H10" s="7"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -806,30 +964,58 @@
       <c r="D11" s="3">
         <v>1.96</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E11" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="G11" s="9">
+        <v>0</v>
+      </c>
+      <c r="H11" s="7"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
       <c r="B12">
         <v>0</v>
       </c>
-      <c r="D12" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D12" s="4">
+        <v>3.5</v>
+      </c>
+      <c r="E12" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="G12" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
       <c r="B13">
         <v>0.56000000000000005</v>
       </c>
-      <c r="D13" s="4">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D13" s="3">
+        <v>0.20799999999999999</v>
+      </c>
+      <c r="E13" s="5">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="G13" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -837,10 +1023,19 @@
         <v>0.35</v>
       </c>
       <c r="D14" s="3">
-        <v>3.5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.25600000000000001</v>
+      </c>
+      <c r="E14" s="5">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="G14" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -851,10 +1046,19 @@
         <v>36</v>
       </c>
       <c r="D15" s="3">
-        <v>3.6</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.23</v>
+      </c>
+      <c r="E15" s="5">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="G15" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="25" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -867,8 +1071,17 @@
       <c r="D16" s="3">
         <v>3.6</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E16" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G16" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="25" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -876,10 +1089,19 @@
         <v>0</v>
       </c>
       <c r="D17" s="3">
-        <v>0.20799999999999999</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+        <v>2</v>
+      </c>
+      <c r="E17" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="25" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -887,10 +1109,19 @@
         <v>0</v>
       </c>
       <c r="D18" s="3">
-        <v>0.25600000000000001</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.18</v>
+      </c>
+      <c r="E18" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G18" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="25" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -898,10 +1129,19 @@
         <v>0</v>
       </c>
       <c r="D19" s="3">
-        <v>0.23</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.36</v>
+      </c>
+      <c r="E19" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G19" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="25" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -909,10 +1149,19 @@
         <v>0</v>
       </c>
       <c r="D20" s="3">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.22</v>
+      </c>
+      <c r="E20" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G20" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="25" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -920,10 +1169,19 @@
         <v>0</v>
       </c>
       <c r="D21" s="3">
-        <v>1.5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.1</v>
+      </c>
+      <c r="E21" s="5">
+        <v>0</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G21" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="25" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -931,10 +1189,19 @@
         <v>0</v>
       </c>
       <c r="D22" s="3">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.67</v>
+      </c>
+      <c r="E22" s="5">
+        <v>0</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G22" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="25" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -942,10 +1209,19 @@
         <v>0</v>
       </c>
       <c r="D23" s="3">
-        <v>3.6</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.18</v>
+      </c>
+      <c r="E23" s="5">
+        <v>0</v>
+      </c>
+      <c r="F23" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G23" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -953,10 +1229,19 @@
         <v>0</v>
       </c>
       <c r="D24" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.35</v>
+      </c>
+      <c r="E24" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F24" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="G24" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -964,10 +1249,19 @@
         <v>0</v>
       </c>
       <c r="D25" s="3">
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.35</v>
+      </c>
+      <c r="E25" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="G25" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -975,10 +1269,19 @@
         <v>0.82</v>
       </c>
       <c r="D26" s="3">
-        <v>0.36</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="E26" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G26" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>24</v>
       </c>
@@ -986,10 +1289,19 @@
         <v>0</v>
       </c>
       <c r="D27" s="3">
-        <v>0.22</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.36</v>
+      </c>
+      <c r="E27" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F27" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G27" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>25</v>
       </c>
@@ -997,10 +1309,19 @@
         <v>0.38</v>
       </c>
       <c r="D28" s="3">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+        <v>1.25</v>
+      </c>
+      <c r="E28" s="6">
+        <v>0</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G28" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>26</v>
       </c>
@@ -1008,10 +1329,19 @@
         <v>0</v>
       </c>
       <c r="D29" s="3">
-        <v>0.67</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+        <v>3.5</v>
+      </c>
+      <c r="E29" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G29" s="9">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>27</v>
       </c>
@@ -1019,10 +1349,19 @@
         <v>0.08</v>
       </c>
       <c r="D30" s="3">
-        <v>0.18</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+        <v>3.6</v>
+      </c>
+      <c r="E30" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G30" s="9">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -1030,10 +1369,19 @@
         <v>0.08</v>
       </c>
       <c r="D31" s="3">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.5</v>
+      </c>
+      <c r="E31" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G31" s="9">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>28</v>
       </c>
@@ -1041,10 +1389,19 @@
         <v>0</v>
       </c>
       <c r="D32" s="3">
-        <v>0.35</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+        <v>3.6</v>
+      </c>
+      <c r="E32" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G32" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>30</v>
       </c>
@@ -1052,10 +1409,19 @@
         <v>0</v>
       </c>
       <c r="D33" s="3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+        <v>1.5</v>
+      </c>
+      <c r="E33" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G33" s="9">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>31</v>
       </c>
@@ -1063,10 +1429,19 @@
         <v>0</v>
       </c>
       <c r="D34" s="3">
-        <v>0.36</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.5</v>
+      </c>
+      <c r="E34" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G34" s="9">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>32</v>
       </c>
@@ -1074,10 +1449,19 @@
         <v>0</v>
       </c>
       <c r="D35" s="3">
-        <v>2.8</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="E35" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>94</v>
+      </c>
+      <c r="G35" s="9">
+        <v>1.23</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>33</v>
       </c>
@@ -1085,10 +1469,19 @@
         <v>0</v>
       </c>
       <c r="D36" s="3">
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+        <v>2.8</v>
+      </c>
+      <c r="E36" s="5">
+        <v>0</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G36" s="9">
+        <v>1.47</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>40</v>
       </c>
@@ -1097,6 +1490,15 @@
       </c>
       <c r="D37" s="3">
         <v>2.0499999999999998</v>
+      </c>
+      <c r="E37" s="6">
+        <v>0</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G37" s="9">
+        <v>0.36749999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1106,7 +1508,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12223D9-0A39-4CC4-B45B-34CE66BF62BA}">
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="22.36328125" customWidth="1"/>
@@ -1119,7 +1521,7 @@
     <col min="9" max="9" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>41</v>
       </c>
@@ -1156,8 +1558,11 @@
       <c r="L1" t="s">
         <v>87</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>42</v>
       </c>
@@ -1197,8 +1602,11 @@
       <c r="L2">
         <v>2.7699999999999999E-2</v>
       </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M2">
+        <v>5.3E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>43</v>
       </c>
@@ -1238,8 +1646,11 @@
       <c r="L3">
         <v>2.5600000000000001E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M3">
+        <v>9.4000000000000004E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>44</v>
       </c>
@@ -1279,8 +1690,11 @@
       <c r="L4">
         <v>2.5600000000000001E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M4">
+        <v>9.4000000000000004E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>45</v>
       </c>
@@ -1320,8 +1734,11 @@
       <c r="L5">
         <v>1.95E-2</v>
       </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>46</v>
       </c>
@@ -1361,8 +1778,11 @@
       <c r="L6">
         <v>2.8299999999999999E-2</v>
       </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="M6">
+        <v>1.7899999999999999E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>47</v>
       </c>
@@ -1401,6 +1821,9 @@
       </c>
       <c r="L7">
         <v>2.7699999999999999E-2</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add atmospheric deposition. Add Nitrogen requirement for plants. Add test_plot.py for new kind of plots (temporary)
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FC15F38-4956-4666-A143-E5C6689C63A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0A1AA82-0C0B-42B1-963A-AAC9C6EDC968}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="103">
   <si>
     <t>Culture</t>
   </si>
@@ -336,6 +336,15 @@
   </si>
   <si>
     <t>%N dairy</t>
+  </si>
+  <si>
+    <t>Surface Fertilization Need (kgN/ha)</t>
+  </si>
+  <si>
+    <t>Fertilization Need (kgN/qtl)</t>
+  </si>
+  <si>
+    <t>Rice</t>
   </si>
 </sst>
 </file>
@@ -368,10 +377,10 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -407,15 +416,13 @@
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -731,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{973E28D2-5D19-4409-920F-79B00DDA2ABC}">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.7265625" customWidth="1"/>
@@ -739,7 +746,7 @@
     <col min="5" max="5" width="14.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -761,8 +768,14 @@
       <c r="G1" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="H1" t="s">
+        <v>101</v>
+      </c>
+      <c r="I1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -775,15 +788,22 @@
       <c r="E2" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="F2" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G2" s="9">
-        <v>0</v>
-      </c>
-      <c r="H2" s="7"/>
-    </row>
-    <row r="3" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="G2" s="8">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="I2" s="9">
+        <v>0</v>
+      </c>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+    </row>
+    <row r="3" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -796,15 +816,22 @@
       <c r="E3" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G3" s="9">
-        <v>0</v>
-      </c>
-      <c r="H3" s="7"/>
-    </row>
-    <row r="4" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="G3" s="8">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="I3" s="9">
+        <v>0</v>
+      </c>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+    </row>
+    <row r="4" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -817,15 +844,22 @@
       <c r="E4" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G4" s="9">
-        <v>0</v>
-      </c>
-      <c r="H4" s="7"/>
-    </row>
-    <row r="5" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="G4" s="8">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="I4" s="9">
+        <v>0</v>
+      </c>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+    </row>
+    <row r="5" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -838,15 +872,22 @@
       <c r="E5" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G5" s="9">
-        <v>0</v>
-      </c>
-      <c r="H5" s="7"/>
-    </row>
-    <row r="6" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="G5" s="8">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="I5" s="9">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+    </row>
+    <row r="6" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -859,17 +900,24 @@
       <c r="E6" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F6" s="8" t="s">
+      <c r="F6" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G6" s="9">
-        <v>0</v>
-      </c>
-      <c r="H6" s="7"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G6" s="8">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="I6" s="9">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="B7">
         <v>0.03</v>
@@ -880,15 +928,22 @@
       <c r="E7" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="G7" s="9">
-        <v>0</v>
-      </c>
-      <c r="H7" s="7"/>
-    </row>
-    <row r="8" spans="1:8" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="G7" s="8">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3">
+        <v>0</v>
+      </c>
+      <c r="I7" s="9">
+        <v>125</v>
+      </c>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+    </row>
+    <row r="8" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -901,15 +956,22 @@
       <c r="E8" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="F8" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G8" s="9">
-        <v>0</v>
-      </c>
-      <c r="H8" s="7"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G8" s="8">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3">
+        <v>2.6</v>
+      </c>
+      <c r="I8" s="9">
+        <v>0</v>
+      </c>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -925,15 +987,22 @@
       <c r="E9" s="5">
         <v>0</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="F9" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G9" s="9">
-        <v>0</v>
-      </c>
-      <c r="H9" s="7"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G9" s="8">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>3</v>
+      </c>
+      <c r="I9" s="9">
+        <v>0</v>
+      </c>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -946,15 +1015,22 @@
       <c r="E10" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G10" s="9">
-        <v>0</v>
-      </c>
-      <c r="H10" s="7"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G10" s="8">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3">
+        <v>7</v>
+      </c>
+      <c r="I10" s="9">
+        <v>0</v>
+      </c>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -967,15 +1043,22 @@
       <c r="E11" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="F11" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G11" s="9">
-        <v>0</v>
-      </c>
-      <c r="H11" s="7"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G11" s="8">
+        <v>0</v>
+      </c>
+      <c r="H11" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="I11" s="9">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -988,14 +1071,22 @@
       <c r="E12" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="F12" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G12" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G12" s="8">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9">
+        <v>5</v>
+      </c>
+      <c r="I12" s="9">
+        <v>0</v>
+      </c>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1008,14 +1099,22 @@
       <c r="E13" s="5">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G13" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G13" s="8">
+        <v>0</v>
+      </c>
+      <c r="H13" s="9">
+        <v>0</v>
+      </c>
+      <c r="I13" s="9">
+        <v>220</v>
+      </c>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1028,14 +1127,22 @@
       <c r="E14" s="5">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="F14" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G14" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G14" s="8">
+        <v>0</v>
+      </c>
+      <c r="H14" s="9">
+        <v>0</v>
+      </c>
+      <c r="I14" s="9">
+        <v>220</v>
+      </c>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1051,14 +1158,22 @@
       <c r="E15" s="5">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="F15" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G15" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" ht="25" x14ac:dyDescent="0.35">
+      <c r="G15" s="8">
+        <v>0</v>
+      </c>
+      <c r="H15" s="9">
+        <v>0</v>
+      </c>
+      <c r="I15" s="9">
+        <v>220</v>
+      </c>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+    </row>
+    <row r="16" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1074,14 +1189,22 @@
       <c r="E16" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="F16" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G16" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="25" x14ac:dyDescent="0.35">
+      <c r="G16" s="8">
+        <v>0</v>
+      </c>
+      <c r="H16" s="9">
+        <v>0</v>
+      </c>
+      <c r="I16" s="9">
+        <v>50</v>
+      </c>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+    </row>
+    <row r="17" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -1094,14 +1217,22 @@
       <c r="E17" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="F17" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G17" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="25" x14ac:dyDescent="0.35">
+      <c r="G17" s="8">
+        <v>0</v>
+      </c>
+      <c r="H17" s="9">
+        <v>0</v>
+      </c>
+      <c r="I17" s="9">
+        <v>100</v>
+      </c>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+    </row>
+    <row r="18" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -1114,14 +1245,22 @@
       <c r="E18" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F18" s="8" t="s">
+      <c r="F18" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G18" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="25" x14ac:dyDescent="0.35">
+      <c r="G18" s="8">
+        <v>0</v>
+      </c>
+      <c r="H18" s="9">
+        <v>0</v>
+      </c>
+      <c r="I18" s="9">
+        <v>180</v>
+      </c>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+    </row>
+    <row r="19" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>16</v>
       </c>
@@ -1134,14 +1273,22 @@
       <c r="E19" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F19" s="8" t="s">
+      <c r="F19" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G19" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" ht="25" x14ac:dyDescent="0.35">
+      <c r="G19" s="8">
+        <v>0</v>
+      </c>
+      <c r="H19" s="9">
+        <v>0</v>
+      </c>
+      <c r="I19" s="9">
+        <v>300</v>
+      </c>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+    </row>
+    <row r="20" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>17</v>
       </c>
@@ -1154,14 +1301,22 @@
       <c r="E20" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F20" s="8" t="s">
+      <c r="F20" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G20" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" ht="25" x14ac:dyDescent="0.35">
+      <c r="G20" s="8">
+        <v>0</v>
+      </c>
+      <c r="H20" s="9">
+        <v>0</v>
+      </c>
+      <c r="I20" s="9">
+        <v>150</v>
+      </c>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+    </row>
+    <row r="21" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>18</v>
       </c>
@@ -1174,14 +1329,22 @@
       <c r="E21" s="5">
         <v>0</v>
       </c>
-      <c r="F21" s="8" t="s">
+      <c r="F21" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G21" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" ht="25" x14ac:dyDescent="0.35">
+      <c r="G21" s="8">
+        <v>0</v>
+      </c>
+      <c r="H21" s="9">
+        <v>0</v>
+      </c>
+      <c r="I21" s="9">
+        <v>100</v>
+      </c>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+    </row>
+    <row r="22" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>19</v>
       </c>
@@ -1194,14 +1357,22 @@
       <c r="E22" s="5">
         <v>0</v>
       </c>
-      <c r="F22" s="8" t="s">
+      <c r="F22" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G22" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" ht="25" x14ac:dyDescent="0.35">
+      <c r="G22" s="8">
+        <v>0</v>
+      </c>
+      <c r="H22" s="9">
+        <v>0</v>
+      </c>
+      <c r="I22" s="9">
+        <v>80</v>
+      </c>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+    </row>
+    <row r="23" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>20</v>
       </c>
@@ -1214,14 +1385,22 @@
       <c r="E23" s="5">
         <v>0</v>
       </c>
-      <c r="F23" s="8" t="s">
+      <c r="F23" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="G23" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G23" s="8">
+        <v>0</v>
+      </c>
+      <c r="H23" s="9">
+        <v>0</v>
+      </c>
+      <c r="I23" s="9">
+        <v>130</v>
+      </c>
+      <c r="J23" s="9"/>
+      <c r="K23" s="9"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>21</v>
       </c>
@@ -1234,14 +1413,22 @@
       <c r="E24" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F24" s="8" t="s">
+      <c r="F24" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G24" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G24" s="8">
+        <v>0</v>
+      </c>
+      <c r="H24" s="9">
+        <v>0</v>
+      </c>
+      <c r="I24" s="9">
+        <v>120</v>
+      </c>
+      <c r="J24" s="9"/>
+      <c r="K24" s="9"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -1254,14 +1441,22 @@
       <c r="E25" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F25" s="8" t="s">
+      <c r="F25" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G25" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G25" s="8">
+        <v>0</v>
+      </c>
+      <c r="H25" s="9">
+        <v>0</v>
+      </c>
+      <c r="I25" s="9">
+        <v>60</v>
+      </c>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>23</v>
       </c>
@@ -1274,14 +1469,22 @@
       <c r="E26" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F26" s="8" t="s">
+      <c r="F26" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G26" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G26" s="8">
+        <v>0</v>
+      </c>
+      <c r="H26" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="I26" s="9">
+        <v>0</v>
+      </c>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>24</v>
       </c>
@@ -1294,14 +1497,22 @@
       <c r="E27" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F27" s="8" t="s">
+      <c r="F27" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G27" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G27" s="8">
+        <v>0</v>
+      </c>
+      <c r="H27" s="9">
+        <v>0</v>
+      </c>
+      <c r="I27" s="9">
+        <v>300</v>
+      </c>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>25</v>
       </c>
@@ -1314,14 +1525,22 @@
       <c r="E28" s="6">
         <v>0</v>
       </c>
-      <c r="F28" s="8" t="s">
+      <c r="F28" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G28" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G28" s="8">
+        <v>0</v>
+      </c>
+      <c r="H28" s="9">
+        <v>0</v>
+      </c>
+      <c r="I28" s="9">
+        <v>150</v>
+      </c>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>26</v>
       </c>
@@ -1334,14 +1553,22 @@
       <c r="E29" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F29" s="8" t="s">
+      <c r="F29" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G29" s="9">
+      <c r="G29" s="8">
         <v>1.23</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H29" s="9">
+        <v>0</v>
+      </c>
+      <c r="I29" s="9">
+        <v>0</v>
+      </c>
+      <c r="J29" s="9"/>
+      <c r="K29" s="9"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>27</v>
       </c>
@@ -1354,14 +1581,22 @@
       <c r="E30" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F30" s="8" t="s">
+      <c r="F30" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G30" s="9">
+      <c r="G30" s="8">
         <v>1.23</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H30" s="9">
+        <v>0</v>
+      </c>
+      <c r="I30" s="9">
+        <v>0</v>
+      </c>
+      <c r="J30" s="9"/>
+      <c r="K30" s="9"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -1374,14 +1609,22 @@
       <c r="E31" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F31" s="8" t="s">
+      <c r="F31" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G31" s="9">
+      <c r="G31" s="8">
         <v>1.23</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H31" s="9">
+        <v>0</v>
+      </c>
+      <c r="I31" s="9">
+        <v>0</v>
+      </c>
+      <c r="J31" s="9"/>
+      <c r="K31" s="9"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>28</v>
       </c>
@@ -1394,14 +1637,22 @@
       <c r="E32" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F32" s="8" t="s">
+      <c r="F32" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G32" s="9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="G32" s="8">
+        <v>0</v>
+      </c>
+      <c r="H32" s="9">
+        <v>0</v>
+      </c>
+      <c r="I32" s="9">
+        <v>0</v>
+      </c>
+      <c r="J32" s="9"/>
+      <c r="K32" s="9"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>30</v>
       </c>
@@ -1414,14 +1665,22 @@
       <c r="E33" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F33" s="8" t="s">
+      <c r="F33" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G33" s="9">
+      <c r="G33" s="8">
         <v>1.23</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H33" s="9">
+        <v>0</v>
+      </c>
+      <c r="I33" s="9">
+        <v>0</v>
+      </c>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>31</v>
       </c>
@@ -1434,14 +1693,22 @@
       <c r="E34" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F34" s="8" t="s">
+      <c r="F34" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G34" s="9">
+      <c r="G34" s="8">
         <v>1.23</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H34" s="9">
+        <v>0</v>
+      </c>
+      <c r="I34" s="9">
+        <v>0</v>
+      </c>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>32</v>
       </c>
@@ -1454,14 +1721,22 @@
       <c r="E35" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F35" s="8" t="s">
+      <c r="F35" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G35" s="9">
+      <c r="G35" s="8">
         <v>1.23</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H35" s="9">
+        <v>0</v>
+      </c>
+      <c r="I35" s="9">
+        <v>0</v>
+      </c>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>33</v>
       </c>
@@ -1474,14 +1749,22 @@
       <c r="E36" s="5">
         <v>0</v>
       </c>
-      <c r="F36" s="8" t="s">
+      <c r="F36" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G36" s="9">
+      <c r="G36" s="8">
         <v>1.47</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H36" s="9">
+        <v>0</v>
+      </c>
+      <c r="I36" s="9">
+        <v>0</v>
+      </c>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>40</v>
       </c>
@@ -1494,12 +1777,20 @@
       <c r="E37" s="6">
         <v>0</v>
       </c>
-      <c r="F37" s="8" t="s">
+      <c r="F37" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="G37" s="9">
+      <c r="G37" s="8">
         <v>0.36749999999999999</v>
       </c>
+      <c r="H37" s="9">
+        <v>0</v>
+      </c>
+      <c r="I37" s="9">
+        <v>150</v>
+      </c>
+      <c r="J37" s="9"/>
+      <c r="K37" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
take off year and region from fluxGenerator class.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -5,15 +5,15 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\informatique\Donnees\GRAFS-E\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2263F683-4EDD-48C7-9D35-25E7E3599F34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FD0152E-33FE-4B40-93D1-7F82A48438A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4800" yWindow="2840" windowWidth="14400" windowHeight="7360" activeTab="1" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
-    <sheet name="Surf N org" sheetId="1" r:id="rId1"/>
+    <sheet name="crops" sheetId="1" r:id="rId1"/>
     <sheet name="Volatilisation" sheetId="2" r:id="rId2"/>
     <sheet name="N_syn" sheetId="3" r:id="rId3"/>
   </sheets>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="103">
   <si>
     <t>Culture</t>
   </si>
@@ -56,251 +56,302 @@
     <t>Grain maize</t>
   </si>
   <si>
+    <t>Other cereals</t>
+  </si>
+  <si>
+    <t>Straw</t>
+  </si>
+  <si>
+    <t>Rapeseed</t>
+  </si>
+  <si>
+    <t>Sunflower</t>
+  </si>
+  <si>
+    <t>Other oil crops</t>
+  </si>
+  <si>
+    <t>Sugar beet</t>
+  </si>
+  <si>
+    <t>Potatoes</t>
+  </si>
+  <si>
+    <t>Other roots</t>
+  </si>
+  <si>
+    <t>Dry vegetables</t>
+  </si>
+  <si>
+    <t>Dry fruits</t>
+  </si>
+  <si>
+    <t>Cabbage</t>
+  </si>
+  <si>
+    <t>Leaves vegetables</t>
+  </si>
+  <si>
+    <t>Fruits</t>
+  </si>
+  <si>
+    <t>Olives</t>
+  </si>
+  <si>
+    <t>Citrus</t>
+  </si>
+  <si>
+    <t>Hemp</t>
+  </si>
+  <si>
+    <t>Flax</t>
+  </si>
+  <si>
+    <t>Forage maize</t>
+  </si>
+  <si>
+    <t>Forage cabbages</t>
+  </si>
+  <si>
+    <t>Non-legume temporary meadow</t>
+  </si>
+  <si>
+    <t>Horse beans and faba beans</t>
+  </si>
+  <si>
+    <t>Peas</t>
+  </si>
+  <si>
+    <t>Other protein crops</t>
+  </si>
+  <si>
+    <t>Green peas</t>
+  </si>
+  <si>
+    <t>Dry beans</t>
+  </si>
+  <si>
+    <t>Green beans</t>
+  </si>
+  <si>
+    <t>Soybean</t>
+  </si>
+  <si>
+    <t>Alfalfa and clover</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>Proche de blé…</t>
+  </si>
+  <si>
+    <t>Entre beteraves et PDT</t>
+  </si>
+  <si>
+    <t>Considéré comme une légumineuse</t>
+  </si>
+  <si>
+    <t>Rye</t>
+  </si>
+  <si>
+    <t>Squash and melons</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Natural meadow </t>
+  </si>
+  <si>
+    <t>Elevage</t>
+  </si>
+  <si>
+    <t>bovines</t>
+  </si>
+  <si>
+    <t>ovines</t>
+  </si>
+  <si>
+    <t>caprines</t>
+  </si>
+  <si>
+    <t>porcines</t>
+  </si>
+  <si>
+    <t>poultry</t>
+  </si>
+  <si>
+    <t>equine</t>
+  </si>
+  <si>
+    <t>N-NH3 EM. slurry indoor</t>
+  </si>
+  <si>
+    <t>N-NH3 EM. outdoor</t>
+  </si>
+  <si>
+    <t>Code région</t>
+  </si>
+  <si>
+    <t>Ammonitrates (t/an)</t>
+  </si>
+  <si>
+    <t>Solutions (t/an)</t>
+  </si>
+  <si>
+    <t>Urée (t/an)</t>
+  </si>
+  <si>
+    <t>Autre (t/an)</t>
+  </si>
+  <si>
+    <t>Composés NK, NPK (t/an)</t>
+  </si>
+  <si>
+    <t>Total (t/an)</t>
+  </si>
+  <si>
+    <t>4,3%</t>
+  </si>
+  <si>
+    <t>7,1%</t>
+  </si>
+  <si>
+    <t>5,1%</t>
+  </si>
+  <si>
+    <t>5,0%</t>
+  </si>
+  <si>
+    <t>5,5%</t>
+  </si>
+  <si>
+    <t>3,9%</t>
+  </si>
+  <si>
+    <t>2,8%</t>
+  </si>
+  <si>
+    <t>6,0%</t>
+  </si>
+  <si>
+    <t>5,7%</t>
+  </si>
+  <si>
+    <t>3,8%</t>
+  </si>
+  <si>
+    <t>3,5%</t>
+  </si>
+  <si>
+    <t>3,1%</t>
+  </si>
+  <si>
+    <t>6,2%</t>
+  </si>
+  <si>
+    <t>7,5%</t>
+  </si>
+  <si>
+    <t>6,1%</t>
+  </si>
+  <si>
+    <t>2,5%</t>
+  </si>
+  <si>
+    <t>7,4%</t>
+  </si>
+  <si>
+    <t>France</t>
+  </si>
+  <si>
+    <t>5,3%</t>
+  </si>
+  <si>
+    <t>Volatilisation NH3 (% N épandu)</t>
+  </si>
+  <si>
+    <t>FE indirect N-N2O (%)</t>
+  </si>
+  <si>
+    <t>N-NH3 EM. manure indoor</t>
+  </si>
+  <si>
+    <t>N-N2 EM. slurry indoor</t>
+  </si>
+  <si>
+    <t>N-N2 EM. manure indoor</t>
+  </si>
+  <si>
+    <t>N-N2 EM. outdoor</t>
+  </si>
+  <si>
+    <t>N-N2O EM. outdoor</t>
+  </si>
+  <si>
+    <t>N-N2O EM. manure indoor</t>
+  </si>
+  <si>
+    <t>N-N2O EM. slurry indoor</t>
+  </si>
+  <si>
+    <t>Nitrogen Content (%)</t>
+  </si>
+  <si>
+    <t>% edible</t>
+  </si>
+  <si>
+    <t>% non edible</t>
+  </si>
+  <si>
+    <t>rice</t>
+  </si>
+  <si>
+    <t>Seed input (kt seeds/kt Ymax)</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>N fixation coef (kgN/kgN)</t>
+  </si>
+  <si>
+    <t>cereals (excluding rice)</t>
+  </si>
+  <si>
+    <t>oleaginous</t>
+  </si>
+  <si>
+    <t>leguminous</t>
+  </si>
+  <si>
+    <t>roots</t>
+  </si>
+  <si>
+    <t>forages</t>
+  </si>
+  <si>
+    <t>grasslands</t>
+  </si>
+  <si>
+    <t>fruits and vegetables</t>
+  </si>
+  <si>
+    <t>%N dairy</t>
+  </si>
+  <si>
+    <t>Surface Fertilization Need (kgN/ha)</t>
+  </si>
+  <si>
+    <t>Fertilization Need (kgN/qtl)</t>
+  </si>
+  <si>
     <t>Rice</t>
-  </si>
-  <si>
-    <t>Other cereals</t>
-  </si>
-  <si>
-    <t>Straw</t>
-  </si>
-  <si>
-    <t>Rapeseed</t>
-  </si>
-  <si>
-    <t>Sunflower</t>
-  </si>
-  <si>
-    <t>Other oil crops</t>
-  </si>
-  <si>
-    <t>Sugar beet</t>
-  </si>
-  <si>
-    <t>Potatoes</t>
-  </si>
-  <si>
-    <t>Other roots</t>
-  </si>
-  <si>
-    <t>Dry vegetables</t>
-  </si>
-  <si>
-    <t>Dry fruits</t>
-  </si>
-  <si>
-    <t>Cabbage</t>
-  </si>
-  <si>
-    <t>Leaves vegetables</t>
-  </si>
-  <si>
-    <t>Fruits</t>
-  </si>
-  <si>
-    <t>Olives</t>
-  </si>
-  <si>
-    <t>Citrus</t>
-  </si>
-  <si>
-    <t>Hemp</t>
-  </si>
-  <si>
-    <t>Flax</t>
-  </si>
-  <si>
-    <t>Forage maize</t>
-  </si>
-  <si>
-    <t>Forage cabbages</t>
-  </si>
-  <si>
-    <t>Non-legume temporary meadow</t>
-  </si>
-  <si>
-    <t>Horse beans and faba beans</t>
-  </si>
-  <si>
-    <t>Peas</t>
-  </si>
-  <si>
-    <t>Other protein crops</t>
-  </si>
-  <si>
-    <t>Green peas</t>
-  </si>
-  <si>
-    <t>Dry beans</t>
-  </si>
-  <si>
-    <t>Green beans</t>
-  </si>
-  <si>
-    <t>Soybean</t>
-  </si>
-  <si>
-    <t>Alfalfa and clover</t>
-  </si>
-  <si>
-    <t>Note</t>
-  </si>
-  <si>
-    <t>Proche de blé…</t>
-  </si>
-  <si>
-    <t>Entre beteraves et PDT</t>
-  </si>
-  <si>
-    <t>Considéré comme une légumineuse</t>
-  </si>
-  <si>
-    <t>Rye</t>
-  </si>
-  <si>
-    <t>Squash and melons</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Natural meadow </t>
-  </si>
-  <si>
-    <t>Elevage</t>
-  </si>
-  <si>
-    <t>bovines</t>
-  </si>
-  <si>
-    <t>ovines</t>
-  </si>
-  <si>
-    <t>caprines</t>
-  </si>
-  <si>
-    <t>porcines</t>
-  </si>
-  <si>
-    <t>poultry</t>
-  </si>
-  <si>
-    <t>equine</t>
-  </si>
-  <si>
-    <t>N-NH3 EM. slurry indoor</t>
-  </si>
-  <si>
-    <t>N-NH3 EM. outdoor</t>
-  </si>
-  <si>
-    <t>Code région</t>
-  </si>
-  <si>
-    <t>Ammonitrates (t/an)</t>
-  </si>
-  <si>
-    <t>Solutions (t/an)</t>
-  </si>
-  <si>
-    <t>Urée (t/an)</t>
-  </si>
-  <si>
-    <t>Autre (t/an)</t>
-  </si>
-  <si>
-    <t>Composés NK, NPK (t/an)</t>
-  </si>
-  <si>
-    <t>Total (t/an)</t>
-  </si>
-  <si>
-    <t>4,3%</t>
-  </si>
-  <si>
-    <t>7,1%</t>
-  </si>
-  <si>
-    <t>5,1%</t>
-  </si>
-  <si>
-    <t>5,0%</t>
-  </si>
-  <si>
-    <t>5,5%</t>
-  </si>
-  <si>
-    <t>3,9%</t>
-  </si>
-  <si>
-    <t>2,8%</t>
-  </si>
-  <si>
-    <t>6,0%</t>
-  </si>
-  <si>
-    <t>5,7%</t>
-  </si>
-  <si>
-    <t>3,8%</t>
-  </si>
-  <si>
-    <t>3,5%</t>
-  </si>
-  <si>
-    <t>3,1%</t>
-  </si>
-  <si>
-    <t>6,2%</t>
-  </si>
-  <si>
-    <t>7,5%</t>
-  </si>
-  <si>
-    <t>6,1%</t>
-  </si>
-  <si>
-    <t>2,5%</t>
-  </si>
-  <si>
-    <t>7,4%</t>
-  </si>
-  <si>
-    <t>France</t>
-  </si>
-  <si>
-    <t>5,3%</t>
-  </si>
-  <si>
-    <t>Volatilisation NH3 (% N épandu)</t>
-  </si>
-  <si>
-    <t>FE indirect N-N2O (%)</t>
-  </si>
-  <si>
-    <t>N-NH3 EM. manure indoor</t>
-  </si>
-  <si>
-    <t>N-N2 EM. slurry indoor</t>
-  </si>
-  <si>
-    <t>N-N2 EM. manure indoor</t>
-  </si>
-  <si>
-    <t>N-N2 EM. outdoor</t>
-  </si>
-  <si>
-    <t>N-N2O EM. outdoor</t>
-  </si>
-  <si>
-    <t>N-N2O EM. manure indoor</t>
-  </si>
-  <si>
-    <t>N-N2O EM. slurry indoor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -310,6 +361,23 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -332,16 +400,33 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Texte explicatif 6" xfId="1" xr:uid="{FA142338-8601-4E55-AA3D-600E38F000DF}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -653,13 +738,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{973E28D2-5D19-4409-920F-79B00DDA2ABC}">
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.7265625" customWidth="1"/>
+    <col min="4" max="4" width="19.6328125" customWidth="1"/>
+    <col min="5" max="5" width="14.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -667,305 +754,1043 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+        <v>34</v>
+      </c>
+      <c r="D1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" t="s">
+        <v>91</v>
+      </c>
+      <c r="H1" t="s">
+        <v>101</v>
+      </c>
+      <c r="I1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
       <c r="B2">
         <v>0.12</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D2" s="3">
+        <v>1.95</v>
+      </c>
+      <c r="E2" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G2" s="8">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="I2" s="9">
+        <v>0</v>
+      </c>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+    </row>
+    <row r="3" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B3">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D3" s="3">
+        <v>1.76</v>
+      </c>
+      <c r="E3" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G3" s="8">
+        <v>0</v>
+      </c>
+      <c r="H3" s="3">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="I3" s="9">
+        <v>0</v>
+      </c>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+    </row>
+    <row r="4" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4">
         <v>0.13</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D4" s="3">
+        <v>1.76</v>
+      </c>
+      <c r="E4" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F4" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G4" s="8">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3">
+        <v>2.5</v>
+      </c>
+      <c r="I4" s="9">
+        <v>0</v>
+      </c>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+    </row>
+    <row r="5" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D5" s="3">
+        <v>2.08</v>
+      </c>
+      <c r="E5" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G5" s="8">
+        <v>0</v>
+      </c>
+      <c r="H5" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="I5" s="9">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+    </row>
+    <row r="6" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6">
         <v>0.4</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D6" s="3">
+        <v>1.52</v>
+      </c>
+      <c r="E6" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G6" s="8">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="I6" s="9">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>6</v>
+        <v>102</v>
       </c>
       <c r="B7">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D7" s="3">
+        <v>1.07</v>
+      </c>
+      <c r="E7" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G7" s="8">
+        <v>0</v>
+      </c>
+      <c r="H7" s="3">
+        <v>0</v>
+      </c>
+      <c r="I7" s="9">
+        <v>125</v>
+      </c>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+    </row>
+    <row r="8" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D8" s="3">
+        <v>1.8</v>
+      </c>
+      <c r="E8" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" s="8">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3">
+        <v>2.6</v>
+      </c>
+      <c r="I8" s="9">
+        <v>0</v>
+      </c>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B9">
         <v>0.1</v>
       </c>
       <c r="C9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+        <v>35</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="E9" s="5">
+        <v>0</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G9" s="8">
+        <v>0</v>
+      </c>
+      <c r="H9" s="3">
+        <v>3</v>
+      </c>
+      <c r="I9" s="9">
+        <v>0</v>
+      </c>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10">
         <v>0.33</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D10" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="E10" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G10" s="8">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3">
+        <v>7</v>
+      </c>
+      <c r="I10" s="9">
+        <v>0</v>
+      </c>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11">
         <v>0.16</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D11" s="3">
+        <v>1.96</v>
+      </c>
+      <c r="E11" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F11" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G11" s="8">
+        <v>0</v>
+      </c>
+      <c r="H11" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="I11" s="9">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12">
+        <v>0</v>
+      </c>
+      <c r="D12" s="4">
+        <v>3.5</v>
+      </c>
+      <c r="E12" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G12" s="8">
+        <v>0</v>
+      </c>
+      <c r="H12" s="9">
+        <v>5</v>
+      </c>
+      <c r="I12" s="9">
+        <v>0</v>
+      </c>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>11</v>
-      </c>
-      <c r="B12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>12</v>
       </c>
       <c r="B13">
         <v>0.56000000000000005</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D13" s="3">
+        <v>0.20799999999999999</v>
+      </c>
+      <c r="E13" s="5">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="F13" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="G13" s="8">
+        <v>0</v>
+      </c>
+      <c r="H13" s="9">
+        <v>0</v>
+      </c>
+      <c r="I13" s="9">
+        <v>220</v>
+      </c>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14">
         <v>0.35</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="D14" s="3">
+        <v>0.25600000000000001</v>
+      </c>
+      <c r="E14" s="5">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="F14" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="G14" s="8">
+        <v>0</v>
+      </c>
+      <c r="H14" s="9">
+        <v>0</v>
+      </c>
+      <c r="I14" s="9">
+        <v>220</v>
+      </c>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15">
         <v>0.45</v>
       </c>
       <c r="C15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0.23</v>
+      </c>
+      <c r="E15" s="5">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="G15" s="8">
+        <v>0</v>
+      </c>
+      <c r="H15" s="9">
+        <v>0</v>
+      </c>
+      <c r="I15" s="9">
+        <v>220</v>
+      </c>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+    </row>
+    <row r="16" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16">
+        <v>0</v>
+      </c>
+      <c r="C16" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="D16" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="E16" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G16" s="8">
+        <v>0</v>
+      </c>
+      <c r="H16" s="9">
+        <v>0</v>
+      </c>
+      <c r="I16" s="9">
+        <v>50</v>
+      </c>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+    </row>
+    <row r="17" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
         <v>15</v>
       </c>
-      <c r="B16">
-        <v>0</v>
-      </c>
-      <c r="C16" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="B17">
+        <v>0</v>
+      </c>
+      <c r="D17" s="3">
+        <v>2</v>
+      </c>
+      <c r="E17" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G17" s="8">
+        <v>0</v>
+      </c>
+      <c r="H17" s="9">
+        <v>0</v>
+      </c>
+      <c r="I17" s="9">
+        <v>100</v>
+      </c>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+    </row>
+    <row r="18" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18">
+        <v>0</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.18</v>
+      </c>
+      <c r="E18" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F18" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G18" s="8">
+        <v>0</v>
+      </c>
+      <c r="H18" s="9">
+        <v>0</v>
+      </c>
+      <c r="I18" s="9">
+        <v>180</v>
+      </c>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+    </row>
+    <row r="19" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>16</v>
       </c>
-      <c r="B17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>40</v>
-      </c>
-      <c r="B18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+      <c r="B19">
+        <v>0</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0.36</v>
+      </c>
+      <c r="E19" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F19" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G19" s="8">
+        <v>0</v>
+      </c>
+      <c r="H19" s="9">
+        <v>0</v>
+      </c>
+      <c r="I19" s="9">
+        <v>300</v>
+      </c>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+    </row>
+    <row r="20" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>17</v>
       </c>
-      <c r="B19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0.22</v>
+      </c>
+      <c r="E20" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F20" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G20" s="8">
+        <v>0</v>
+      </c>
+      <c r="H20" s="9">
+        <v>0</v>
+      </c>
+      <c r="I20" s="9">
+        <v>150</v>
+      </c>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+    </row>
+    <row r="21" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>18</v>
       </c>
-      <c r="B20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+      <c r="B21">
+        <v>0</v>
+      </c>
+      <c r="D21" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="E21" s="5">
+        <v>0</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G21" s="8">
+        <v>0</v>
+      </c>
+      <c r="H21" s="9">
+        <v>0</v>
+      </c>
+      <c r="I21" s="9">
+        <v>100</v>
+      </c>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+    </row>
+    <row r="22" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>19</v>
       </c>
-      <c r="B21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+      <c r="B22">
+        <v>0</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0.67</v>
+      </c>
+      <c r="E22" s="5">
+        <v>0</v>
+      </c>
+      <c r="F22" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G22" s="8">
+        <v>0</v>
+      </c>
+      <c r="H22" s="9">
+        <v>0</v>
+      </c>
+      <c r="I22" s="9">
+        <v>80</v>
+      </c>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+    </row>
+    <row r="23" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>20</v>
       </c>
-      <c r="B22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0.18</v>
+      </c>
+      <c r="E23" s="5">
+        <v>0</v>
+      </c>
+      <c r="F23" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="G23" s="8">
+        <v>0</v>
+      </c>
+      <c r="H23" s="9">
+        <v>0</v>
+      </c>
+      <c r="I23" s="9">
+        <v>130</v>
+      </c>
+      <c r="J23" s="9"/>
+      <c r="K23" s="9"/>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>21</v>
       </c>
-      <c r="B23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0.35</v>
+      </c>
+      <c r="E24" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F24" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G24" s="8">
+        <v>0</v>
+      </c>
+      <c r="H24" s="9">
+        <v>0</v>
+      </c>
+      <c r="I24" s="9">
+        <v>120</v>
+      </c>
+      <c r="J24" s="9"/>
+      <c r="K24" s="9"/>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>22</v>
       </c>
-      <c r="B24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+      <c r="B25">
+        <v>0</v>
+      </c>
+      <c r="D25" s="3">
+        <v>0.35</v>
+      </c>
+      <c r="E25" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F25" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="G25" s="8">
+        <v>0</v>
+      </c>
+      <c r="H25" s="9">
+        <v>0</v>
+      </c>
+      <c r="I25" s="9">
+        <v>60</v>
+      </c>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>23</v>
-      </c>
-      <c r="B25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>24</v>
       </c>
       <c r="B26">
         <v>0.82</v>
       </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D26" s="3">
+        <v>1</v>
+      </c>
+      <c r="E26" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F26" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G26" s="8">
+        <v>0</v>
+      </c>
+      <c r="H26" s="9">
+        <v>1.3</v>
+      </c>
+      <c r="I26" s="9">
+        <v>0</v>
+      </c>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27">
+        <v>0</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0.36</v>
+      </c>
+      <c r="E27" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F27" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G27" s="8">
+        <v>0</v>
+      </c>
+      <c r="H27" s="9">
+        <v>0</v>
+      </c>
+      <c r="I27" s="9">
+        <v>300</v>
+      </c>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>25</v>
-      </c>
-      <c r="B27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>26</v>
       </c>
       <c r="B28">
         <v>0.38</v>
       </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D28" s="3">
+        <v>1.25</v>
+      </c>
+      <c r="E28" s="6">
+        <v>0</v>
+      </c>
+      <c r="F28" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G28" s="8">
+        <v>0</v>
+      </c>
+      <c r="H28" s="9">
+        <v>0</v>
+      </c>
+      <c r="I28" s="9">
+        <v>150</v>
+      </c>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
+        <v>26</v>
+      </c>
+      <c r="B29">
+        <v>0</v>
+      </c>
+      <c r="D29" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="E29" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F29" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G29" s="8">
+        <v>1.23</v>
+      </c>
+      <c r="H29" s="9">
+        <v>0</v>
+      </c>
+      <c r="I29" s="9">
+        <v>0</v>
+      </c>
+      <c r="J29" s="9"/>
+      <c r="K29" s="9"/>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>27</v>
-      </c>
-      <c r="B29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>28</v>
       </c>
       <c r="B30">
         <v>0.08</v>
       </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D30" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="E30" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F30" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G30" s="8">
+        <v>1.23</v>
+      </c>
+      <c r="H30" s="9">
+        <v>0</v>
+      </c>
+      <c r="I30" s="9">
+        <v>0</v>
+      </c>
+      <c r="J30" s="9"/>
+      <c r="K30" s="9"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31">
         <v>0.08</v>
       </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D31" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="E31" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F31" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G31" s="8">
+        <v>1.23</v>
+      </c>
+      <c r="H31" s="9">
+        <v>0</v>
+      </c>
+      <c r="I31" s="9">
+        <v>0</v>
+      </c>
+      <c r="J31" s="9"/>
+      <c r="K31" s="9"/>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B32">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D32" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="E32" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F32" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G32" s="8">
+        <v>1.23</v>
+      </c>
+      <c r="H32" s="9">
+        <v>0</v>
+      </c>
+      <c r="I32" s="9">
+        <v>0</v>
+      </c>
+      <c r="J32" s="9"/>
+      <c r="K32" s="9"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
+        <v>30</v>
+      </c>
+      <c r="B33">
+        <v>0</v>
+      </c>
+      <c r="D33" s="3">
+        <v>1.5</v>
+      </c>
+      <c r="E33" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F33" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G33" s="8">
+        <v>1.23</v>
+      </c>
+      <c r="H33" s="9">
+        <v>0</v>
+      </c>
+      <c r="I33" s="9">
+        <v>0</v>
+      </c>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>31</v>
       </c>
-      <c r="B33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+      <c r="B34">
+        <v>0</v>
+      </c>
+      <c r="D34" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="E34" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F34" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G34" s="8">
+        <v>1.23</v>
+      </c>
+      <c r="H34" s="9">
+        <v>0</v>
+      </c>
+      <c r="I34" s="9">
+        <v>0</v>
+      </c>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>32</v>
       </c>
-      <c r="B34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="D35" s="3">
+        <v>6</v>
+      </c>
+      <c r="E35" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="F35" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="G35" s="8">
+        <v>1.23</v>
+      </c>
+      <c r="H35" s="9">
+        <v>0</v>
+      </c>
+      <c r="I35" s="9">
+        <v>0</v>
+      </c>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>33</v>
       </c>
-      <c r="B35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>34</v>
-      </c>
       <c r="B36">
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="D36" s="3">
+        <v>2.8</v>
+      </c>
+      <c r="E36" s="5">
+        <v>0</v>
+      </c>
+      <c r="F36" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="G36" s="8">
+        <v>1.47</v>
+      </c>
+      <c r="H36" s="9">
+        <v>0</v>
+      </c>
+      <c r="I36" s="9">
+        <v>0</v>
+      </c>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B37">
         <v>0.25</v>
       </c>
+      <c r="D37" s="3">
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="E37" s="6">
+        <v>0</v>
+      </c>
+      <c r="F37" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="G37" s="8">
+        <v>0.36749999999999999</v>
+      </c>
+      <c r="H37" s="9">
+        <v>0</v>
+      </c>
+      <c r="I37" s="9">
+        <v>150</v>
+      </c>
+      <c r="J37" s="9"/>
+      <c r="K37" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -974,7 +1799,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12223D9-0A39-4CC4-B45B-34CE66BF62BA}">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="22.36328125" customWidth="1"/>
@@ -987,41 +1812,50 @@
     <col min="9" max="9" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" t="s">
+        <v>82</v>
+      </c>
+      <c r="H1" t="s">
+        <v>79</v>
+      </c>
+      <c r="I1" t="s">
+        <v>80</v>
+      </c>
+      <c r="J1" t="s">
+        <v>81</v>
+      </c>
+      <c r="K1" t="s">
+        <v>86</v>
+      </c>
+      <c r="L1" t="s">
+        <v>87</v>
+      </c>
+      <c r="M1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
         <v>42</v>
-      </c>
-      <c r="B1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D1" t="s">
-        <v>50</v>
-      </c>
-      <c r="E1" t="s">
-        <v>85</v>
-      </c>
-      <c r="F1" t="s">
-        <v>84</v>
-      </c>
-      <c r="G1" t="s">
-        <v>83</v>
-      </c>
-      <c r="H1" t="s">
-        <v>80</v>
-      </c>
-      <c r="I1" t="s">
-        <v>81</v>
-      </c>
-      <c r="J1" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>43</v>
       </c>
       <c r="B2">
         <f>1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -1053,10 +1887,19 @@
         <f>G2*5</f>
         <v>0.1</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K2">
+        <v>2.2700000000000001E-2</v>
+      </c>
+      <c r="L2">
+        <v>2.7699999999999999E-2</v>
+      </c>
+      <c r="M2">
+        <v>5.3E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3">
         <f>1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -1088,10 +1931,19 @@
         <f t="shared" ref="J3:J7" si="1">G3*5</f>
         <v>0.05</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K3">
+        <v>2.12E-2</v>
+      </c>
+      <c r="L3">
+        <v>2.5600000000000001E-2</v>
+      </c>
+      <c r="M3">
+        <v>9.4000000000000004E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B4">
         <f t="shared" ref="B4:B7" si="2">1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -1123,10 +1975,19 @@
         <f t="shared" si="1"/>
         <v>0.05</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K4">
+        <v>2.12E-2</v>
+      </c>
+      <c r="L4">
+        <v>2.5600000000000001E-2</v>
+      </c>
+      <c r="M4">
+        <v>9.4000000000000004E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B5">
         <f t="shared" si="2"/>
@@ -1158,10 +2019,19 @@
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K5">
+        <v>2.8299999999999999E-2</v>
+      </c>
+      <c r="L5">
+        <v>1.95E-2</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6">
         <f>1-(1-0.5)*(1-0.2)*(1-0.2)</f>
@@ -1193,10 +2063,19 @@
         <f t="shared" si="1"/>
         <v>0.1</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="K6">
+        <v>2.07E-2</v>
+      </c>
+      <c r="L6">
+        <v>2.8299999999999999E-2</v>
+      </c>
+      <c r="M6">
+        <v>1.7899999999999999E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B7">
         <f t="shared" si="2"/>
@@ -1227,6 +2106,15 @@
       <c r="J7">
         <f t="shared" si="1"/>
         <v>0.05</v>
+      </c>
+      <c r="K7">
+        <v>2.2700000000000001E-2</v>
+      </c>
+      <c r="L7">
+        <v>2.7699999999999999E-2</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -1241,39 +2129,39 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="5.7265625" customWidth="1"/>
-    <col min="3" max="3" width="4.6328125" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" customWidth="1"/>
     <col min="4" max="4" width="5.7265625" customWidth="1"/>
-    <col min="5" max="5" width="3.90625" customWidth="1"/>
-    <col min="6" max="6" width="4.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.90625" customWidth="1"/>
+    <col min="6" max="6" width="14" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" t="s">
         <v>51</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>52</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>53</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>54</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" t="s">
         <v>56</v>
       </c>
-      <c r="G1" t="s">
-        <v>57</v>
-      </c>
       <c r="H1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I1" t="s">
         <v>77</v>
-      </c>
-      <c r="I1" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -1299,7 +2187,7 @@
         <v>54417</v>
       </c>
       <c r="H2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I2" s="1">
         <f>2*14/(2*14+16)*(0.01164*B2+0.00594*C2+0.00594*F2)/(B2+C2+F2)*100</f>
@@ -1329,7 +2217,7 @@
         <v>266265</v>
       </c>
       <c r="H3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I3" s="1">
         <f t="shared" ref="I3:I24" si="0">2*14/(2*14+16)*(0.01164*B3+0.00594*C3+0.00594*F3)/(B3+C3+F3)*100</f>
@@ -1359,7 +2247,7 @@
         <v>168251</v>
       </c>
       <c r="H4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I4" s="1">
         <f t="shared" si="0"/>
@@ -1389,7 +2277,7 @@
         <v>80548</v>
       </c>
       <c r="H5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I5" s="1">
         <f t="shared" si="0"/>
@@ -1419,7 +2307,7 @@
         <v>256528</v>
       </c>
       <c r="H6" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I6" s="1">
         <f t="shared" si="0"/>
@@ -1449,7 +2337,7 @@
         <v>74606</v>
       </c>
       <c r="H7" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I7" s="1">
         <f t="shared" si="0"/>
@@ -1479,7 +2367,7 @@
         <v>96358</v>
       </c>
       <c r="H8" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I8" s="1">
         <f t="shared" si="0"/>
@@ -1509,7 +2397,7 @@
         <v>87002</v>
       </c>
       <c r="H9" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" si="0"/>
@@ -1539,7 +2427,7 @@
         <v>116150</v>
       </c>
       <c r="H10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I10" s="1">
         <f t="shared" si="0"/>
@@ -1569,7 +2457,7 @@
         <v>35716</v>
       </c>
       <c r="H11" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I11" s="1">
         <f t="shared" si="0"/>
@@ -1599,7 +2487,7 @@
         <v>29157</v>
       </c>
       <c r="H12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I12" s="1">
         <f t="shared" si="0"/>
@@ -1629,7 +2517,7 @@
         <v>141243</v>
       </c>
       <c r="H13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I13" s="1">
         <f t="shared" si="0"/>
@@ -1659,7 +2547,7 @@
         <v>111801</v>
       </c>
       <c r="H14" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I14" s="1">
         <f t="shared" si="0"/>
@@ -1689,7 +2577,7 @@
         <v>184174</v>
       </c>
       <c r="H15" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I15" s="1">
         <f t="shared" si="0"/>
@@ -1719,7 +2607,7 @@
         <v>133267</v>
       </c>
       <c r="H16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I16" s="1">
         <f t="shared" si="0"/>
@@ -1749,7 +2637,7 @@
         <v>135672</v>
       </c>
       <c r="H17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I17" s="1">
         <f t="shared" si="0"/>
@@ -1779,7 +2667,7 @@
         <v>18541</v>
       </c>
       <c r="H18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I18" s="1">
         <f t="shared" si="0"/>
@@ -1809,7 +2697,7 @@
         <v>66736</v>
       </c>
       <c r="H19" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I19" s="1">
         <f t="shared" si="0"/>
@@ -1839,7 +2727,7 @@
         <v>50349</v>
       </c>
       <c r="H20" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I20" s="1">
         <f>2*14/(2*14+16)*(0.01164*B20+0.00594*C20+0.00594*F20)/(B20+C20+F20)*100</f>
@@ -1869,7 +2757,7 @@
         <v>31445</v>
       </c>
       <c r="H21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I21" s="1">
         <f t="shared" si="0"/>
@@ -1899,7 +2787,7 @@
         <v>21502</v>
       </c>
       <c r="H22" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I22" s="1">
         <f t="shared" si="0"/>
@@ -1918,7 +2806,7 @@
       </c>
       <c r="F23" s="2"/>
       <c r="H23" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I23" s="1">
         <f t="shared" si="0"/>
@@ -1927,7 +2815,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B24">
         <v>924490</v>
@@ -1948,7 +2836,7 @@
         <v>2205890</v>
       </c>
       <c r="H24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I24" s="1">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Changed columns name in GRAFS_data
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FD0152E-33FE-4B40-93D1-7F82A48438A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3229BD7-C214-4CDC-8BB0-81AFA9B110E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
@@ -41,9 +41,6 @@
     <t>Culture</t>
   </si>
   <si>
-    <t>Surface recevant N organique maîtrisable</t>
-  </si>
-  <si>
     <t>Wheat</t>
   </si>
   <si>
@@ -345,6 +342,9 @@
   </si>
   <si>
     <t>Rice</t>
+  </si>
+  <si>
+    <t>Spreading Rate (%)</t>
   </si>
 </sst>
 </file>
@@ -751,33 +751,33 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>102</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E1" t="s">
+        <v>88</v>
+      </c>
+      <c r="F1" t="s">
         <v>89</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>90</v>
       </c>
-      <c r="G1" t="s">
-        <v>91</v>
-      </c>
       <c r="H1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="I1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B2">
         <v>0.12</v>
@@ -789,7 +789,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G2" s="8">
         <v>0</v>
@@ -805,7 +805,7 @@
     </row>
     <row r="3" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B3">
         <v>0.03</v>
@@ -817,7 +817,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G3" s="8">
         <v>0</v>
@@ -833,7 +833,7 @@
     </row>
     <row r="4" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4">
         <v>0.13</v>
@@ -845,7 +845,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G4" s="8">
         <v>0</v>
@@ -861,7 +861,7 @@
     </row>
     <row r="5" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5">
         <v>0.03</v>
@@ -873,7 +873,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G5" s="8">
         <v>0</v>
@@ -889,7 +889,7 @@
     </row>
     <row r="6" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6">
         <v>0.4</v>
@@ -901,7 +901,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G6" s="8">
         <v>0</v>
@@ -917,7 +917,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B7">
         <v>0.03</v>
@@ -929,7 +929,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G7" s="8">
         <v>0</v>
@@ -945,7 +945,7 @@
     </row>
     <row r="8" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B8">
         <v>0.03</v>
@@ -957,7 +957,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G8" s="8">
         <v>0</v>
@@ -973,13 +973,13 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9">
         <v>0.1</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D9" s="3">
         <v>0.5</v>
@@ -988,7 +988,7 @@
         <v>0</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G9" s="8">
         <v>0</v>
@@ -1004,7 +1004,7 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B10">
         <v>0.33</v>
@@ -1016,7 +1016,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F10" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G10" s="8">
         <v>0</v>
@@ -1032,7 +1032,7 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B11">
         <v>0.16</v>
@@ -1044,7 +1044,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G11" s="8">
         <v>0</v>
@@ -1060,7 +1060,7 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12">
         <v>0</v>
@@ -1072,7 +1072,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G12" s="8">
         <v>0</v>
@@ -1088,7 +1088,7 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B13">
         <v>0.56000000000000005</v>
@@ -1100,7 +1100,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G13" s="8">
         <v>0</v>
@@ -1116,7 +1116,7 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B14">
         <v>0.35</v>
@@ -1128,7 +1128,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G14" s="8">
         <v>0</v>
@@ -1144,13 +1144,13 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15">
         <v>0.45</v>
       </c>
       <c r="C15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D15" s="3">
         <v>0.23</v>
@@ -1159,7 +1159,7 @@
         <v>5.6000000000000001E-2</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G15" s="8">
         <v>0</v>
@@ -1175,13 +1175,13 @@
     </row>
     <row r="16" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B16">
         <v>0</v>
       </c>
       <c r="C16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D16" s="3">
         <v>3.6</v>
@@ -1190,7 +1190,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G16" s="8">
         <v>0</v>
@@ -1206,7 +1206,7 @@
     </row>
     <row r="17" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B17">
         <v>0</v>
@@ -1218,7 +1218,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G17" s="8">
         <v>0</v>
@@ -1234,7 +1234,7 @@
     </row>
     <row r="18" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B18">
         <v>0</v>
@@ -1246,7 +1246,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G18" s="8">
         <v>0</v>
@@ -1262,7 +1262,7 @@
     </row>
     <row r="19" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19">
         <v>0</v>
@@ -1274,7 +1274,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G19" s="8">
         <v>0</v>
@@ -1290,7 +1290,7 @@
     </row>
     <row r="20" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B20">
         <v>0</v>
@@ -1302,7 +1302,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G20" s="8">
         <v>0</v>
@@ -1318,7 +1318,7 @@
     </row>
     <row r="21" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B21">
         <v>0</v>
@@ -1330,7 +1330,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G21" s="8">
         <v>0</v>
@@ -1346,7 +1346,7 @@
     </row>
     <row r="22" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B22">
         <v>0</v>
@@ -1358,7 +1358,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G22" s="8">
         <v>0</v>
@@ -1374,7 +1374,7 @@
     </row>
     <row r="23" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B23">
         <v>0</v>
@@ -1386,7 +1386,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G23" s="8">
         <v>0</v>
@@ -1402,7 +1402,7 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B24">
         <v>0</v>
@@ -1414,7 +1414,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G24" s="8">
         <v>0</v>
@@ -1430,7 +1430,7 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B25">
         <v>0</v>
@@ -1442,7 +1442,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G25" s="8">
         <v>0</v>
@@ -1458,7 +1458,7 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B26">
         <v>0.82</v>
@@ -1470,7 +1470,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G26" s="8">
         <v>0</v>
@@ -1486,7 +1486,7 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B27">
         <v>0</v>
@@ -1498,7 +1498,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G27" s="8">
         <v>0</v>
@@ -1514,7 +1514,7 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B28">
         <v>0.38</v>
@@ -1526,7 +1526,7 @@
         <v>0</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G28" s="8">
         <v>0</v>
@@ -1542,7 +1542,7 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B29">
         <v>0</v>
@@ -1554,7 +1554,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G29" s="8">
         <v>1.23</v>
@@ -1570,7 +1570,7 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B30">
         <v>0.08</v>
@@ -1582,7 +1582,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G30" s="8">
         <v>1.23</v>
@@ -1598,7 +1598,7 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B31">
         <v>0.08</v>
@@ -1610,7 +1610,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G31" s="8">
         <v>1.23</v>
@@ -1626,7 +1626,7 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B32">
         <v>0</v>
@@ -1638,7 +1638,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G32" s="8">
         <v>1.23</v>
@@ -1654,7 +1654,7 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B33">
         <v>0</v>
@@ -1666,7 +1666,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G33" s="8">
         <v>1.23</v>
@@ -1682,7 +1682,7 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B34">
         <v>0</v>
@@ -1694,7 +1694,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G34" s="8">
         <v>1.23</v>
@@ -1710,7 +1710,7 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B35">
         <v>0</v>
@@ -1722,7 +1722,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G35" s="8">
         <v>1.23</v>
@@ -1738,7 +1738,7 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B36">
         <v>0</v>
@@ -1750,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G36" s="8">
         <v>1.47</v>
@@ -1766,7 +1766,7 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B37">
         <v>0.25</v>
@@ -1778,7 +1778,7 @@
         <v>0</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G37" s="8">
         <v>0.36749999999999999</v>
@@ -1814,48 +1814,48 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D1" t="s">
         <v>48</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G1" t="s">
+        <v>81</v>
+      </c>
+      <c r="H1" t="s">
         <v>78</v>
       </c>
-      <c r="D1" t="s">
-        <v>49</v>
-      </c>
-      <c r="E1" t="s">
-        <v>84</v>
-      </c>
-      <c r="F1" t="s">
-        <v>83</v>
-      </c>
-      <c r="G1" t="s">
-        <v>82</v>
-      </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>79</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>80</v>
       </c>
-      <c r="J1" t="s">
-        <v>81</v>
-      </c>
       <c r="K1" t="s">
+        <v>85</v>
+      </c>
+      <c r="L1" t="s">
         <v>86</v>
       </c>
-      <c r="L1" t="s">
-        <v>87</v>
-      </c>
       <c r="M1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B2">
         <f>1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -1899,7 +1899,7 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3">
         <f>1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -1943,7 +1943,7 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4">
         <f t="shared" ref="B4:B7" si="2">1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -1987,7 +1987,7 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5">
         <f t="shared" si="2"/>
@@ -2031,7 +2031,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6">
         <f>1-(1-0.5)*(1-0.2)*(1-0.2)</f>
@@ -2075,7 +2075,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B7">
         <f t="shared" si="2"/>
@@ -2137,31 +2137,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
         <v>50</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>51</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>52</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>53</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" t="s">
         <v>55</v>
       </c>
-      <c r="G1" t="s">
-        <v>56</v>
-      </c>
       <c r="H1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" t="s">
         <v>76</v>
-      </c>
-      <c r="I1" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -2187,7 +2187,7 @@
         <v>54417</v>
       </c>
       <c r="H2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I2" s="1">
         <f>2*14/(2*14+16)*(0.01164*B2+0.00594*C2+0.00594*F2)/(B2+C2+F2)*100</f>
@@ -2217,7 +2217,7 @@
         <v>266265</v>
       </c>
       <c r="H3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="I3" s="1">
         <f t="shared" ref="I3:I24" si="0">2*14/(2*14+16)*(0.01164*B3+0.00594*C3+0.00594*F3)/(B3+C3+F3)*100</f>
@@ -2247,7 +2247,7 @@
         <v>168251</v>
       </c>
       <c r="H4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I4" s="1">
         <f t="shared" si="0"/>
@@ -2277,7 +2277,7 @@
         <v>80548</v>
       </c>
       <c r="H5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I5" s="1">
         <f t="shared" si="0"/>
@@ -2307,7 +2307,7 @@
         <v>256528</v>
       </c>
       <c r="H6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I6" s="1">
         <f t="shared" si="0"/>
@@ -2337,7 +2337,7 @@
         <v>74606</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I7" s="1">
         <f t="shared" si="0"/>
@@ -2367,7 +2367,7 @@
         <v>96358</v>
       </c>
       <c r="H8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I8" s="1">
         <f t="shared" si="0"/>
@@ -2397,7 +2397,7 @@
         <v>87002</v>
       </c>
       <c r="H9" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" si="0"/>
@@ -2427,7 +2427,7 @@
         <v>116150</v>
       </c>
       <c r="H10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I10" s="1">
         <f t="shared" si="0"/>
@@ -2457,7 +2457,7 @@
         <v>35716</v>
       </c>
       <c r="H11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I11" s="1">
         <f t="shared" si="0"/>
@@ -2487,7 +2487,7 @@
         <v>29157</v>
       </c>
       <c r="H12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I12" s="1">
         <f t="shared" si="0"/>
@@ -2517,7 +2517,7 @@
         <v>141243</v>
       </c>
       <c r="H13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I13" s="1">
         <f t="shared" si="0"/>
@@ -2547,7 +2547,7 @@
         <v>111801</v>
       </c>
       <c r="H14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I14" s="1">
         <f t="shared" si="0"/>
@@ -2577,7 +2577,7 @@
         <v>184174</v>
       </c>
       <c r="H15" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I15" s="1">
         <f t="shared" si="0"/>
@@ -2607,7 +2607,7 @@
         <v>133267</v>
       </c>
       <c r="H16" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="I16" s="1">
         <f t="shared" si="0"/>
@@ -2637,7 +2637,7 @@
         <v>135672</v>
       </c>
       <c r="H17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="I17" s="1">
         <f t="shared" si="0"/>
@@ -2667,7 +2667,7 @@
         <v>18541</v>
       </c>
       <c r="H18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="I18" s="1">
         <f t="shared" si="0"/>
@@ -2697,7 +2697,7 @@
         <v>66736</v>
       </c>
       <c r="H19" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I19" s="1">
         <f t="shared" si="0"/>
@@ -2727,7 +2727,7 @@
         <v>50349</v>
       </c>
       <c r="H20" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I20" s="1">
         <f>2*14/(2*14+16)*(0.01164*B20+0.00594*C20+0.00594*F20)/(B20+C20+F20)*100</f>
@@ -2757,7 +2757,7 @@
         <v>31445</v>
       </c>
       <c r="H21" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I21" s="1">
         <f t="shared" si="0"/>
@@ -2787,7 +2787,7 @@
         <v>21502</v>
       </c>
       <c r="H22" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="I22" s="1">
         <f t="shared" si="0"/>
@@ -2806,7 +2806,7 @@
       </c>
       <c r="F23" s="2"/>
       <c r="H23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I23" s="1">
         <f t="shared" si="0"/>
@@ -2815,7 +2815,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B24">
         <v>924490</v>
@@ -2836,7 +2836,7 @@
         <v>2205890</v>
       </c>
       <c r="H24" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I24" s="1">
         <f t="shared" si="0"/>

</xml_diff>

<commit_message>
Correction d'un bug sur les nouvelles catégories (natural meadow, temporary meadow, forages)
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3229BD7-C214-4CDC-8BB0-81AFA9B110E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65DA067B-9A3C-4317-A53A-A5FF14E4D8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="104">
   <si>
     <t>Culture</t>
   </si>
@@ -326,9 +326,6 @@
     <t>forages</t>
   </si>
   <si>
-    <t>grasslands</t>
-  </si>
-  <si>
     <t>fruits and vegetables</t>
   </si>
   <si>
@@ -345,6 +342,12 @@
   </si>
   <si>
     <t>Spreading Rate (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">natural meadows </t>
+  </si>
+  <si>
+    <t>temporary meadows</t>
   </si>
 </sst>
 </file>
@@ -751,7 +754,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C1" t="s">
         <v>33</v>
@@ -769,10 +772,10 @@
         <v>90</v>
       </c>
       <c r="H1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
@@ -917,7 +920,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B7">
         <v>0.03</v>
@@ -1190,7 +1193,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G16" s="8">
         <v>0</v>
@@ -1218,7 +1221,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G17" s="8">
         <v>0</v>
@@ -1246,7 +1249,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G18" s="8">
         <v>0</v>
@@ -1274,7 +1277,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G19" s="8">
         <v>0</v>
@@ -1302,7 +1305,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G20" s="8">
         <v>0</v>
@@ -1330,7 +1333,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G21" s="8">
         <v>0</v>
@@ -1358,7 +1361,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G22" s="8">
         <v>0</v>
@@ -1386,7 +1389,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G23" s="8">
         <v>0</v>
@@ -1512,7 +1515,7 @@
       <c r="J27" s="9"/>
       <c r="K27" s="9"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>24</v>
       </c>
@@ -1526,7 +1529,7 @@
         <v>0</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="G28" s="8">
         <v>0</v>
@@ -1736,7 +1739,7 @@
       <c r="J35" s="9"/>
       <c r="K35" s="9"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>32</v>
       </c>
@@ -1750,7 +1753,7 @@
         <v>0</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="G36" s="8">
         <v>1.47</v>
@@ -1764,7 +1767,7 @@
       <c r="J36" s="9"/>
       <c r="K36" s="9"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>39</v>
       </c>
@@ -1778,7 +1781,7 @@
         <v>0</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="G37" s="8">
         <v>0.36749999999999999</v>
@@ -1850,7 +1853,7 @@
         <v>86</v>
       </c>
       <c r="M1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Resolve "Correction bug méline"
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3229BD7-C214-4CDC-8BB0-81AFA9B110E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65DA067B-9A3C-4317-A53A-A5FF14E4D8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="104">
   <si>
     <t>Culture</t>
   </si>
@@ -326,9 +326,6 @@
     <t>forages</t>
   </si>
   <si>
-    <t>grasslands</t>
-  </si>
-  <si>
     <t>fruits and vegetables</t>
   </si>
   <si>
@@ -345,6 +342,12 @@
   </si>
   <si>
     <t>Spreading Rate (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">natural meadows </t>
+  </si>
+  <si>
+    <t>temporary meadows</t>
   </si>
 </sst>
 </file>
@@ -751,7 +754,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C1" t="s">
         <v>33</v>
@@ -769,10 +772,10 @@
         <v>90</v>
       </c>
       <c r="H1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
@@ -917,7 +920,7 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B7">
         <v>0.03</v>
@@ -1190,7 +1193,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G16" s="8">
         <v>0</v>
@@ -1218,7 +1221,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G17" s="8">
         <v>0</v>
@@ -1246,7 +1249,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G18" s="8">
         <v>0</v>
@@ -1274,7 +1277,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F19" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G19" s="8">
         <v>0</v>
@@ -1302,7 +1305,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G20" s="8">
         <v>0</v>
@@ -1330,7 +1333,7 @@
         <v>0</v>
       </c>
       <c r="F21" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G21" s="8">
         <v>0</v>
@@ -1358,7 +1361,7 @@
         <v>0</v>
       </c>
       <c r="F22" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G22" s="8">
         <v>0</v>
@@ -1386,7 +1389,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G23" s="8">
         <v>0</v>
@@ -1512,7 +1515,7 @@
       <c r="J27" s="9"/>
       <c r="K27" s="9"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>24</v>
       </c>
@@ -1526,7 +1529,7 @@
         <v>0</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="G28" s="8">
         <v>0</v>
@@ -1736,7 +1739,7 @@
       <c r="J35" s="9"/>
       <c r="K35" s="9"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>32</v>
       </c>
@@ -1750,7 +1753,7 @@
         <v>0</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="G36" s="8">
         <v>1.47</v>
@@ -1764,7 +1767,7 @@
       <c r="J36" s="9"/>
       <c r="K36" s="9"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" ht="25" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>39</v>
       </c>
@@ -1778,7 +1781,7 @@
         <v>0</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="G37" s="8">
         <v>0.36749999999999999</v>
@@ -1850,7 +1853,7 @@
         <v>86</v>
       </c>
       <c r="M1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Added table under map tab. Add two tabs in GRAFS_data.xlsx for import/export and methanisation. Remove import_export xlsx file.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65DA067B-9A3C-4317-A53A-A5FF14E4D8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122AF7EF-3B37-423F-9A7B-1E288CB36E1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10380" activeTab="1" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
-    <sheet name="Volatilisation" sheetId="2" r:id="rId2"/>
-    <sheet name="N_syn" sheetId="3" r:id="rId3"/>
+    <sheet name="Energy_prod" sheetId="4" r:id="rId2"/>
+    <sheet name="import_export" sheetId="5" r:id="rId3"/>
+    <sheet name="Volatilisation" sheetId="2" r:id="rId4"/>
+    <sheet name="N_syn" sheetId="3" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="141">
   <si>
     <t>Culture</t>
   </si>
@@ -348,13 +350,124 @@
   </si>
   <si>
     <t>temporary meadows</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Ile de France</t>
+  </si>
+  <si>
+    <t>Eure</t>
+  </si>
+  <si>
+    <t>Eure-et-Loir</t>
+  </si>
+  <si>
+    <t>Picardie</t>
+  </si>
+  <si>
+    <t>Calvados-Orne</t>
+  </si>
+  <si>
+    <t>Seine Maritime</t>
+  </si>
+  <si>
+    <t>Manche</t>
+  </si>
+  <si>
+    <t>Nord Pas de Calais</t>
+  </si>
+  <si>
+    <t>Champ-Ard-Yonne</t>
+  </si>
+  <si>
+    <t>Bourgogne</t>
+  </si>
+  <si>
+    <t>Grande Lorraine</t>
+  </si>
+  <si>
+    <t>Alsace</t>
+  </si>
+  <si>
+    <t>Bretagne</t>
+  </si>
+  <si>
+    <t>Vendée-Charente</t>
+  </si>
+  <si>
+    <t>Loire aval</t>
+  </si>
+  <si>
+    <t>Loire Centrale</t>
+  </si>
+  <si>
+    <t>Loire Amont</t>
+  </si>
+  <si>
+    <t>Grand Jura</t>
+  </si>
+  <si>
+    <t>Savoie</t>
+  </si>
+  <si>
+    <t>Ain-Rhône</t>
+  </si>
+  <si>
+    <t>Alpes</t>
+  </si>
+  <si>
+    <t>Isère-Drôme Ardèche</t>
+  </si>
+  <si>
+    <t>Aveyron-Lozère</t>
+  </si>
+  <si>
+    <t>Garonne</t>
+  </si>
+  <si>
+    <t>Gironde</t>
+  </si>
+  <si>
+    <t>Pyrénées occidentales</t>
+  </si>
+  <si>
+    <t>Landes</t>
+  </si>
+  <si>
+    <t>Dor-Lot</t>
+  </si>
+  <si>
+    <t>Cantal-Corrèze</t>
+  </si>
+  <si>
+    <t>Grand Marseille</t>
+  </si>
+  <si>
+    <t>Côte d'Azur</t>
+  </si>
+  <si>
+    <t>Gard-Hérault</t>
+  </si>
+  <si>
+    <t>Pyrénées Orientales</t>
+  </si>
+  <si>
+    <t>Import</t>
+  </si>
+  <si>
+    <t>Export</t>
+  </si>
+  <si>
+    <t>Méthaniseur</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -385,6 +498,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -394,7 +513,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -402,12 +521,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -426,6 +560,12 @@
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1801,6 +1941,662 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EEDC770-986F-473C-8664-8C9A88803BEB}">
+  <dimension ref="A1:AI44"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1" t="s">
+        <v>110</v>
+      </c>
+      <c r="H1" t="s">
+        <v>111</v>
+      </c>
+      <c r="I1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K1" t="s">
+        <v>114</v>
+      </c>
+      <c r="L1" t="s">
+        <v>115</v>
+      </c>
+      <c r="M1" t="s">
+        <v>116</v>
+      </c>
+      <c r="N1" t="s">
+        <v>117</v>
+      </c>
+      <c r="O1" t="s">
+        <v>118</v>
+      </c>
+      <c r="P1" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>120</v>
+      </c>
+      <c r="R1" t="s">
+        <v>121</v>
+      </c>
+      <c r="S1" t="s">
+        <v>122</v>
+      </c>
+      <c r="T1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U1" t="s">
+        <v>124</v>
+      </c>
+      <c r="V1" t="s">
+        <v>125</v>
+      </c>
+      <c r="W1" t="s">
+        <v>126</v>
+      </c>
+      <c r="X1" t="s">
+        <v>127</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>128</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>129</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>131</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>132</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>133</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>134</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>136</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>137</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B2">
+        <v>348</v>
+      </c>
+      <c r="C2">
+        <v>53</v>
+      </c>
+      <c r="D2">
+        <v>24</v>
+      </c>
+      <c r="E2">
+        <v>458</v>
+      </c>
+      <c r="F2">
+        <v>97</v>
+      </c>
+      <c r="G2">
+        <v>63</v>
+      </c>
+      <c r="H2">
+        <v>65</v>
+      </c>
+      <c r="I2">
+        <v>275</v>
+      </c>
+      <c r="J2">
+        <v>548</v>
+      </c>
+      <c r="K2">
+        <v>90</v>
+      </c>
+      <c r="L2">
+        <v>397</v>
+      </c>
+      <c r="M2">
+        <v>108</v>
+      </c>
+      <c r="N2">
+        <v>388</v>
+      </c>
+      <c r="O2">
+        <v>105</v>
+      </c>
+      <c r="P2">
+        <v>199</v>
+      </c>
+      <c r="Q2">
+        <v>99</v>
+      </c>
+      <c r="R2">
+        <v>115</v>
+      </c>
+      <c r="S2">
+        <v>64</v>
+      </c>
+      <c r="T2">
+        <v>32</v>
+      </c>
+      <c r="U2">
+        <v>67</v>
+      </c>
+      <c r="V2">
+        <v>18</v>
+      </c>
+      <c r="W2">
+        <v>71</v>
+      </c>
+      <c r="X2">
+        <v>141</v>
+      </c>
+      <c r="Y2">
+        <v>197</v>
+      </c>
+      <c r="Z2">
+        <v>15</v>
+      </c>
+      <c r="AA2">
+        <v>79</v>
+      </c>
+      <c r="AB2">
+        <v>27</v>
+      </c>
+      <c r="AC2">
+        <v>56</v>
+      </c>
+      <c r="AD2">
+        <v>68</v>
+      </c>
+      <c r="AE2">
+        <v>28</v>
+      </c>
+      <c r="AF2">
+        <v>24</v>
+      </c>
+      <c r="AG2">
+        <v>12</v>
+      </c>
+      <c r="AH2">
+        <v>3</v>
+      </c>
+      <c r="AI2">
+        <v>4337</v>
+      </c>
+    </row>
+    <row r="11" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="12" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R12" s="10"/>
+    </row>
+    <row r="13" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R13" s="10"/>
+    </row>
+    <row r="14" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R14" s="10"/>
+    </row>
+    <row r="15" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R15" s="10"/>
+    </row>
+    <row r="16" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R16" s="10"/>
+    </row>
+    <row r="17" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R17" s="11"/>
+    </row>
+    <row r="18" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R18" s="10"/>
+    </row>
+    <row r="19" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R19" s="10"/>
+    </row>
+    <row r="20" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R20" s="10"/>
+    </row>
+    <row r="21" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R21" s="10"/>
+    </row>
+    <row r="22" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R22" s="10"/>
+    </row>
+    <row r="23" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R23" s="10"/>
+    </row>
+    <row r="24" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R24" s="10"/>
+    </row>
+    <row r="25" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R25" s="11"/>
+    </row>
+    <row r="26" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R26" s="10"/>
+    </row>
+    <row r="27" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R27" s="10"/>
+    </row>
+    <row r="28" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R28" s="10"/>
+    </row>
+    <row r="29" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R29" s="10"/>
+    </row>
+    <row r="30" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R30" s="10"/>
+    </row>
+    <row r="31" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R31" s="11"/>
+    </row>
+    <row r="32" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R32" s="10"/>
+    </row>
+    <row r="33" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R33" s="10"/>
+    </row>
+    <row r="34" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R34" s="10"/>
+    </row>
+    <row r="35" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R35" s="10"/>
+    </row>
+    <row r="36" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R36" s="10"/>
+    </row>
+    <row r="37" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R37" s="10"/>
+    </row>
+    <row r="38" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R38" s="10"/>
+    </row>
+    <row r="39" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R39" s="10"/>
+    </row>
+    <row r="40" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R40" s="11"/>
+    </row>
+    <row r="41" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R41" s="10"/>
+    </row>
+    <row r="42" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R42" s="10"/>
+    </row>
+    <row r="43" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R43" s="10"/>
+    </row>
+    <row r="44" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R44" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B24DCEF-E7C2-4526-9D13-3C67B63444AD}">
+  <dimension ref="A1:AI3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1" t="s">
+        <v>110</v>
+      </c>
+      <c r="H1" t="s">
+        <v>111</v>
+      </c>
+      <c r="I1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K1" t="s">
+        <v>114</v>
+      </c>
+      <c r="L1" t="s">
+        <v>115</v>
+      </c>
+      <c r="M1" t="s">
+        <v>116</v>
+      </c>
+      <c r="N1" t="s">
+        <v>117</v>
+      </c>
+      <c r="O1" t="s">
+        <v>118</v>
+      </c>
+      <c r="P1" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>120</v>
+      </c>
+      <c r="R1" t="s">
+        <v>121</v>
+      </c>
+      <c r="S1" t="s">
+        <v>122</v>
+      </c>
+      <c r="T1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U1" t="s">
+        <v>124</v>
+      </c>
+      <c r="V1" t="s">
+        <v>125</v>
+      </c>
+      <c r="W1" t="s">
+        <v>126</v>
+      </c>
+      <c r="X1" t="s">
+        <v>127</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>128</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>129</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>131</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>132</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>133</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>134</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>136</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>137</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2">
+        <v>92.113959999999992</v>
+      </c>
+      <c r="C2">
+        <v>9.3678999999999988</v>
+      </c>
+      <c r="D2">
+        <v>7.9292200000000008</v>
+      </c>
+      <c r="E2">
+        <v>32.702010000000001</v>
+      </c>
+      <c r="F2">
+        <v>28.21088000000001</v>
+      </c>
+      <c r="G2">
+        <v>97.652479999999954</v>
+      </c>
+      <c r="H2">
+        <v>15.820459999999995</v>
+      </c>
+      <c r="I2">
+        <v>66.401299999999992</v>
+      </c>
+      <c r="J2">
+        <v>35.252930000000006</v>
+      </c>
+      <c r="K2">
+        <v>14.638589999999997</v>
+      </c>
+      <c r="L2">
+        <v>44.824680000000001</v>
+      </c>
+      <c r="M2">
+        <v>31.32692999999999</v>
+      </c>
+      <c r="N2">
+        <v>160.72521</v>
+      </c>
+      <c r="O2">
+        <v>43.248719999999992</v>
+      </c>
+      <c r="P2">
+        <v>206.58865999999998</v>
+      </c>
+      <c r="Q2">
+        <v>32.781079999999989</v>
+      </c>
+      <c r="R2">
+        <v>58.299580000000006</v>
+      </c>
+      <c r="S2">
+        <v>8.6474600000000006</v>
+      </c>
+      <c r="T2">
+        <v>7.5009900000000016</v>
+      </c>
+      <c r="U2">
+        <v>24.510950000000001</v>
+      </c>
+      <c r="V2">
+        <v>1.1988499999999997</v>
+      </c>
+      <c r="W2">
+        <v>17.228110000000004</v>
+      </c>
+      <c r="X2">
+        <v>10.933770000000001</v>
+      </c>
+      <c r="Y2">
+        <v>27.44576</v>
+      </c>
+      <c r="Z2">
+        <v>48.051410000000011</v>
+      </c>
+      <c r="AA2">
+        <v>13.837059999999997</v>
+      </c>
+      <c r="AB2">
+        <v>10.718019999999999</v>
+      </c>
+      <c r="AC2">
+        <v>11.926820000000003</v>
+      </c>
+      <c r="AD2">
+        <v>12.789459999999996</v>
+      </c>
+      <c r="AE2">
+        <v>27.769340000000007</v>
+      </c>
+      <c r="AF2">
+        <v>5.3662799999999971</v>
+      </c>
+      <c r="AG2">
+        <v>11.832720000000002</v>
+      </c>
+      <c r="AH2">
+        <v>4.6259899999999998</v>
+      </c>
+      <c r="AI2">
+        <v>437.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3">
+        <v>58.260291000000002</v>
+      </c>
+      <c r="C3">
+        <v>43.361862000000002</v>
+      </c>
+      <c r="D3">
+        <v>30.468439999999994</v>
+      </c>
+      <c r="E3">
+        <v>91.869658000000001</v>
+      </c>
+      <c r="F3">
+        <v>23.830795000000002</v>
+      </c>
+      <c r="G3">
+        <v>125.05385200000001</v>
+      </c>
+      <c r="H3">
+        <v>7.2032819999999997</v>
+      </c>
+      <c r="I3">
+        <v>93.045423999999997</v>
+      </c>
+      <c r="J3">
+        <v>90.388374000000013</v>
+      </c>
+      <c r="K3">
+        <v>32.028894000000015</v>
+      </c>
+      <c r="L3">
+        <v>61.268584499999996</v>
+      </c>
+      <c r="M3">
+        <v>43.307626499999998</v>
+      </c>
+      <c r="N3">
+        <v>48.774823999999995</v>
+      </c>
+      <c r="O3">
+        <v>45.255763000000016</v>
+      </c>
+      <c r="P3">
+        <v>79.412431000000012</v>
+      </c>
+      <c r="Q3">
+        <v>93.641458999999998</v>
+      </c>
+      <c r="R3">
+        <v>47.56297</v>
+      </c>
+      <c r="S3">
+        <v>13.527467</v>
+      </c>
+      <c r="T3">
+        <v>4.7963090000000008</v>
+      </c>
+      <c r="U3">
+        <v>22.102628000000003</v>
+      </c>
+      <c r="V3">
+        <v>2.5489359999999999</v>
+      </c>
+      <c r="W3">
+        <v>19.579385000000002</v>
+      </c>
+      <c r="X3">
+        <v>3.6610950000000004</v>
+      </c>
+      <c r="Y3">
+        <v>59.672404000000043</v>
+      </c>
+      <c r="Z3">
+        <v>30.027981</v>
+      </c>
+      <c r="AA3">
+        <v>27.866744999999998</v>
+      </c>
+      <c r="AB3">
+        <v>20.721993000000001</v>
+      </c>
+      <c r="AC3">
+        <v>4.8341580000000004</v>
+      </c>
+      <c r="AD3">
+        <v>3.4297689999999998</v>
+      </c>
+      <c r="AE3">
+        <v>23.448231999999997</v>
+      </c>
+      <c r="AF3">
+        <v>1.181686</v>
+      </c>
+      <c r="AG3">
+        <v>24.802152999999997</v>
+      </c>
+      <c r="AH3">
+        <v>6.1657950000000001</v>
+      </c>
+      <c r="AI3">
+        <v>498.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12223D9-0A39-4CC4-B45B-34CE66BF62BA}">
   <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2126,7 +2922,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D061B11-9C82-42EB-AFA7-28C01EBEFD7E}">
   <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Added meth_power tab in grafs_data
Added methanizer regime tab in grafs_data
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,16 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{122AF7EF-3B37-423F-9A7B-1E288CB36E1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25D9AA85-5439-4E60-BE06-F2297C951363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10380" activeTab="1" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
     <sheet name="Energy_prod" sheetId="4" r:id="rId2"/>
-    <sheet name="import_export" sheetId="5" r:id="rId3"/>
-    <sheet name="Volatilisation" sheetId="2" r:id="rId4"/>
-    <sheet name="N_syn" sheetId="3" r:id="rId5"/>
+    <sheet name="Energy_power" sheetId="6" r:id="rId3"/>
+    <sheet name="Energy_regime" sheetId="7" r:id="rId4"/>
+    <sheet name="import_export" sheetId="5" r:id="rId5"/>
+    <sheet name="Volatilisation" sheetId="2" r:id="rId6"/>
+    <sheet name="N_syn" sheetId="3" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="170">
   <si>
     <t>Culture</t>
   </si>
@@ -461,6 +463,93 @@
   </si>
   <si>
     <t>Méthaniseur</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Methanization power (GWh/tMS)</t>
+  </si>
+  <si>
+    <t>Rapeseed straw</t>
+  </si>
+  <si>
+    <t>Maize straw</t>
+  </si>
+  <si>
+    <t>Bovines manure</t>
+  </si>
+  <si>
+    <t>Poultry slurry</t>
+  </si>
+  <si>
+    <t>Bovines slurry</t>
+  </si>
+  <si>
+    <t>CIVE</t>
+  </si>
+  <si>
+    <t>Sunflower straw</t>
+  </si>
+  <si>
+    <t>Sugar beet residues</t>
+  </si>
+  <si>
+    <t>Soybean straw</t>
+  </si>
+  <si>
+    <t>Potatoes residues</t>
+  </si>
+  <si>
+    <t>Green waste</t>
+  </si>
+  <si>
+    <t>meadows</t>
+  </si>
+  <si>
+    <t>Cereal straw</t>
+  </si>
+  <si>
+    <t>Slaughterhouse IAA</t>
+  </si>
+  <si>
+    <t>Sludges</t>
+  </si>
+  <si>
+    <t>Waste IAA</t>
+  </si>
+  <si>
+    <t>Waste population</t>
+  </si>
+  <si>
+    <t>Porcines slurry</t>
+  </si>
+  <si>
+    <t>Porcines manure</t>
+  </si>
+  <si>
+    <t>MB</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Crop residues</t>
+  </si>
+  <si>
+    <t>Dedicated culture</t>
+  </si>
+  <si>
+    <t>Non edible animal</t>
+  </si>
+  <si>
+    <t>Livestock effluent</t>
+  </si>
+  <si>
+    <t>Share</t>
   </si>
 </sst>
 </file>
@@ -2266,6 +2355,407 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0C8FA35-4843-4FEC-9720-CB1F6CC19C35}">
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="7" max="7" width="17.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B2">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>163</v>
+      </c>
+      <c r="D2" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>144</v>
+      </c>
+      <c r="B3">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4">
+        <v>3.5500000000000002E-3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D4" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5">
+        <v>2.8999999999999998E-3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>163</v>
+      </c>
+      <c r="D5" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>150</v>
+      </c>
+      <c r="B6">
+        <v>3.5E-4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>163</v>
+      </c>
+      <c r="D6" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>151</v>
+      </c>
+      <c r="B7">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>163</v>
+      </c>
+      <c r="D7" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>152</v>
+      </c>
+      <c r="B8">
+        <v>5.5000000000000003E-4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>163</v>
+      </c>
+      <c r="D8" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B9">
+        <v>2.0999999999999999E-3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>163</v>
+      </c>
+      <c r="D9" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>163</v>
+      </c>
+      <c r="D10" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>154</v>
+      </c>
+      <c r="B11">
+        <v>2.0999999999999999E-3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>163</v>
+      </c>
+      <c r="D11" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>155</v>
+      </c>
+      <c r="B12">
+        <v>2.5500000000000002E-3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>163</v>
+      </c>
+      <c r="D12" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>156</v>
+      </c>
+      <c r="B13">
+        <v>5.8E-4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>164</v>
+      </c>
+      <c r="D13" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>157</v>
+      </c>
+      <c r="B14">
+        <v>5.5000000000000003E-4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>164</v>
+      </c>
+      <c r="D14" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>158</v>
+      </c>
+      <c r="B15">
+        <v>4.4999999999999999E-4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>164</v>
+      </c>
+      <c r="D15" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>159</v>
+      </c>
+      <c r="B16">
+        <v>7.5000000000000002E-4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>164</v>
+      </c>
+      <c r="D16" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>160</v>
+      </c>
+      <c r="B17">
+        <v>9.0000000000000006E-5</v>
+      </c>
+      <c r="C17" t="s">
+        <v>164</v>
+      </c>
+      <c r="D17" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>147</v>
+      </c>
+      <c r="B18">
+        <v>1.7000000000000001E-4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>164</v>
+      </c>
+      <c r="D18" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>161</v>
+      </c>
+      <c r="B19">
+        <v>5.9999999999999995E-4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>164</v>
+      </c>
+      <c r="D19" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>145</v>
+      </c>
+      <c r="B20">
+        <v>4.0000000000000002E-4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>164</v>
+      </c>
+      <c r="D20" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>146</v>
+      </c>
+      <c r="B21">
+        <v>1.6000000000000001E-3</v>
+      </c>
+      <c r="C21" t="s">
+        <v>164</v>
+      </c>
+      <c r="D21" t="s">
+        <v>168</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDCA4DCB-FE4A-48BA-AD0E-D81C83744525}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B4">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>166</v>
+      </c>
+      <c r="B5">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>167</v>
+      </c>
+      <c r="B6">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>158</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>159</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B10">
+        <v>0.79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B24DCEF-E7C2-4526-9D13-3C67B63444AD}">
   <dimension ref="A1:AI3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2596,7 +3086,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12223D9-0A39-4CC4-B45B-34CE66BF62BA}">
   <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2922,7 +3412,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D061B11-9C82-42EB-AFA7-28C01EBEFD7E}">
   <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Updated Meth_power tab in grafs_data
Added green waste in ext

Added energy regime in scenario sheet technical tab.

Did a new energy_power tab with clear connexion to GRAFS-E items

Added DM% for every cultures product
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25D9AA85-5439-4E60-BE06-F2297C951363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C25F80B-7E4F-42E7-B425-8BF1D82792BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
     <sheet name="Energy_prod" sheetId="4" r:id="rId2"/>
-    <sheet name="Energy_power" sheetId="6" r:id="rId3"/>
-    <sheet name="Energy_regime" sheetId="7" r:id="rId4"/>
-    <sheet name="import_export" sheetId="5" r:id="rId5"/>
-    <sheet name="Volatilisation" sheetId="2" r:id="rId6"/>
-    <sheet name="N_syn" sheetId="3" r:id="rId7"/>
+    <sheet name="Energy_power_old" sheetId="6" r:id="rId3"/>
+    <sheet name="Energy_power" sheetId="8" r:id="rId4"/>
+    <sheet name="Energy_regime" sheetId="7" r:id="rId5"/>
+    <sheet name="import_export" sheetId="5" r:id="rId6"/>
+    <sheet name="Volatilisation" sheetId="2" r:id="rId7"/>
+    <sheet name="N_syn" sheetId="3" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="183">
   <si>
     <t>Culture</t>
   </si>
@@ -504,9 +505,6 @@
     <t>Green waste</t>
   </si>
   <si>
-    <t>meadows</t>
-  </si>
-  <si>
     <t>Cereal straw</t>
   </si>
   <si>
@@ -550,6 +548,48 @@
   </si>
   <si>
     <t>Share</t>
+  </si>
+  <si>
+    <t>Poultry manure</t>
+  </si>
+  <si>
+    <t>Caprines slurry</t>
+  </si>
+  <si>
+    <t>Caprines manure</t>
+  </si>
+  <si>
+    <t>Equines slurry</t>
+  </si>
+  <si>
+    <t>Equines manure</t>
+  </si>
+  <si>
+    <t>Taken as manure</t>
+  </si>
+  <si>
+    <t>Ovines slurry</t>
+  </si>
+  <si>
+    <t>Ovines manure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Natural meadows </t>
+  </si>
+  <si>
+    <t>Non legume temporary meadow</t>
+  </si>
+  <si>
+    <t>DM content (% of gross matter)</t>
+  </si>
+  <si>
+    <t>DM content done with https://www.feedtables.com/content/dry-matter and https://fdc.nal.usda.gov/</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Methanization power (GWh/tMB)</t>
   </si>
 </sst>
 </file>
@@ -970,15 +1010,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{973E28D2-5D19-4409-920F-79B00DDA2ABC}">
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.7265625" customWidth="1"/>
-    <col min="4" max="4" width="19.6328125" customWidth="1"/>
-    <col min="5" max="5" width="14.90625" customWidth="1"/>
+    <col min="5" max="5" width="19.6328125" customWidth="1"/>
+    <col min="6" max="6" width="14.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -989,221 +1029,248 @@
         <v>33</v>
       </c>
       <c r="D1" t="s">
+        <v>179</v>
+      </c>
+      <c r="E1" t="s">
         <v>84</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>88</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>89</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>90</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>99</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2">
         <v>0.12</v>
       </c>
-      <c r="D2" s="3">
+      <c r="C2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D2">
+        <v>86.9</v>
+      </c>
+      <c r="E2" s="3">
         <v>1.95</v>
       </c>
-      <c r="E2" s="5">
+      <c r="F2" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G2" s="8">
-        <v>0</v>
-      </c>
-      <c r="H2" s="3">
+      <c r="H2" s="8">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3">
         <v>3.5</v>
       </c>
-      <c r="I2" s="9">
-        <v>0</v>
-      </c>
-      <c r="J2" s="9"/>
+      <c r="J2" s="9">
+        <v>0</v>
+      </c>
       <c r="K2" s="9"/>
-    </row>
-    <row r="3" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="L2" s="9"/>
+    </row>
+    <row r="3" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
       <c r="B3">
         <v>0.03</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3">
+        <v>86.7</v>
+      </c>
+      <c r="E3" s="3">
         <v>1.76</v>
       </c>
-      <c r="E3" s="5">
+      <c r="F3" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G3" s="8">
-        <v>0</v>
-      </c>
-      <c r="H3" s="3">
+      <c r="H3" s="8">
+        <v>0</v>
+      </c>
+      <c r="I3" s="3">
         <v>2.2999999999999998</v>
       </c>
-      <c r="I3" s="9">
-        <v>0</v>
-      </c>
-      <c r="J3" s="9"/>
+      <c r="J3" s="9">
+        <v>0</v>
+      </c>
       <c r="K3" s="9"/>
-    </row>
-    <row r="4" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="L3" s="9"/>
+    </row>
+    <row r="4" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4">
         <v>0.13</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4">
+        <v>87.2</v>
+      </c>
+      <c r="E4" s="3">
         <v>1.76</v>
       </c>
-      <c r="E4" s="5">
+      <c r="F4" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G4" s="8">
-        <v>0</v>
-      </c>
-      <c r="H4" s="3">
+      <c r="H4" s="8">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3">
         <v>2.5</v>
       </c>
-      <c r="I4" s="9">
-        <v>0</v>
-      </c>
-      <c r="J4" s="9"/>
+      <c r="J4" s="9">
+        <v>0</v>
+      </c>
       <c r="K4" s="9"/>
-    </row>
-    <row r="5" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="L4" s="9"/>
+    </row>
+    <row r="5" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5">
         <v>0.03</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5">
+        <v>87.6</v>
+      </c>
+      <c r="E5" s="3">
         <v>2.08</v>
       </c>
-      <c r="E5" s="5">
+      <c r="F5" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G5" s="8">
-        <v>0</v>
-      </c>
-      <c r="H5" s="3">
+      <c r="H5" s="8">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="I5" s="9">
-        <v>0</v>
-      </c>
-      <c r="J5" s="9"/>
+      <c r="J5" s="9">
+        <v>0</v>
+      </c>
       <c r="K5" s="9"/>
-    </row>
-    <row r="6" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="L5" s="9"/>
+    </row>
+    <row r="6" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6">
         <v>0.4</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6">
+        <v>86.3</v>
+      </c>
+      <c r="E6" s="3">
         <v>1.52</v>
       </c>
-      <c r="E6" s="5">
+      <c r="F6" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G6" s="8">
-        <v>0</v>
-      </c>
-      <c r="H6" s="3">
+      <c r="H6" s="8">
+        <v>0</v>
+      </c>
+      <c r="I6" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="I6" s="9">
-        <v>0</v>
-      </c>
-      <c r="J6" s="9"/>
+      <c r="J6" s="9">
+        <v>0</v>
+      </c>
       <c r="K6" s="9"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L6" s="9"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>100</v>
       </c>
       <c r="B7">
         <v>0.03</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7">
+        <v>88</v>
+      </c>
+      <c r="E7" s="3">
         <v>1.07</v>
       </c>
-      <c r="E7" s="5">
+      <c r="F7" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="G7" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="G7" s="8">
-        <v>0</v>
-      </c>
-      <c r="H7" s="3">
-        <v>0</v>
-      </c>
-      <c r="I7" s="9">
+      <c r="H7" s="8">
+        <v>0</v>
+      </c>
+      <c r="I7" s="3">
+        <v>0</v>
+      </c>
+      <c r="J7" s="9">
         <v>125</v>
       </c>
-      <c r="J7" s="9"/>
       <c r="K7" s="9"/>
-    </row>
-    <row r="8" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="L7" s="9"/>
+    </row>
+    <row r="8" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>5</v>
       </c>
       <c r="B8">
         <v>0.03</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8">
+        <v>89.6</v>
+      </c>
+      <c r="E8" s="3">
         <v>1.8</v>
       </c>
-      <c r="E8" s="5">
+      <c r="F8" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="G8" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G8" s="8">
-        <v>0</v>
-      </c>
-      <c r="H8" s="3">
+      <c r="H8" s="8">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3">
         <v>2.6</v>
       </c>
-      <c r="I8" s="9">
-        <v>0</v>
-      </c>
-      <c r="J8" s="9"/>
+      <c r="J8" s="9">
+        <v>0</v>
+      </c>
       <c r="K8" s="9"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L8" s="9"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -1213,168 +1280,186 @@
       <c r="C9" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9">
+        <v>90.3</v>
+      </c>
+      <c r="E9" s="3">
         <v>0.5</v>
       </c>
-      <c r="E9" s="5">
-        <v>0</v>
-      </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="5">
+        <v>0</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G9" s="8">
-        <v>0</v>
-      </c>
-      <c r="H9" s="3">
+      <c r="H9" s="8">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3">
         <v>3</v>
       </c>
-      <c r="I9" s="9">
-        <v>0</v>
-      </c>
-      <c r="J9" s="9"/>
+      <c r="J9" s="9">
+        <v>0</v>
+      </c>
       <c r="K9" s="9"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L9" s="9"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>7</v>
       </c>
       <c r="B10">
         <v>0.33</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10">
+        <v>92.4</v>
+      </c>
+      <c r="E10" s="3">
         <v>3.5</v>
       </c>
-      <c r="E10" s="5">
+      <c r="F10" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="G10" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G10" s="8">
-        <v>0</v>
-      </c>
-      <c r="H10" s="3">
+      <c r="H10" s="8">
+        <v>0</v>
+      </c>
+      <c r="I10" s="3">
         <v>7</v>
       </c>
-      <c r="I10" s="9">
-        <v>0</v>
-      </c>
-      <c r="J10" s="9"/>
+      <c r="J10" s="9">
+        <v>0</v>
+      </c>
       <c r="K10" s="9"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L10" s="9"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
       <c r="B11">
         <v>0.16</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11">
+        <v>92.8</v>
+      </c>
+      <c r="E11" s="3">
         <v>1.96</v>
       </c>
-      <c r="E11" s="5">
+      <c r="F11" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="G11" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G11" s="8">
-        <v>0</v>
-      </c>
-      <c r="H11" s="3">
+      <c r="H11" s="8">
+        <v>0</v>
+      </c>
+      <c r="I11" s="3">
         <v>4.5</v>
       </c>
-      <c r="I11" s="9">
-        <v>0</v>
-      </c>
-      <c r="J11" s="9"/>
+      <c r="J11" s="9">
+        <v>0</v>
+      </c>
       <c r="K11" s="9"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L11" s="9"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>9</v>
       </c>
       <c r="B12">
         <v>0</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12">
+        <v>88.1</v>
+      </c>
+      <c r="E12" s="4">
         <v>3.5</v>
       </c>
-      <c r="E12" s="5">
+      <c r="F12" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G12" s="8">
-        <v>0</v>
-      </c>
-      <c r="H12" s="9">
+      <c r="H12" s="8">
+        <v>0</v>
+      </c>
+      <c r="I12" s="9">
         <v>5</v>
       </c>
-      <c r="I12" s="9">
-        <v>0</v>
-      </c>
-      <c r="J12" s="9"/>
+      <c r="J12" s="9">
+        <v>0</v>
+      </c>
       <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L12" s="9"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>10</v>
       </c>
       <c r="B13">
         <v>0.56000000000000005</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13">
+        <v>17.8</v>
+      </c>
+      <c r="E13" s="3">
         <v>0.20799999999999999</v>
       </c>
-      <c r="E13" s="5">
+      <c r="F13" s="5">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="G13" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G13" s="8">
-        <v>0</v>
-      </c>
-      <c r="H13" s="9">
+      <c r="H13" s="8">
         <v>0</v>
       </c>
       <c r="I13" s="9">
+        <v>0</v>
+      </c>
+      <c r="J13" s="9">
         <v>220</v>
       </c>
-      <c r="J13" s="9"/>
       <c r="K13" s="9"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L13" s="9"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>11</v>
       </c>
       <c r="B14">
         <v>0.35</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14">
+        <v>18.899999999999999</v>
+      </c>
+      <c r="E14" s="3">
         <v>0.25600000000000001</v>
       </c>
-      <c r="E14" s="5">
+      <c r="F14" s="5">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="G14" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G14" s="8">
-        <v>0</v>
-      </c>
-      <c r="H14" s="9">
+      <c r="H14" s="8">
         <v>0</v>
       </c>
       <c r="I14" s="9">
+        <v>0</v>
+      </c>
+      <c r="J14" s="9">
         <v>220</v>
       </c>
-      <c r="J14" s="9"/>
       <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L14" s="9"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -1384,28 +1469,31 @@
       <c r="C15" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15">
+        <v>17.8</v>
+      </c>
+      <c r="E15" s="3">
         <v>0.23</v>
       </c>
-      <c r="E15" s="5">
+      <c r="F15" s="5">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="G15" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G15" s="8">
-        <v>0</v>
-      </c>
-      <c r="H15" s="9">
+      <c r="H15" s="8">
         <v>0</v>
       </c>
       <c r="I15" s="9">
+        <v>0</v>
+      </c>
+      <c r="J15" s="9">
         <v>220</v>
       </c>
-      <c r="J15" s="9"/>
       <c r="K15" s="9"/>
-    </row>
-    <row r="16" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L15" s="9"/>
+    </row>
+    <row r="16" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1415,614 +1503,677 @@
       <c r="C16" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16">
+        <v>88.4</v>
+      </c>
+      <c r="E16" s="3">
         <v>3.6</v>
       </c>
-      <c r="E16" s="5">
+      <c r="F16" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="G16" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G16" s="8">
-        <v>0</v>
-      </c>
-      <c r="H16" s="9">
+      <c r="H16" s="8">
         <v>0</v>
       </c>
       <c r="I16" s="9">
+        <v>0</v>
+      </c>
+      <c r="J16" s="9">
         <v>50</v>
       </c>
-      <c r="J16" s="9"/>
       <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L16" s="9"/>
+    </row>
+    <row r="17" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>14</v>
       </c>
       <c r="B17">
         <v>0</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17">
+        <v>80</v>
+      </c>
+      <c r="E17" s="3">
         <v>2</v>
       </c>
-      <c r="E17" s="5">
+      <c r="F17" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="G17" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G17" s="8">
-        <v>0</v>
-      </c>
-      <c r="H17" s="9">
+      <c r="H17" s="8">
         <v>0</v>
       </c>
       <c r="I17" s="9">
+        <v>0</v>
+      </c>
+      <c r="J17" s="9">
         <v>100</v>
       </c>
-      <c r="J17" s="9"/>
       <c r="K17" s="9"/>
-    </row>
-    <row r="18" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L17" s="9"/>
+    </row>
+    <row r="18" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>38</v>
       </c>
       <c r="B18">
         <v>0</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="E18" s="3">
         <v>0.18</v>
       </c>
-      <c r="E18" s="5">
+      <c r="F18" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="G18" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G18" s="8">
-        <v>0</v>
-      </c>
-      <c r="H18" s="9">
+      <c r="H18" s="8">
         <v>0</v>
       </c>
       <c r="I18" s="9">
+        <v>0</v>
+      </c>
+      <c r="J18" s="9">
         <v>180</v>
       </c>
-      <c r="J18" s="9"/>
       <c r="K18" s="9"/>
-    </row>
-    <row r="19" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L18" s="9"/>
+    </row>
+    <row r="19" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>15</v>
       </c>
       <c r="B19">
         <v>0</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19">
+        <v>8.1</v>
+      </c>
+      <c r="E19" s="3">
         <v>0.36</v>
       </c>
-      <c r="E19" s="5">
+      <c r="F19" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="G19" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G19" s="8">
-        <v>0</v>
-      </c>
-      <c r="H19" s="9">
+      <c r="H19" s="8">
         <v>0</v>
       </c>
       <c r="I19" s="9">
+        <v>0</v>
+      </c>
+      <c r="J19" s="9">
         <v>300</v>
       </c>
-      <c r="J19" s="9"/>
       <c r="K19" s="9"/>
-    </row>
-    <row r="20" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L19" s="9"/>
+    </row>
+    <row r="20" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>16</v>
       </c>
       <c r="B20">
         <v>0</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20">
+        <v>4.5</v>
+      </c>
+      <c r="E20" s="3">
         <v>0.22</v>
       </c>
-      <c r="E20" s="5">
+      <c r="F20" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="G20" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G20" s="8">
-        <v>0</v>
-      </c>
-      <c r="H20" s="9">
+      <c r="H20" s="8">
         <v>0</v>
       </c>
       <c r="I20" s="9">
+        <v>0</v>
+      </c>
+      <c r="J20" s="9">
         <v>150</v>
       </c>
-      <c r="J20" s="9"/>
       <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L20" s="9"/>
+    </row>
+    <row r="21" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>17</v>
       </c>
       <c r="B21">
         <v>0</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21">
+        <v>16.399999999999999</v>
+      </c>
+      <c r="E21" s="3">
         <v>0.1</v>
       </c>
-      <c r="E21" s="5">
-        <v>0</v>
-      </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="5">
+        <v>0</v>
+      </c>
+      <c r="G21" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G21" s="8">
-        <v>0</v>
-      </c>
-      <c r="H21" s="9">
+      <c r="H21" s="8">
         <v>0</v>
       </c>
       <c r="I21" s="9">
+        <v>0</v>
+      </c>
+      <c r="J21" s="9">
         <v>100</v>
       </c>
-      <c r="J21" s="9"/>
       <c r="K21" s="9"/>
-    </row>
-    <row r="22" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L21" s="9"/>
+    </row>
+    <row r="22" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>18</v>
       </c>
       <c r="B22">
         <v>0</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22">
+        <v>24.7</v>
+      </c>
+      <c r="E22" s="3">
         <v>0.67</v>
       </c>
-      <c r="E22" s="5">
-        <v>0</v>
-      </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="5">
+        <v>0</v>
+      </c>
+      <c r="G22" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G22" s="8">
-        <v>0</v>
-      </c>
-      <c r="H22" s="9">
+      <c r="H22" s="8">
         <v>0</v>
       </c>
       <c r="I22" s="9">
+        <v>0</v>
+      </c>
+      <c r="J22" s="9">
         <v>80</v>
       </c>
-      <c r="J22" s="9"/>
       <c r="K22" s="9"/>
-    </row>
-    <row r="23" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L22" s="9"/>
+    </row>
+    <row r="23" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>19</v>
       </c>
       <c r="B23">
         <v>0</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23">
+        <v>17.5</v>
+      </c>
+      <c r="E23" s="3">
         <v>0.18</v>
       </c>
-      <c r="E23" s="5">
-        <v>0</v>
-      </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="5">
+        <v>0</v>
+      </c>
+      <c r="G23" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G23" s="8">
-        <v>0</v>
-      </c>
-      <c r="H23" s="9">
+      <c r="H23" s="8">
         <v>0</v>
       </c>
       <c r="I23" s="9">
+        <v>0</v>
+      </c>
+      <c r="J23" s="9">
         <v>130</v>
       </c>
-      <c r="J23" s="9"/>
       <c r="K23" s="9"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L23" s="9"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>20</v>
       </c>
       <c r="B24">
         <v>0</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D24">
+        <v>95</v>
+      </c>
+      <c r="E24" s="3">
         <v>0.35</v>
       </c>
-      <c r="E24" s="5">
+      <c r="F24" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="G24" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G24" s="8">
-        <v>0</v>
-      </c>
-      <c r="H24" s="9">
+      <c r="H24" s="8">
         <v>0</v>
       </c>
       <c r="I24" s="9">
+        <v>0</v>
+      </c>
+      <c r="J24" s="9">
         <v>120</v>
       </c>
-      <c r="J24" s="9"/>
       <c r="K24" s="9"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L24" s="9"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>21</v>
       </c>
       <c r="B25">
         <v>0</v>
       </c>
-      <c r="D25" s="3">
+      <c r="D25">
+        <v>93.2</v>
+      </c>
+      <c r="E25" s="3">
         <v>0.35</v>
       </c>
-      <c r="E25" s="5">
+      <c r="F25" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="G25" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G25" s="8">
-        <v>0</v>
-      </c>
-      <c r="H25" s="9">
+      <c r="H25" s="8">
         <v>0</v>
       </c>
       <c r="I25" s="9">
+        <v>0</v>
+      </c>
+      <c r="J25" s="9">
         <v>60</v>
       </c>
-      <c r="J25" s="9"/>
       <c r="K25" s="9"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L25" s="9"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>22</v>
       </c>
       <c r="B26">
         <v>0.82</v>
       </c>
-      <c r="D26" s="3">
+      <c r="E26" s="3">
         <v>1</v>
       </c>
-      <c r="E26" s="5">
+      <c r="F26" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="G26" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G26" s="8">
-        <v>0</v>
-      </c>
-      <c r="H26" s="9">
+      <c r="H26" s="8">
+        <v>0</v>
+      </c>
+      <c r="I26" s="9">
         <v>1.3</v>
       </c>
-      <c r="I26" s="9">
-        <v>0</v>
-      </c>
-      <c r="J26" s="9"/>
+      <c r="J26" s="9">
+        <v>0</v>
+      </c>
       <c r="K26" s="9"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L26" s="9"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>23</v>
       </c>
       <c r="B27">
         <v>0</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D27">
+        <v>7.8</v>
+      </c>
+      <c r="E27" s="3">
         <v>0.36</v>
       </c>
-      <c r="E27" s="5">
+      <c r="F27" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="G27" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G27" s="8">
-        <v>0</v>
-      </c>
-      <c r="H27" s="9">
+      <c r="H27" s="8">
         <v>0</v>
       </c>
       <c r="I27" s="9">
+        <v>0</v>
+      </c>
+      <c r="J27" s="9">
         <v>300</v>
       </c>
-      <c r="J27" s="9"/>
       <c r="K27" s="9"/>
-    </row>
-    <row r="28" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L27" s="9"/>
+    </row>
+    <row r="28" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>24</v>
       </c>
       <c r="B28">
         <v>0.38</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28">
+        <v>17</v>
+      </c>
+      <c r="E28" s="3">
         <v>1.25</v>
       </c>
-      <c r="E28" s="6">
-        <v>0</v>
-      </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="6">
+        <v>0</v>
+      </c>
+      <c r="G28" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="G28" s="8">
-        <v>0</v>
-      </c>
-      <c r="H28" s="9">
+      <c r="H28" s="8">
         <v>0</v>
       </c>
       <c r="I28" s="9">
+        <v>0</v>
+      </c>
+      <c r="J28" s="9">
         <v>150</v>
       </c>
-      <c r="J28" s="9"/>
       <c r="K28" s="9"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L28" s="9"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>25</v>
       </c>
       <c r="B29">
         <v>0</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D29">
+        <v>88</v>
+      </c>
+      <c r="E29" s="3">
         <v>3.5</v>
       </c>
-      <c r="E29" s="5">
+      <c r="F29" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="G29" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G29" s="8">
+      <c r="H29" s="8">
         <v>1.23</v>
       </c>
-      <c r="H29" s="9">
-        <v>0</v>
-      </c>
       <c r="I29" s="9">
         <v>0</v>
       </c>
-      <c r="J29" s="9"/>
+      <c r="J29" s="9">
+        <v>0</v>
+      </c>
       <c r="K29" s="9"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L29" s="9"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>26</v>
       </c>
       <c r="B30">
         <v>0.08</v>
       </c>
-      <c r="D30" s="3">
+      <c r="D30">
+        <v>87</v>
+      </c>
+      <c r="E30" s="3">
         <v>3.6</v>
       </c>
-      <c r="E30" s="5">
+      <c r="F30" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="G30" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G30" s="8">
+      <c r="H30" s="8">
         <v>1.23</v>
       </c>
-      <c r="H30" s="9">
-        <v>0</v>
-      </c>
       <c r="I30" s="9">
         <v>0</v>
       </c>
-      <c r="J30" s="9"/>
+      <c r="J30" s="9">
+        <v>0</v>
+      </c>
       <c r="K30" s="9"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L30" s="9"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>28</v>
       </c>
       <c r="B31">
         <v>0.08</v>
       </c>
-      <c r="D31" s="3">
+      <c r="D31">
+        <v>18</v>
+      </c>
+      <c r="E31" s="3">
         <v>0.5</v>
       </c>
-      <c r="E31" s="5">
+      <c r="F31" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="G31" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G31" s="8">
+      <c r="H31" s="8">
         <v>1.23</v>
       </c>
-      <c r="H31" s="9">
-        <v>0</v>
-      </c>
       <c r="I31" s="9">
         <v>0</v>
       </c>
-      <c r="J31" s="9"/>
+      <c r="J31" s="9">
+        <v>0</v>
+      </c>
       <c r="K31" s="9"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L31" s="9"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>27</v>
       </c>
       <c r="B32">
         <v>0</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32">
+        <v>88</v>
+      </c>
+      <c r="E32" s="3">
         <v>3.6</v>
       </c>
-      <c r="E32" s="5">
+      <c r="F32" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="G32" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G32" s="8">
+      <c r="H32" s="8">
         <v>1.23</v>
       </c>
-      <c r="H32" s="9">
-        <v>0</v>
-      </c>
       <c r="I32" s="9">
         <v>0</v>
       </c>
-      <c r="J32" s="9"/>
+      <c r="J32" s="9">
+        <v>0</v>
+      </c>
       <c r="K32" s="9"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L32" s="9"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>29</v>
       </c>
       <c r="B33">
         <v>0</v>
       </c>
-      <c r="D33" s="3">
+      <c r="D33">
+        <v>87.7</v>
+      </c>
+      <c r="E33" s="3">
         <v>1.5</v>
       </c>
-      <c r="E33" s="5">
+      <c r="F33" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="G33" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G33" s="8">
+      <c r="H33" s="8">
         <v>1.23</v>
       </c>
-      <c r="H33" s="9">
-        <v>0</v>
-      </c>
       <c r="I33" s="9">
         <v>0</v>
       </c>
-      <c r="J33" s="9"/>
+      <c r="J33" s="9">
+        <v>0</v>
+      </c>
       <c r="K33" s="9"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L33" s="9"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>30</v>
       </c>
       <c r="B34">
         <v>0</v>
       </c>
-      <c r="D34" s="3">
+      <c r="D34">
+        <v>10.3</v>
+      </c>
+      <c r="E34" s="3">
         <v>0.5</v>
       </c>
-      <c r="E34" s="5">
+      <c r="F34" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="G34" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G34" s="8">
+      <c r="H34" s="8">
         <v>1.23</v>
       </c>
-      <c r="H34" s="9">
-        <v>0</v>
-      </c>
       <c r="I34" s="9">
         <v>0</v>
       </c>
-      <c r="J34" s="9"/>
+      <c r="J34" s="9">
+        <v>0</v>
+      </c>
       <c r="K34" s="9"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L34" s="9"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>31</v>
       </c>
       <c r="B35">
         <v>0</v>
       </c>
-      <c r="D35" s="3">
+      <c r="D35">
+        <v>90</v>
+      </c>
+      <c r="E35" s="3">
         <v>6</v>
       </c>
-      <c r="E35" s="5">
+      <c r="F35" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="G35" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G35" s="8">
+      <c r="H35" s="8">
         <v>1.23</v>
       </c>
-      <c r="H35" s="9">
-        <v>0</v>
-      </c>
       <c r="I35" s="9">
         <v>0</v>
       </c>
-      <c r="J35" s="9"/>
+      <c r="J35" s="9">
+        <v>0</v>
+      </c>
       <c r="K35" s="9"/>
-    </row>
-    <row r="36" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L35" s="9"/>
+    </row>
+    <row r="36" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>32</v>
       </c>
       <c r="B36">
         <v>0</v>
       </c>
-      <c r="D36" s="3">
+      <c r="D36">
+        <v>17.7</v>
+      </c>
+      <c r="E36" s="3">
         <v>2.8</v>
       </c>
-      <c r="E36" s="5">
-        <v>0</v>
-      </c>
-      <c r="F36" s="7" t="s">
+      <c r="F36" s="5">
+        <v>0</v>
+      </c>
+      <c r="G36" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="G36" s="8">
+      <c r="H36" s="8">
         <v>1.47</v>
       </c>
-      <c r="H36" s="9">
-        <v>0</v>
-      </c>
       <c r="I36" s="9">
         <v>0</v>
       </c>
-      <c r="J36" s="9"/>
+      <c r="J36" s="9">
+        <v>0</v>
+      </c>
       <c r="K36" s="9"/>
-    </row>
-    <row r="37" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L36" s="9"/>
+    </row>
+    <row r="37" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>39</v>
       </c>
       <c r="B37">
         <v>0.25</v>
       </c>
-      <c r="D37" s="3">
+      <c r="D37">
+        <v>86</v>
+      </c>
+      <c r="E37" s="3">
         <v>2.0499999999999998</v>
       </c>
-      <c r="E37" s="6">
-        <v>0</v>
-      </c>
-      <c r="F37" s="7" t="s">
+      <c r="F37" s="6">
+        <v>0</v>
+      </c>
+      <c r="G37" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="G37" s="8">
+      <c r="H37" s="8">
         <v>0.36749999999999999</v>
       </c>
-      <c r="H37" s="9">
-        <v>0</v>
-      </c>
       <c r="I37" s="9">
+        <v>0</v>
+      </c>
+      <c r="J37" s="9">
         <v>150</v>
       </c>
-      <c r="J37" s="9"/>
       <c r="K37" s="9"/>
+      <c r="L37" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2356,10 +2507,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0C8FA35-4843-4FEC-9720-CB1F6CC19C35}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
     <col min="7" max="7" width="17.36328125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2371,7 +2523,7 @@
         <v>142</v>
       </c>
       <c r="C1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D1" t="s">
         <v>89</v>
@@ -2379,282 +2531,403 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B2">
         <v>3.0999999999999999E-3</v>
       </c>
       <c r="C2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D2" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B3">
-        <v>3.0999999999999999E-3</v>
+        <v>2.5026398888888901E-3</v>
       </c>
       <c r="C3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B4">
-        <v>3.5500000000000002E-3</v>
+        <v>2.5191576000000004E-3</v>
       </c>
       <c r="C4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B5">
-        <v>2.8999999999999998E-3</v>
+        <v>3.4014885333333339E-3</v>
       </c>
       <c r="C5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B6">
-        <v>3.5E-4</v>
+        <v>8.9999999999999998E-4</v>
       </c>
       <c r="C6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B7">
-        <v>8.9999999999999998E-4</v>
+        <v>5.5000000000000003E-4</v>
       </c>
       <c r="C7" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B8">
-        <v>5.5000000000000003E-4</v>
+        <v>5.5731720329999998E-4</v>
       </c>
       <c r="C8" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D8" t="s">
-        <v>165</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>153</v>
+        <v>22</v>
       </c>
       <c r="B9">
-        <v>2.0999999999999999E-3</v>
+        <v>2.8934473500000003E-3</v>
       </c>
       <c r="C9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D9" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="B10">
-        <v>3.0999999999999999E-3</v>
+        <v>2.5331492083333334E-3</v>
       </c>
       <c r="C10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D10" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>154</v>
+        <v>178</v>
       </c>
       <c r="B11">
-        <v>2.0999999999999999E-3</v>
+        <v>2.5165149883414934E-3</v>
       </c>
       <c r="C11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>155</v>
+        <v>177</v>
       </c>
       <c r="B12">
-        <v>2.5500000000000002E-3</v>
+        <v>2.44344375E-3</v>
       </c>
       <c r="C12" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D12" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B13">
-        <v>5.8E-4</v>
+        <v>2.2090262539682538E-3</v>
       </c>
       <c r="C13" t="s">
+        <v>162</v>
+      </c>
+      <c r="D13" t="s">
         <v>164</v>
-      </c>
-      <c r="D13" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B14">
-        <v>5.5000000000000003E-4</v>
+        <v>5.8E-4</v>
       </c>
       <c r="C14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D14" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="B15">
-        <v>4.4999999999999999E-4</v>
+        <v>5.5000000000000003E-4</v>
       </c>
       <c r="C15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D15" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>157</v>
+      </c>
+      <c r="B16">
+        <v>4.4999999999999999E-4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D16" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>158</v>
+      </c>
+      <c r="B17">
+        <v>7.5000000000000002E-4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>163</v>
+      </c>
+      <c r="D17" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
         <v>159</v>
       </c>
-      <c r="B16">
-        <v>7.5000000000000002E-4</v>
-      </c>
-      <c r="C16" t="s">
-        <v>164</v>
-      </c>
-      <c r="D16" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="B18">
+        <v>2.0631828E-4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>163</v>
+      </c>
+      <c r="D18" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
         <v>160</v>
       </c>
-      <c r="B17">
-        <v>9.0000000000000006E-5</v>
-      </c>
-      <c r="C17" t="s">
-        <v>164</v>
-      </c>
-      <c r="D17" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+      <c r="B19">
+        <v>5.4262139775921735E-4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>163</v>
+      </c>
+      <c r="D19" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
         <v>147</v>
       </c>
-      <c r="B18">
-        <v>1.7000000000000001E-4</v>
-      </c>
-      <c r="C18" t="s">
-        <v>164</v>
-      </c>
-      <c r="D18" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>161</v>
-      </c>
-      <c r="B19">
-        <v>5.9999999999999995E-4</v>
-      </c>
-      <c r="C19" t="s">
-        <v>164</v>
-      </c>
-      <c r="D19" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+      <c r="B20">
+        <v>2.3440000000000003E-4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>163</v>
+      </c>
+      <c r="D20" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>145</v>
       </c>
-      <c r="B20">
-        <v>4.0000000000000002E-4</v>
-      </c>
-      <c r="C20" t="s">
-        <v>164</v>
-      </c>
-      <c r="D20" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+      <c r="B21">
+        <v>2.9231999999999999E-4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>163</v>
+      </c>
+      <c r="D21" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>146</v>
       </c>
-      <c r="B21">
-        <v>1.6000000000000001E-3</v>
-      </c>
-      <c r="C21" t="s">
-        <v>164</v>
-      </c>
-      <c r="D21" t="s">
-        <v>168</v>
+      <c r="B22">
+        <v>1.5964523839999997E-3</v>
+      </c>
+      <c r="C22" t="s">
+        <v>163</v>
+      </c>
+      <c r="D22" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>169</v>
+      </c>
+      <c r="B23">
+        <v>1.8285932799999999E-3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>163</v>
+      </c>
+      <c r="D23" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>170</v>
+      </c>
+      <c r="B24">
+        <v>3.6662312908139748E-4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>163</v>
+      </c>
+      <c r="D24" t="s">
+        <v>167</v>
+      </c>
+      <c r="E24" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>171</v>
+      </c>
+      <c r="B25">
+        <v>3.6662312908139748E-4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>163</v>
+      </c>
+      <c r="D25" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>172</v>
+      </c>
+      <c r="B26">
+        <v>1.1635199999999999E-3</v>
+      </c>
+      <c r="C26" t="s">
+        <v>163</v>
+      </c>
+      <c r="D26" t="s">
+        <v>167</v>
+      </c>
+      <c r="E26" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>173</v>
+      </c>
+      <c r="B27">
+        <v>1.1635199999999999E-3</v>
+      </c>
+      <c r="C27" t="s">
+        <v>163</v>
+      </c>
+      <c r="D27" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>175</v>
+      </c>
+      <c r="B28">
+        <v>5.7248880000000007E-4</v>
+      </c>
+      <c r="C28" t="s">
+        <v>163</v>
+      </c>
+      <c r="D28" t="s">
+        <v>167</v>
+      </c>
+      <c r="E28" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>176</v>
+      </c>
+      <c r="B29">
+        <v>5.7248880000000007E-4</v>
+      </c>
+      <c r="C29" t="s">
+        <v>163</v>
+      </c>
+      <c r="D29" t="s">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
@@ -2663,6 +2936,242 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3D8FFD4-4EA9-47C1-BA4E-47263EF1D3B0}">
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.08984375" customWidth="1"/>
+    <col min="2" max="2" width="24.90625" customWidth="1"/>
+    <col min="3" max="3" width="18.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>155</v>
+      </c>
+      <c r="B2">
+        <v>5.8E-4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B3">
+        <v>2.0631828E-4</v>
+      </c>
+      <c r="C3" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>160</v>
+      </c>
+      <c r="B4">
+        <v>5.4262139775921735E-4</v>
+      </c>
+      <c r="C4" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5">
+        <v>2.3440000000000003E-4</v>
+      </c>
+      <c r="C5" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>145</v>
+      </c>
+      <c r="B6">
+        <v>2.9231999999999999E-4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>146</v>
+      </c>
+      <c r="B7">
+        <v>1.5964523839999997E-3</v>
+      </c>
+      <c r="C7" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>169</v>
+      </c>
+      <c r="B8">
+        <v>1.8285932799999999E-3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>170</v>
+      </c>
+      <c r="B9">
+        <v>3.6662312908139748E-4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>167</v>
+      </c>
+      <c r="D9" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>171</v>
+      </c>
+      <c r="B10">
+        <v>3.6662312908139748E-4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>172</v>
+      </c>
+      <c r="B11">
+        <v>1.1635199999999999E-3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>167</v>
+      </c>
+      <c r="D11" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>173</v>
+      </c>
+      <c r="B12">
+        <v>1.1635199999999999E-3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>175</v>
+      </c>
+      <c r="B13">
+        <v>5.7248880000000007E-4</v>
+      </c>
+      <c r="C13" t="s">
+        <v>167</v>
+      </c>
+      <c r="D13" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>176</v>
+      </c>
+      <c r="B14">
+        <v>5.7248880000000007E-4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B15">
+        <v>1.9282590170888892E-3</v>
+      </c>
+      <c r="C15" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16">
+        <v>7.789160266200002E-4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>153</v>
+      </c>
+      <c r="B17">
+        <v>5.5731720329999998E-4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>32</v>
+      </c>
+      <c r="B18">
+        <v>2.5331492083333334E-3</v>
+      </c>
+      <c r="C18" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>178</v>
+      </c>
+      <c r="B19">
+        <v>2.5165149883414934E-3</v>
+      </c>
+      <c r="C19" t="s">
+        <v>164</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDCA4DCB-FE4A-48BA-AD0E-D81C83744525}">
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -2675,7 +3184,7 @@
         <v>89</v>
       </c>
       <c r="B1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
@@ -2688,7 +3197,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B3">
         <v>0.06</v>
@@ -2704,7 +3213,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B5">
         <v>0.09</v>
@@ -2712,7 +3221,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B6">
         <v>0.04</v>
@@ -2720,7 +3229,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -2728,7 +3237,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -2736,7 +3245,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -2744,7 +3253,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B10">
         <v>0.79</v>
@@ -2755,7 +3264,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B24DCEF-E7C2-4526-9D13-3C67B63444AD}">
   <dimension ref="A1:AI3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3086,7 +3595,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12223D9-0A39-4CC4-B45B-34CE66BF62BA}">
   <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -3412,7 +3921,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D061B11-9C82-42EB-AFA7-28C01EBEFD7E}">
   <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Added available manure and slurry after volatilization columns in df_elevage
Added spread nitrogen from livestock in calculer_azote_epandu

Added Nitrogen content of slurry and manure in data_grafs.xlsx

modifications of objectives function and set up variables to compute methanization input and production.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C25F80B-7E4F-42E7-B425-8BF1D82792BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E11F330-AC30-455B-BE53-FC9C1877ADAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="2" activeTab="3" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="193">
   <si>
     <t>Culture</t>
   </si>
@@ -590,6 +590,36 @@
   </si>
   <si>
     <t>Methanization power (GWh/tMB)</t>
+  </si>
+  <si>
+    <t>Manure nitrogen Content (%)</t>
+  </si>
+  <si>
+    <t>Slurry nitrogen Content (%)</t>
+  </si>
+  <si>
+    <t>bovines waste</t>
+  </si>
+  <si>
+    <t>ovines waste</t>
+  </si>
+  <si>
+    <t>caprines waste</t>
+  </si>
+  <si>
+    <t>porcines waste</t>
+  </si>
+  <si>
+    <t>poultry waste</t>
+  </si>
+  <si>
+    <t>equines waste</t>
+  </si>
+  <si>
+    <t>Taken as bovines</t>
+  </si>
+  <si>
+    <t>Taken as ovines</t>
   </si>
 </sst>
 </file>
@@ -1014,6 +1044,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.7265625" customWidth="1"/>
+    <col min="2" max="2" width="18.1796875" customWidth="1"/>
     <col min="5" max="5" width="19.6328125" customWidth="1"/>
     <col min="6" max="6" width="14.90625" customWidth="1"/>
   </cols>
@@ -2937,11 +2968,11 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3D8FFD4-4EA9-47C1-BA4E-47263EF1D3B0}">
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.08984375" customWidth="1"/>
-    <col min="2" max="2" width="24.90625" customWidth="1"/>
+    <col min="2" max="2" width="29.1796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.90625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2961,10 +2992,10 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>155</v>
+        <v>185</v>
       </c>
       <c r="B2">
-        <v>5.8E-4</v>
+        <v>6.7174054999999996E-4</v>
       </c>
       <c r="C2" t="s">
         <v>166</v>
@@ -2972,65 +3003,71 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>159</v>
+        <v>186</v>
       </c>
       <c r="B3">
-        <v>2.0631828E-4</v>
+        <v>5.0052599999999992E-3</v>
       </c>
       <c r="C3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>160</v>
+        <v>187</v>
       </c>
       <c r="B4">
-        <v>5.4262139775921735E-4</v>
+        <v>5.0052599999999992E-3</v>
       </c>
       <c r="C4" t="s">
-        <v>167</v>
+        <v>166</v>
+      </c>
+      <c r="D4" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>188</v>
       </c>
       <c r="B5">
-        <v>2.3440000000000003E-4</v>
+        <v>4.3945200000000007E-3</v>
       </c>
       <c r="C5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>145</v>
+        <v>189</v>
       </c>
       <c r="B6">
-        <v>2.9231999999999999E-4</v>
+        <v>1.1705850000000001E-4</v>
       </c>
       <c r="C6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>146</v>
+        <v>190</v>
       </c>
       <c r="B7">
-        <v>1.5964523839999997E-3</v>
+        <v>6.7174054999999996E-4</v>
       </c>
       <c r="C7" t="s">
-        <v>167</v>
+        <v>166</v>
+      </c>
+      <c r="D7" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="B8">
-        <v>1.8285932799999999E-3</v>
+        <v>2.0631828E-4</v>
       </c>
       <c r="C8" t="s">
         <v>167</v>
@@ -3038,24 +3075,21 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="B9">
-        <v>3.6662312908139748E-4</v>
+        <v>5.4262139775921735E-4</v>
       </c>
       <c r="C9" t="s">
         <v>167</v>
       </c>
-      <c r="D9" t="s">
-        <v>174</v>
-      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>171</v>
+        <v>147</v>
       </c>
       <c r="B10">
-        <v>3.6662312908139748E-4</v>
+        <v>2.3440000000000003E-4</v>
       </c>
       <c r="C10" t="s">
         <v>167</v>
@@ -3063,24 +3097,21 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>172</v>
+        <v>145</v>
       </c>
       <c r="B11">
-        <v>1.1635199999999999E-3</v>
+        <v>2.9231999999999999E-4</v>
       </c>
       <c r="C11" t="s">
         <v>167</v>
       </c>
-      <c r="D11" t="s">
-        <v>174</v>
-      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>173</v>
+        <v>146</v>
       </c>
       <c r="B12">
-        <v>1.1635199999999999E-3</v>
+        <v>1.5964523839999997E-3</v>
       </c>
       <c r="C12" t="s">
         <v>167</v>
@@ -3088,81 +3119,142 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B13">
-        <v>5.7248880000000007E-4</v>
+        <v>1.8285932799999999E-3</v>
       </c>
       <c r="C13" t="s">
         <v>167</v>
       </c>
-      <c r="D13" t="s">
-        <v>174</v>
-      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="B14">
-        <v>5.7248880000000007E-4</v>
+        <v>3.6662312908139748E-4</v>
       </c>
       <c r="C14" t="s">
         <v>167</v>
       </c>
+      <c r="D14" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>6</v>
+        <v>171</v>
       </c>
       <c r="B15">
-        <v>1.9282590170888892E-3</v>
+        <v>3.6662312908139748E-4</v>
       </c>
       <c r="C15" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
+        <v>172</v>
+      </c>
+      <c r="B16">
+        <v>1.1635199999999999E-3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>167</v>
+      </c>
+      <c r="D16" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17">
+        <v>1.1635199999999999E-3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>175</v>
+      </c>
+      <c r="B18">
+        <v>5.7248880000000007E-4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>167</v>
+      </c>
+      <c r="D18" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>176</v>
+      </c>
+      <c r="B19">
+        <v>5.7248880000000007E-4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20">
+        <v>1.9282590170888892E-3</v>
+      </c>
+      <c r="C20" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>22</v>
       </c>
-      <c r="B16">
+      <c r="B21">
         <v>7.789160266200002E-4</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C21" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>153</v>
       </c>
-      <c r="B17">
+      <c r="B22">
         <v>5.5731720329999998E-4</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C22" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>32</v>
       </c>
-      <c r="B18">
+      <c r="B23">
         <v>2.5331492083333334E-3</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C23" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>178</v>
       </c>
-      <c r="B19">
+      <c r="B24">
         <v>2.5165149883414934E-3</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C24" t="s">
         <v>164</v>
       </c>
     </row>
@@ -3597,7 +3689,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12223D9-0A39-4CC4-B45B-34CE66BF62BA}">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="22.36328125" customWidth="1"/>
@@ -3610,7 +3702,7 @@
     <col min="9" max="9" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>40</v>
       </c>
@@ -3650,8 +3742,14 @@
       <c r="M1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N1" t="s">
+        <v>183</v>
+      </c>
+      <c r="O1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -3694,8 +3792,14 @@
       <c r="M2">
         <v>5.3E-3</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N2">
+        <v>0.49</v>
+      </c>
+      <c r="O2">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -3738,8 +3842,14 @@
       <c r="M3">
         <v>9.4000000000000004E-3</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N3">
+        <v>0.7</v>
+      </c>
+      <c r="O3">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -3782,8 +3892,14 @@
       <c r="M4">
         <v>9.4000000000000004E-3</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N4">
+        <v>1.96</v>
+      </c>
+      <c r="O4">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -3826,8 +3942,14 @@
       <c r="M5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N5">
+        <v>0.9</v>
+      </c>
+      <c r="O5">
+        <v>0.57999999999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>45</v>
       </c>
@@ -3870,8 +3992,14 @@
       <c r="M6">
         <v>1.7899999999999999E-2</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N6">
+        <v>3.95</v>
+      </c>
+      <c r="O6">
+        <v>3.68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -3913,6 +4041,12 @@
       </c>
       <c r="M7">
         <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0.41</v>
+      </c>
+      <c r="O7">
+        <v>0.41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added limits over organic nitrogen spreading.
improved sankey app display.

Take off Natural meadows from potential import.

Removed a change in NH3 and N2O emission without generate_flux...

Added correction on "other manure" category for emission

updated scenario.xlsx for methaniser production

updated meth production data with 2023 data
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F7E0EAA-C38A-4795-AACD-C92C0A4587FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A4C28D-35CC-4E52-91E2-E4EC4192805F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" activeTab="3" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-15165" yWindow="-16680" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
@@ -2367,106 +2367,107 @@
         <v>140</v>
       </c>
       <c r="B2">
-        <v>348</v>
+        <v>877</v>
       </c>
       <c r="C2">
-        <v>53</v>
+        <v>169</v>
       </c>
       <c r="D2">
-        <v>24</v>
+        <v>116</v>
       </c>
       <c r="E2">
-        <v>458</v>
+        <v>1437</v>
       </c>
       <c r="F2">
-        <v>97</v>
+        <v>534</v>
       </c>
       <c r="G2">
-        <v>63</v>
+        <v>131</v>
       </c>
       <c r="H2">
-        <v>65</v>
+        <v>122</v>
       </c>
       <c r="I2">
-        <v>275</v>
+        <v>604</v>
       </c>
       <c r="J2">
-        <v>548</v>
+        <v>1561</v>
       </c>
       <c r="K2">
-        <v>90</v>
+        <v>213</v>
       </c>
       <c r="L2">
-        <v>397</v>
+        <v>742</v>
       </c>
       <c r="M2">
-        <v>108</v>
+        <v>315</v>
       </c>
       <c r="N2">
-        <v>388</v>
+        <v>846</v>
       </c>
       <c r="O2">
-        <v>105</v>
+        <v>316</v>
       </c>
       <c r="P2">
-        <v>199</v>
+        <v>859</v>
       </c>
       <c r="Q2">
-        <v>99</v>
+        <v>479</v>
       </c>
       <c r="R2">
-        <v>115</v>
+        <v>571</v>
       </c>
       <c r="S2">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="T2">
-        <v>32</v>
+        <v>50</v>
       </c>
       <c r="U2">
-        <v>67</v>
+        <v>153</v>
       </c>
       <c r="V2">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="W2">
+        <v>196</v>
+      </c>
+      <c r="X2">
+        <v>75</v>
+      </c>
+      <c r="Y2">
+        <v>338</v>
+      </c>
+      <c r="Z2">
+        <v>189</v>
+      </c>
+      <c r="AA2">
+        <v>401</v>
+      </c>
+      <c r="AB2">
+        <v>149</v>
+      </c>
+      <c r="AC2">
         <v>71</v>
       </c>
-      <c r="X2">
-        <v>141</v>
-      </c>
-      <c r="Y2">
-        <v>197</v>
-      </c>
-      <c r="Z2">
-        <v>15</v>
-      </c>
-      <c r="AA2">
-        <v>79</v>
-      </c>
-      <c r="AB2">
-        <v>27</v>
-      </c>
-      <c r="AC2">
-        <v>56</v>
-      </c>
       <c r="AD2">
-        <v>68</v>
+        <v>29</v>
       </c>
       <c r="AE2">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="AF2">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="AG2">
         <v>12</v>
       </c>
       <c r="AH2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AI2">
-        <v>4337</v>
+        <f>SUM(B2:AH2)</f>
+        <v>11583</v>
       </c>
     </row>
     <row r="11" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>

</xml_diff>

<commit_message>
remove True in typology.
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -8,14 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65DA067B-9A3C-4317-A53A-A5FF14E4D8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A4C28D-35CC-4E52-91E2-E4EC4192805F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="-15165" yWindow="-16680" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
-    <sheet name="Volatilisation" sheetId="2" r:id="rId2"/>
-    <sheet name="N_syn" sheetId="3" r:id="rId3"/>
+    <sheet name="Energy_prod" sheetId="4" r:id="rId2"/>
+    <sheet name="Energy_power_old" sheetId="6" r:id="rId3"/>
+    <sheet name="Energy_power" sheetId="8" r:id="rId4"/>
+    <sheet name="Energy_regime" sheetId="7" r:id="rId5"/>
+    <sheet name="import_export" sheetId="5" r:id="rId6"/>
+    <sheet name="Volatilisation" sheetId="2" r:id="rId7"/>
+    <sheet name="N_syn" sheetId="3" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="205">
   <si>
     <t>Culture</t>
   </si>
@@ -348,13 +353,316 @@
   </si>
   <si>
     <t>temporary meadows</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Ile de France</t>
+  </si>
+  <si>
+    <t>Eure</t>
+  </si>
+  <si>
+    <t>Eure-et-Loir</t>
+  </si>
+  <si>
+    <t>Picardie</t>
+  </si>
+  <si>
+    <t>Calvados-Orne</t>
+  </si>
+  <si>
+    <t>Seine Maritime</t>
+  </si>
+  <si>
+    <t>Manche</t>
+  </si>
+  <si>
+    <t>Nord Pas de Calais</t>
+  </si>
+  <si>
+    <t>Champ-Ard-Yonne</t>
+  </si>
+  <si>
+    <t>Bourgogne</t>
+  </si>
+  <si>
+    <t>Grande Lorraine</t>
+  </si>
+  <si>
+    <t>Alsace</t>
+  </si>
+  <si>
+    <t>Bretagne</t>
+  </si>
+  <si>
+    <t>Vendée-Charente</t>
+  </si>
+  <si>
+    <t>Loire aval</t>
+  </si>
+  <si>
+    <t>Loire Centrale</t>
+  </si>
+  <si>
+    <t>Loire Amont</t>
+  </si>
+  <si>
+    <t>Grand Jura</t>
+  </si>
+  <si>
+    <t>Savoie</t>
+  </si>
+  <si>
+    <t>Ain-Rhône</t>
+  </si>
+  <si>
+    <t>Alpes</t>
+  </si>
+  <si>
+    <t>Isère-Drôme Ardèche</t>
+  </si>
+  <si>
+    <t>Aveyron-Lozère</t>
+  </si>
+  <si>
+    <t>Garonne</t>
+  </si>
+  <si>
+    <t>Gironde</t>
+  </si>
+  <si>
+    <t>Pyrénées occidentales</t>
+  </si>
+  <si>
+    <t>Landes</t>
+  </si>
+  <si>
+    <t>Dor-Lot</t>
+  </si>
+  <si>
+    <t>Cantal-Corrèze</t>
+  </si>
+  <si>
+    <t>Grand Marseille</t>
+  </si>
+  <si>
+    <t>Côte d'Azur</t>
+  </si>
+  <si>
+    <t>Gard-Hérault</t>
+  </si>
+  <si>
+    <t>Pyrénées Orientales</t>
+  </si>
+  <si>
+    <t>Import</t>
+  </si>
+  <si>
+    <t>Export</t>
+  </si>
+  <si>
+    <t>Méthaniseur</t>
+  </si>
+  <si>
+    <t>Item</t>
+  </si>
+  <si>
+    <t>Methanization power (GWh/tMS)</t>
+  </si>
+  <si>
+    <t>Rapeseed straw</t>
+  </si>
+  <si>
+    <t>Maize straw</t>
+  </si>
+  <si>
+    <t>Bovines manure</t>
+  </si>
+  <si>
+    <t>Poultry slurry</t>
+  </si>
+  <si>
+    <t>Bovines slurry</t>
+  </si>
+  <si>
+    <t>CIVE</t>
+  </si>
+  <si>
+    <t>Sunflower straw</t>
+  </si>
+  <si>
+    <t>Sugar beet residues</t>
+  </si>
+  <si>
+    <t>Soybean straw</t>
+  </si>
+  <si>
+    <t>Potatoes residues</t>
+  </si>
+  <si>
+    <t>Green waste</t>
+  </si>
+  <si>
+    <t>Cereal straw</t>
+  </si>
+  <si>
+    <t>Slaughterhouse IAA</t>
+  </si>
+  <si>
+    <t>Sludges</t>
+  </si>
+  <si>
+    <t>Waste IAA</t>
+  </si>
+  <si>
+    <t>Waste population</t>
+  </si>
+  <si>
+    <t>Porcines slurry</t>
+  </si>
+  <si>
+    <t>Porcines manure</t>
+  </si>
+  <si>
+    <t>MB</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Crop residues</t>
+  </si>
+  <si>
+    <t>Dedicated culture</t>
+  </si>
+  <si>
+    <t>Non edible animal</t>
+  </si>
+  <si>
+    <t>Livestock effluent</t>
+  </si>
+  <si>
+    <t>Share</t>
+  </si>
+  <si>
+    <t>Poultry manure</t>
+  </si>
+  <si>
+    <t>Caprines slurry</t>
+  </si>
+  <si>
+    <t>Caprines manure</t>
+  </si>
+  <si>
+    <t>Equines slurry</t>
+  </si>
+  <si>
+    <t>Equines manure</t>
+  </si>
+  <si>
+    <t>Taken as manure</t>
+  </si>
+  <si>
+    <t>Ovines slurry</t>
+  </si>
+  <si>
+    <t>Ovines manure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Natural meadows </t>
+  </si>
+  <si>
+    <t>Non legume temporary meadow</t>
+  </si>
+  <si>
+    <t>DM content (% of gross matter)</t>
+  </si>
+  <si>
+    <t>DM content done with https://www.feedtables.com/content/dry-matter and https://fdc.nal.usda.gov/</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Methanization power (GWh/tMB)</t>
+  </si>
+  <si>
+    <t>Manure nitrogen Content (%)</t>
+  </si>
+  <si>
+    <t>Slurry nitrogen Content (%)</t>
+  </si>
+  <si>
+    <t>bovines waste</t>
+  </si>
+  <si>
+    <t>ovines waste</t>
+  </si>
+  <si>
+    <t>caprines waste</t>
+  </si>
+  <si>
+    <t>porcines waste</t>
+  </si>
+  <si>
+    <t>poultry waste</t>
+  </si>
+  <si>
+    <t>Taken as bovines</t>
+  </si>
+  <si>
+    <t>Taken as ovines</t>
+  </si>
+  <si>
+    <t>bovines slurry</t>
+  </si>
+  <si>
+    <t>porcines manure</t>
+  </si>
+  <si>
+    <t>porcines slurry</t>
+  </si>
+  <si>
+    <t>bovines manure</t>
+  </si>
+  <si>
+    <t>poultry slurry</t>
+  </si>
+  <si>
+    <t>poultry manure</t>
+  </si>
+  <si>
+    <t>caprines slurry</t>
+  </si>
+  <si>
+    <t>caprines manure</t>
+  </si>
+  <si>
+    <t>ovines slurry</t>
+  </si>
+  <si>
+    <t>ovines manure</t>
+  </si>
+  <si>
+    <t>equine waste</t>
+  </si>
+  <si>
+    <t>equine slurry</t>
+  </si>
+  <si>
+    <t>equine manure</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -385,6 +693,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -394,7 +708,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -402,12 +716,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -426,6 +755,12 @@
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -741,15 +1076,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{973E28D2-5D19-4409-920F-79B00DDA2ABC}">
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.7265625" customWidth="1"/>
-    <col min="4" max="4" width="19.6328125" customWidth="1"/>
-    <col min="5" max="5" width="14.90625" customWidth="1"/>
+    <col min="2" max="2" width="18.1796875" customWidth="1"/>
+    <col min="5" max="5" width="19.6328125" customWidth="1"/>
+    <col min="6" max="6" width="14.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -760,221 +1096,248 @@
         <v>33</v>
       </c>
       <c r="D1" t="s">
+        <v>179</v>
+      </c>
+      <c r="E1" t="s">
         <v>84</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>88</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>89</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>90</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>99</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2">
         <v>0.12</v>
       </c>
-      <c r="D2" s="3">
+      <c r="C2" t="s">
+        <v>180</v>
+      </c>
+      <c r="D2">
+        <v>86.9</v>
+      </c>
+      <c r="E2" s="3">
         <v>1.95</v>
       </c>
-      <c r="E2" s="5">
+      <c r="F2" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="G2" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G2" s="8">
-        <v>0</v>
-      </c>
-      <c r="H2" s="3">
+      <c r="H2" s="8">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3">
         <v>3.5</v>
       </c>
-      <c r="I2" s="9">
-        <v>0</v>
-      </c>
-      <c r="J2" s="9"/>
+      <c r="J2" s="9">
+        <v>0</v>
+      </c>
       <c r="K2" s="9"/>
-    </row>
-    <row r="3" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="L2" s="9"/>
+    </row>
+    <row r="3" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>37</v>
       </c>
       <c r="B3">
         <v>0.03</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3">
+        <v>86.7</v>
+      </c>
+      <c r="E3" s="3">
         <v>1.76</v>
       </c>
-      <c r="E3" s="5">
+      <c r="F3" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F3" s="7" t="s">
+      <c r="G3" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G3" s="8">
-        <v>0</v>
-      </c>
-      <c r="H3" s="3">
+      <c r="H3" s="8">
+        <v>0</v>
+      </c>
+      <c r="I3" s="3">
         <v>2.2999999999999998</v>
       </c>
-      <c r="I3" s="9">
-        <v>0</v>
-      </c>
-      <c r="J3" s="9"/>
+      <c r="J3" s="9">
+        <v>0</v>
+      </c>
       <c r="K3" s="9"/>
-    </row>
-    <row r="4" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="L3" s="9"/>
+    </row>
+    <row r="4" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
       <c r="B4">
         <v>0.13</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4">
+        <v>87.2</v>
+      </c>
+      <c r="E4" s="3">
         <v>1.76</v>
       </c>
-      <c r="E4" s="5">
+      <c r="F4" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="G4" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G4" s="8">
-        <v>0</v>
-      </c>
-      <c r="H4" s="3">
+      <c r="H4" s="8">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3">
         <v>2.5</v>
       </c>
-      <c r="I4" s="9">
-        <v>0</v>
-      </c>
-      <c r="J4" s="9"/>
+      <c r="J4" s="9">
+        <v>0</v>
+      </c>
       <c r="K4" s="9"/>
-    </row>
-    <row r="5" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="L4" s="9"/>
+    </row>
+    <row r="5" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
       <c r="B5">
         <v>0.03</v>
       </c>
-      <c r="D5" s="3">
+      <c r="D5">
+        <v>87.6</v>
+      </c>
+      <c r="E5" s="3">
         <v>2.08</v>
       </c>
-      <c r="E5" s="5">
+      <c r="F5" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="G5" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G5" s="8">
-        <v>0</v>
-      </c>
-      <c r="H5" s="3">
+      <c r="H5" s="8">
+        <v>0</v>
+      </c>
+      <c r="I5" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="I5" s="9">
-        <v>0</v>
-      </c>
-      <c r="J5" s="9"/>
+      <c r="J5" s="9">
+        <v>0</v>
+      </c>
       <c r="K5" s="9"/>
-    </row>
-    <row r="6" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="L5" s="9"/>
+    </row>
+    <row r="6" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="B6">
         <v>0.4</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6">
+        <v>86.3</v>
+      </c>
+      <c r="E6" s="3">
         <v>1.52</v>
       </c>
-      <c r="E6" s="5">
+      <c r="F6" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="G6" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G6" s="8">
-        <v>0</v>
-      </c>
-      <c r="H6" s="3">
+      <c r="H6" s="8">
+        <v>0</v>
+      </c>
+      <c r="I6" s="3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="I6" s="9">
-        <v>0</v>
-      </c>
-      <c r="J6" s="9"/>
+      <c r="J6" s="9">
+        <v>0</v>
+      </c>
       <c r="K6" s="9"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L6" s="9"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>100</v>
       </c>
       <c r="B7">
         <v>0.03</v>
       </c>
-      <c r="D7" s="3">
+      <c r="D7">
+        <v>88</v>
+      </c>
+      <c r="E7" s="3">
         <v>1.07</v>
       </c>
-      <c r="E7" s="5">
+      <c r="F7" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="G7" s="7" t="s">
         <v>87</v>
       </c>
-      <c r="G7" s="8">
-        <v>0</v>
-      </c>
-      <c r="H7" s="3">
-        <v>0</v>
-      </c>
-      <c r="I7" s="9">
+      <c r="H7" s="8">
+        <v>0</v>
+      </c>
+      <c r="I7" s="3">
+        <v>0</v>
+      </c>
+      <c r="J7" s="9">
         <v>125</v>
       </c>
-      <c r="J7" s="9"/>
       <c r="K7" s="9"/>
-    </row>
-    <row r="8" spans="1:11" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="L7" s="9"/>
+    </row>
+    <row r="8" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>5</v>
       </c>
       <c r="B8">
         <v>0.03</v>
       </c>
-      <c r="D8" s="3">
+      <c r="D8">
+        <v>89.6</v>
+      </c>
+      <c r="E8" s="3">
         <v>1.8</v>
       </c>
-      <c r="E8" s="5">
+      <c r="F8" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F8" s="7" t="s">
+      <c r="G8" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="G8" s="8">
-        <v>0</v>
-      </c>
-      <c r="H8" s="3">
+      <c r="H8" s="8">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3">
         <v>2.6</v>
       </c>
-      <c r="I8" s="9">
-        <v>0</v>
-      </c>
-      <c r="J8" s="9"/>
+      <c r="J8" s="9">
+        <v>0</v>
+      </c>
       <c r="K8" s="9"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L8" s="9"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>6</v>
       </c>
@@ -984,168 +1347,186 @@
       <c r="C9" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="3">
+      <c r="D9">
+        <v>90.3</v>
+      </c>
+      <c r="E9" s="3">
         <v>0.5</v>
       </c>
-      <c r="E9" s="5">
-        <v>0</v>
-      </c>
-      <c r="F9" s="7" t="s">
+      <c r="F9" s="5">
+        <v>0</v>
+      </c>
+      <c r="G9" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G9" s="8">
-        <v>0</v>
-      </c>
-      <c r="H9" s="3">
+      <c r="H9" s="8">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3">
         <v>3</v>
       </c>
-      <c r="I9" s="9">
-        <v>0</v>
-      </c>
-      <c r="J9" s="9"/>
+      <c r="J9" s="9">
+        <v>0</v>
+      </c>
       <c r="K9" s="9"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L9" s="9"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>7</v>
       </c>
       <c r="B10">
         <v>0.33</v>
       </c>
-      <c r="D10" s="3">
+      <c r="D10">
+        <v>92.4</v>
+      </c>
+      <c r="E10" s="3">
         <v>3.5</v>
       </c>
-      <c r="E10" s="5">
+      <c r="F10" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F10" s="7" t="s">
+      <c r="G10" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G10" s="8">
-        <v>0</v>
-      </c>
-      <c r="H10" s="3">
+      <c r="H10" s="8">
+        <v>0</v>
+      </c>
+      <c r="I10" s="3">
         <v>7</v>
       </c>
-      <c r="I10" s="9">
-        <v>0</v>
-      </c>
-      <c r="J10" s="9"/>
+      <c r="J10" s="9">
+        <v>0</v>
+      </c>
       <c r="K10" s="9"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L10" s="9"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>8</v>
       </c>
       <c r="B11">
         <v>0.16</v>
       </c>
-      <c r="D11" s="3">
+      <c r="D11">
+        <v>92.8</v>
+      </c>
+      <c r="E11" s="3">
         <v>1.96</v>
       </c>
-      <c r="E11" s="5">
+      <c r="F11" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F11" s="7" t="s">
+      <c r="G11" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G11" s="8">
-        <v>0</v>
-      </c>
-      <c r="H11" s="3">
+      <c r="H11" s="8">
+        <v>0</v>
+      </c>
+      <c r="I11" s="3">
         <v>4.5</v>
       </c>
-      <c r="I11" s="9">
-        <v>0</v>
-      </c>
-      <c r="J11" s="9"/>
+      <c r="J11" s="9">
+        <v>0</v>
+      </c>
       <c r="K11" s="9"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L11" s="9"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>9</v>
       </c>
       <c r="B12">
         <v>0</v>
       </c>
-      <c r="D12" s="4">
+      <c r="D12">
+        <v>88.1</v>
+      </c>
+      <c r="E12" s="4">
         <v>3.5</v>
       </c>
-      <c r="E12" s="5">
+      <c r="F12" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F12" s="7" t="s">
+      <c r="G12" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G12" s="8">
-        <v>0</v>
-      </c>
-      <c r="H12" s="9">
+      <c r="H12" s="8">
+        <v>0</v>
+      </c>
+      <c r="I12" s="9">
         <v>5</v>
       </c>
-      <c r="I12" s="9">
-        <v>0</v>
-      </c>
-      <c r="J12" s="9"/>
+      <c r="J12" s="9">
+        <v>0</v>
+      </c>
       <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L12" s="9"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>10</v>
       </c>
       <c r="B13">
         <v>0.56000000000000005</v>
       </c>
-      <c r="D13" s="3">
+      <c r="D13">
+        <v>17.8</v>
+      </c>
+      <c r="E13" s="3">
         <v>0.20799999999999999</v>
       </c>
-      <c r="E13" s="5">
+      <c r="F13" s="5">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="F13" s="7" t="s">
+      <c r="G13" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G13" s="8">
-        <v>0</v>
-      </c>
-      <c r="H13" s="9">
+      <c r="H13" s="8">
         <v>0</v>
       </c>
       <c r="I13" s="9">
+        <v>0</v>
+      </c>
+      <c r="J13" s="9">
         <v>220</v>
       </c>
-      <c r="J13" s="9"/>
       <c r="K13" s="9"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L13" s="9"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>11</v>
       </c>
       <c r="B14">
         <v>0.35</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14">
+        <v>18.899999999999999</v>
+      </c>
+      <c r="E14" s="3">
         <v>0.25600000000000001</v>
       </c>
-      <c r="E14" s="5">
+      <c r="F14" s="5">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="F14" s="7" t="s">
+      <c r="G14" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G14" s="8">
-        <v>0</v>
-      </c>
-      <c r="H14" s="9">
+      <c r="H14" s="8">
         <v>0</v>
       </c>
       <c r="I14" s="9">
+        <v>0</v>
+      </c>
+      <c r="J14" s="9">
         <v>220</v>
       </c>
-      <c r="J14" s="9"/>
       <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L14" s="9"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>12</v>
       </c>
@@ -1155,28 +1536,31 @@
       <c r="C15" t="s">
         <v>35</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15">
+        <v>17.8</v>
+      </c>
+      <c r="E15" s="3">
         <v>0.23</v>
       </c>
-      <c r="E15" s="5">
+      <c r="F15" s="5">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="F15" s="7" t="s">
+      <c r="G15" s="7" t="s">
         <v>94</v>
       </c>
-      <c r="G15" s="8">
-        <v>0</v>
-      </c>
-      <c r="H15" s="9">
+      <c r="H15" s="8">
         <v>0</v>
       </c>
       <c r="I15" s="9">
+        <v>0</v>
+      </c>
+      <c r="J15" s="9">
         <v>220</v>
       </c>
-      <c r="J15" s="9"/>
       <c r="K15" s="9"/>
-    </row>
-    <row r="16" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L15" s="9"/>
+    </row>
+    <row r="16" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -1186,614 +1570,680 @@
       <c r="C16" t="s">
         <v>36</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16">
+        <v>88.4</v>
+      </c>
+      <c r="E16" s="3">
         <v>3.6</v>
       </c>
-      <c r="E16" s="5">
+      <c r="F16" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F16" s="7" t="s">
+      <c r="G16" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G16" s="8">
-        <v>0</v>
-      </c>
-      <c r="H16" s="9">
+      <c r="H16" s="8">
         <v>0</v>
       </c>
       <c r="I16" s="9">
+        <v>0</v>
+      </c>
+      <c r="J16" s="9">
         <v>50</v>
       </c>
-      <c r="J16" s="9"/>
       <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L16" s="9"/>
+    </row>
+    <row r="17" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>14</v>
       </c>
       <c r="B17">
         <v>0</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17">
+        <v>80</v>
+      </c>
+      <c r="E17" s="3">
         <v>2</v>
       </c>
-      <c r="E17" s="5">
+      <c r="F17" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F17" s="7" t="s">
+      <c r="G17" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G17" s="8">
-        <v>0</v>
-      </c>
-      <c r="H17" s="9">
+      <c r="H17" s="8">
         <v>0</v>
       </c>
       <c r="I17" s="9">
+        <v>0</v>
+      </c>
+      <c r="J17" s="9">
         <v>100</v>
       </c>
-      <c r="J17" s="9"/>
       <c r="K17" s="9"/>
-    </row>
-    <row r="18" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L17" s="9"/>
+    </row>
+    <row r="18" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>38</v>
       </c>
       <c r="B18">
         <v>0</v>
       </c>
-      <c r="D18" s="3">
+      <c r="D18">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="E18" s="3">
         <v>0.18</v>
       </c>
-      <c r="E18" s="5">
+      <c r="F18" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F18" s="7" t="s">
+      <c r="G18" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G18" s="8">
-        <v>0</v>
-      </c>
-      <c r="H18" s="9">
+      <c r="H18" s="8">
         <v>0</v>
       </c>
       <c r="I18" s="9">
+        <v>0</v>
+      </c>
+      <c r="J18" s="9">
         <v>180</v>
       </c>
-      <c r="J18" s="9"/>
       <c r="K18" s="9"/>
-    </row>
-    <row r="19" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L18" s="9"/>
+    </row>
+    <row r="19" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>15</v>
       </c>
       <c r="B19">
         <v>0</v>
       </c>
-      <c r="D19" s="3">
+      <c r="D19">
+        <v>8.1</v>
+      </c>
+      <c r="E19" s="3">
         <v>0.36</v>
       </c>
-      <c r="E19" s="5">
+      <c r="F19" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F19" s="7" t="s">
+      <c r="G19" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G19" s="8">
-        <v>0</v>
-      </c>
-      <c r="H19" s="9">
+      <c r="H19" s="8">
         <v>0</v>
       </c>
       <c r="I19" s="9">
+        <v>0</v>
+      </c>
+      <c r="J19" s="9">
         <v>300</v>
       </c>
-      <c r="J19" s="9"/>
       <c r="K19" s="9"/>
-    </row>
-    <row r="20" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L19" s="9"/>
+    </row>
+    <row r="20" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>16</v>
       </c>
       <c r="B20">
         <v>0</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20">
+        <v>4.5</v>
+      </c>
+      <c r="E20" s="3">
         <v>0.22</v>
       </c>
-      <c r="E20" s="5">
+      <c r="F20" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F20" s="7" t="s">
+      <c r="G20" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G20" s="8">
-        <v>0</v>
-      </c>
-      <c r="H20" s="9">
+      <c r="H20" s="8">
         <v>0</v>
       </c>
       <c r="I20" s="9">
+        <v>0</v>
+      </c>
+      <c r="J20" s="9">
         <v>150</v>
       </c>
-      <c r="J20" s="9"/>
       <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L20" s="9"/>
+    </row>
+    <row r="21" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>17</v>
       </c>
       <c r="B21">
         <v>0</v>
       </c>
-      <c r="D21" s="3">
+      <c r="D21">
+        <v>16.399999999999999</v>
+      </c>
+      <c r="E21" s="3">
         <v>0.1</v>
       </c>
-      <c r="E21" s="5">
-        <v>0</v>
-      </c>
-      <c r="F21" s="7" t="s">
+      <c r="F21" s="5">
+        <v>0</v>
+      </c>
+      <c r="G21" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G21" s="8">
-        <v>0</v>
-      </c>
-      <c r="H21" s="9">
+      <c r="H21" s="8">
         <v>0</v>
       </c>
       <c r="I21" s="9">
+        <v>0</v>
+      </c>
+      <c r="J21" s="9">
         <v>100</v>
       </c>
-      <c r="J21" s="9"/>
       <c r="K21" s="9"/>
-    </row>
-    <row r="22" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L21" s="9"/>
+    </row>
+    <row r="22" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>18</v>
       </c>
       <c r="B22">
         <v>0</v>
       </c>
-      <c r="D22" s="3">
+      <c r="D22">
+        <v>24.7</v>
+      </c>
+      <c r="E22" s="3">
         <v>0.67</v>
       </c>
-      <c r="E22" s="5">
-        <v>0</v>
-      </c>
-      <c r="F22" s="7" t="s">
+      <c r="F22" s="5">
+        <v>0</v>
+      </c>
+      <c r="G22" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G22" s="8">
-        <v>0</v>
-      </c>
-      <c r="H22" s="9">
+      <c r="H22" s="8">
         <v>0</v>
       </c>
       <c r="I22" s="9">
+        <v>0</v>
+      </c>
+      <c r="J22" s="9">
         <v>80</v>
       </c>
-      <c r="J22" s="9"/>
       <c r="K22" s="9"/>
-    </row>
-    <row r="23" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L22" s="9"/>
+    </row>
+    <row r="23" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>19</v>
       </c>
       <c r="B23">
         <v>0</v>
       </c>
-      <c r="D23" s="3">
+      <c r="D23">
+        <v>17.5</v>
+      </c>
+      <c r="E23" s="3">
         <v>0.18</v>
       </c>
-      <c r="E23" s="5">
-        <v>0</v>
-      </c>
-      <c r="F23" s="7" t="s">
+      <c r="F23" s="5">
+        <v>0</v>
+      </c>
+      <c r="G23" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="G23" s="8">
-        <v>0</v>
-      </c>
-      <c r="H23" s="9">
+      <c r="H23" s="8">
         <v>0</v>
       </c>
       <c r="I23" s="9">
+        <v>0</v>
+      </c>
+      <c r="J23" s="9">
         <v>130</v>
       </c>
-      <c r="J23" s="9"/>
       <c r="K23" s="9"/>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L23" s="9"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>20</v>
       </c>
       <c r="B24">
         <v>0</v>
       </c>
-      <c r="D24" s="3">
+      <c r="D24">
+        <v>95</v>
+      </c>
+      <c r="E24" s="3">
         <v>0.35</v>
       </c>
-      <c r="E24" s="5">
+      <c r="F24" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F24" s="7" t="s">
+      <c r="G24" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G24" s="8">
-        <v>0</v>
-      </c>
-      <c r="H24" s="9">
+      <c r="H24" s="8">
         <v>0</v>
       </c>
       <c r="I24" s="9">
+        <v>0</v>
+      </c>
+      <c r="J24" s="9">
         <v>120</v>
       </c>
-      <c r="J24" s="9"/>
       <c r="K24" s="9"/>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L24" s="9"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>21</v>
       </c>
       <c r="B25">
         <v>0</v>
       </c>
-      <c r="D25" s="3">
+      <c r="D25">
+        <v>93.2</v>
+      </c>
+      <c r="E25" s="3">
         <v>0.35</v>
       </c>
-      <c r="E25" s="5">
+      <c r="F25" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F25" s="7" t="s">
+      <c r="G25" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="G25" s="8">
-        <v>0</v>
-      </c>
-      <c r="H25" s="9">
+      <c r="H25" s="8">
         <v>0</v>
       </c>
       <c r="I25" s="9">
+        <v>0</v>
+      </c>
+      <c r="J25" s="9">
         <v>60</v>
       </c>
-      <c r="J25" s="9"/>
       <c r="K25" s="9"/>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L25" s="9"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>22</v>
       </c>
       <c r="B26">
         <v>0.82</v>
       </c>
-      <c r="D26" s="3">
+      <c r="D26">
+        <v>32</v>
+      </c>
+      <c r="E26" s="3">
         <v>1</v>
       </c>
-      <c r="E26" s="5">
+      <c r="F26" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F26" s="7" t="s">
+      <c r="G26" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G26" s="8">
-        <v>0</v>
-      </c>
-      <c r="H26" s="9">
+      <c r="H26" s="8">
+        <v>0</v>
+      </c>
+      <c r="I26" s="9">
         <v>1.3</v>
       </c>
-      <c r="I26" s="9">
-        <v>0</v>
-      </c>
-      <c r="J26" s="9"/>
+      <c r="J26" s="9">
+        <v>0</v>
+      </c>
       <c r="K26" s="9"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L26" s="9"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>23</v>
       </c>
       <c r="B27">
         <v>0</v>
       </c>
-      <c r="D27" s="3">
+      <c r="D27">
+        <v>7.8</v>
+      </c>
+      <c r="E27" s="3">
         <v>0.36</v>
       </c>
-      <c r="E27" s="5">
+      <c r="F27" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F27" s="7" t="s">
+      <c r="G27" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="G27" s="8">
-        <v>0</v>
-      </c>
-      <c r="H27" s="9">
+      <c r="H27" s="8">
         <v>0</v>
       </c>
       <c r="I27" s="9">
+        <v>0</v>
+      </c>
+      <c r="J27" s="9">
         <v>300</v>
       </c>
-      <c r="J27" s="9"/>
       <c r="K27" s="9"/>
-    </row>
-    <row r="28" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L27" s="9"/>
+    </row>
+    <row r="28" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>24</v>
       </c>
       <c r="B28">
         <v>0.38</v>
       </c>
-      <c r="D28" s="3">
+      <c r="D28">
+        <v>17</v>
+      </c>
+      <c r="E28" s="3">
         <v>1.25</v>
       </c>
-      <c r="E28" s="6">
-        <v>0</v>
-      </c>
-      <c r="F28" s="7" t="s">
+      <c r="F28" s="6">
+        <v>0</v>
+      </c>
+      <c r="G28" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="G28" s="8">
-        <v>0</v>
-      </c>
-      <c r="H28" s="9">
+      <c r="H28" s="8">
         <v>0</v>
       </c>
       <c r="I28" s="9">
+        <v>0</v>
+      </c>
+      <c r="J28" s="9">
         <v>150</v>
       </c>
-      <c r="J28" s="9"/>
       <c r="K28" s="9"/>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L28" s="9"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>25</v>
       </c>
       <c r="B29">
         <v>0</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D29">
+        <v>88</v>
+      </c>
+      <c r="E29" s="3">
         <v>3.5</v>
       </c>
-      <c r="E29" s="5">
+      <c r="F29" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="G29" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G29" s="8">
+      <c r="H29" s="8">
         <v>1.23</v>
       </c>
-      <c r="H29" s="9">
-        <v>0</v>
-      </c>
       <c r="I29" s="9">
         <v>0</v>
       </c>
-      <c r="J29" s="9"/>
+      <c r="J29" s="9">
+        <v>0</v>
+      </c>
       <c r="K29" s="9"/>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L29" s="9"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>26</v>
       </c>
       <c r="B30">
         <v>0.08</v>
       </c>
-      <c r="D30" s="3">
+      <c r="D30">
+        <v>87</v>
+      </c>
+      <c r="E30" s="3">
         <v>3.6</v>
       </c>
-      <c r="E30" s="5">
+      <c r="F30" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F30" s="7" t="s">
+      <c r="G30" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G30" s="8">
+      <c r="H30" s="8">
         <v>1.23</v>
       </c>
-      <c r="H30" s="9">
-        <v>0</v>
-      </c>
       <c r="I30" s="9">
         <v>0</v>
       </c>
-      <c r="J30" s="9"/>
+      <c r="J30" s="9">
+        <v>0</v>
+      </c>
       <c r="K30" s="9"/>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L30" s="9"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>28</v>
       </c>
       <c r="B31">
         <v>0.08</v>
       </c>
-      <c r="D31" s="3">
+      <c r="D31">
+        <v>18</v>
+      </c>
+      <c r="E31" s="3">
         <v>0.5</v>
       </c>
-      <c r="E31" s="5">
+      <c r="F31" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F31" s="7" t="s">
+      <c r="G31" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G31" s="8">
+      <c r="H31" s="8">
         <v>1.23</v>
       </c>
-      <c r="H31" s="9">
-        <v>0</v>
-      </c>
       <c r="I31" s="9">
         <v>0</v>
       </c>
-      <c r="J31" s="9"/>
+      <c r="J31" s="9">
+        <v>0</v>
+      </c>
       <c r="K31" s="9"/>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L31" s="9"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>27</v>
       </c>
       <c r="B32">
         <v>0</v>
       </c>
-      <c r="D32" s="3">
+      <c r="D32">
+        <v>88</v>
+      </c>
+      <c r="E32" s="3">
         <v>3.6</v>
       </c>
-      <c r="E32" s="5">
+      <c r="F32" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F32" s="7" t="s">
+      <c r="G32" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G32" s="8">
+      <c r="H32" s="8">
         <v>1.23</v>
       </c>
-      <c r="H32" s="9">
-        <v>0</v>
-      </c>
       <c r="I32" s="9">
         <v>0</v>
       </c>
-      <c r="J32" s="9"/>
+      <c r="J32" s="9">
+        <v>0</v>
+      </c>
       <c r="K32" s="9"/>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L32" s="9"/>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>29</v>
       </c>
       <c r="B33">
         <v>0</v>
       </c>
-      <c r="D33" s="3">
+      <c r="D33">
+        <v>87.7</v>
+      </c>
+      <c r="E33" s="3">
         <v>1.5</v>
       </c>
-      <c r="E33" s="5">
+      <c r="F33" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F33" s="7" t="s">
+      <c r="G33" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G33" s="8">
+      <c r="H33" s="8">
         <v>1.23</v>
       </c>
-      <c r="H33" s="9">
-        <v>0</v>
-      </c>
       <c r="I33" s="9">
         <v>0</v>
       </c>
-      <c r="J33" s="9"/>
+      <c r="J33" s="9">
+        <v>0</v>
+      </c>
       <c r="K33" s="9"/>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L33" s="9"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>30</v>
       </c>
       <c r="B34">
         <v>0</v>
       </c>
-      <c r="D34" s="3">
+      <c r="D34">
+        <v>10.3</v>
+      </c>
+      <c r="E34" s="3">
         <v>0.5</v>
       </c>
-      <c r="E34" s="5">
+      <c r="F34" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F34" s="7" t="s">
+      <c r="G34" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G34" s="8">
+      <c r="H34" s="8">
         <v>1.23</v>
       </c>
-      <c r="H34" s="9">
-        <v>0</v>
-      </c>
       <c r="I34" s="9">
         <v>0</v>
       </c>
-      <c r="J34" s="9"/>
+      <c r="J34" s="9">
+        <v>0</v>
+      </c>
       <c r="K34" s="9"/>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="L34" s="9"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>31</v>
       </c>
       <c r="B35">
         <v>0</v>
       </c>
-      <c r="D35" s="3">
+      <c r="D35">
+        <v>90</v>
+      </c>
+      <c r="E35" s="3">
         <v>6</v>
       </c>
-      <c r="E35" s="5">
+      <c r="F35" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="F35" s="7" t="s">
+      <c r="G35" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="G35" s="8">
+      <c r="H35" s="8">
         <v>1.23</v>
       </c>
-      <c r="H35" s="9">
-        <v>0</v>
-      </c>
       <c r="I35" s="9">
         <v>0</v>
       </c>
-      <c r="J35" s="9"/>
+      <c r="J35" s="9">
+        <v>0</v>
+      </c>
       <c r="K35" s="9"/>
-    </row>
-    <row r="36" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L35" s="9"/>
+    </row>
+    <row r="36" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>32</v>
       </c>
       <c r="B36">
         <v>0</v>
       </c>
-      <c r="D36" s="3">
+      <c r="D36">
+        <v>17.7</v>
+      </c>
+      <c r="E36" s="3">
         <v>2.8</v>
       </c>
-      <c r="E36" s="5">
-        <v>0</v>
-      </c>
-      <c r="F36" s="7" t="s">
+      <c r="F36" s="5">
+        <v>0</v>
+      </c>
+      <c r="G36" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="G36" s="8">
+      <c r="H36" s="8">
         <v>1.47</v>
       </c>
-      <c r="H36" s="9">
-        <v>0</v>
-      </c>
       <c r="I36" s="9">
         <v>0</v>
       </c>
-      <c r="J36" s="9"/>
+      <c r="J36" s="9">
+        <v>0</v>
+      </c>
       <c r="K36" s="9"/>
-    </row>
-    <row r="37" spans="1:11" ht="25" x14ac:dyDescent="0.35">
+      <c r="L36" s="9"/>
+    </row>
+    <row r="37" spans="1:12" ht="25" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>39</v>
       </c>
       <c r="B37">
         <v>0.25</v>
       </c>
-      <c r="D37" s="3">
+      <c r="D37">
+        <v>86</v>
+      </c>
+      <c r="E37" s="3">
         <v>2.0499999999999998</v>
       </c>
-      <c r="E37" s="6">
-        <v>0</v>
-      </c>
-      <c r="F37" s="7" t="s">
+      <c r="F37" s="6">
+        <v>0</v>
+      </c>
+      <c r="G37" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="G37" s="8">
+      <c r="H37" s="8">
         <v>0.36749999999999999</v>
       </c>
-      <c r="H37" s="9">
-        <v>0</v>
-      </c>
       <c r="I37" s="9">
+        <v>0</v>
+      </c>
+      <c r="J37" s="9">
         <v>150</v>
       </c>
-      <c r="J37" s="9"/>
       <c r="K37" s="9"/>
+      <c r="L37" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1801,8 +2251,1485 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7EEDC770-986F-473C-8664-8C9A88803BEB}">
+  <dimension ref="A1:AI44"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1" t="s">
+        <v>110</v>
+      </c>
+      <c r="H1" t="s">
+        <v>111</v>
+      </c>
+      <c r="I1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K1" t="s">
+        <v>114</v>
+      </c>
+      <c r="L1" t="s">
+        <v>115</v>
+      </c>
+      <c r="M1" t="s">
+        <v>116</v>
+      </c>
+      <c r="N1" t="s">
+        <v>117</v>
+      </c>
+      <c r="O1" t="s">
+        <v>118</v>
+      </c>
+      <c r="P1" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>120</v>
+      </c>
+      <c r="R1" t="s">
+        <v>121</v>
+      </c>
+      <c r="S1" t="s">
+        <v>122</v>
+      </c>
+      <c r="T1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U1" t="s">
+        <v>124</v>
+      </c>
+      <c r="V1" t="s">
+        <v>125</v>
+      </c>
+      <c r="W1" t="s">
+        <v>126</v>
+      </c>
+      <c r="X1" t="s">
+        <v>127</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>128</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>129</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>131</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>132</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>133</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>134</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>136</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>137</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B2">
+        <v>877</v>
+      </c>
+      <c r="C2">
+        <v>169</v>
+      </c>
+      <c r="D2">
+        <v>116</v>
+      </c>
+      <c r="E2">
+        <v>1437</v>
+      </c>
+      <c r="F2">
+        <v>534</v>
+      </c>
+      <c r="G2">
+        <v>131</v>
+      </c>
+      <c r="H2">
+        <v>122</v>
+      </c>
+      <c r="I2">
+        <v>604</v>
+      </c>
+      <c r="J2">
+        <v>1561</v>
+      </c>
+      <c r="K2">
+        <v>213</v>
+      </c>
+      <c r="L2">
+        <v>742</v>
+      </c>
+      <c r="M2">
+        <v>315</v>
+      </c>
+      <c r="N2">
+        <v>846</v>
+      </c>
+      <c r="O2">
+        <v>316</v>
+      </c>
+      <c r="P2">
+        <v>859</v>
+      </c>
+      <c r="Q2">
+        <v>479</v>
+      </c>
+      <c r="R2">
+        <v>571</v>
+      </c>
+      <c r="S2">
+        <v>28</v>
+      </c>
+      <c r="T2">
+        <v>50</v>
+      </c>
+      <c r="U2">
+        <v>153</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>196</v>
+      </c>
+      <c r="X2">
+        <v>75</v>
+      </c>
+      <c r="Y2">
+        <v>338</v>
+      </c>
+      <c r="Z2">
+        <v>189</v>
+      </c>
+      <c r="AA2">
+        <v>401</v>
+      </c>
+      <c r="AB2">
+        <v>149</v>
+      </c>
+      <c r="AC2">
+        <v>71</v>
+      </c>
+      <c r="AD2">
+        <v>29</v>
+      </c>
+      <c r="AE2">
+        <v>0</v>
+      </c>
+      <c r="AF2">
+        <v>0</v>
+      </c>
+      <c r="AG2">
+        <v>12</v>
+      </c>
+      <c r="AH2">
+        <v>0</v>
+      </c>
+      <c r="AI2">
+        <f>SUM(B2:AH2)</f>
+        <v>11583</v>
+      </c>
+    </row>
+    <row r="11" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="12" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R12" s="10"/>
+    </row>
+    <row r="13" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R13" s="10"/>
+    </row>
+    <row r="14" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R14" s="10"/>
+    </row>
+    <row r="15" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R15" s="10"/>
+    </row>
+    <row r="16" spans="1:35" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R16" s="10"/>
+    </row>
+    <row r="17" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R17" s="11"/>
+    </row>
+    <row r="18" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R18" s="10"/>
+    </row>
+    <row r="19" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R19" s="10"/>
+    </row>
+    <row r="20" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R20" s="10"/>
+    </row>
+    <row r="21" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R21" s="10"/>
+    </row>
+    <row r="22" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R22" s="10"/>
+    </row>
+    <row r="23" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R23" s="10"/>
+    </row>
+    <row r="24" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R24" s="10"/>
+    </row>
+    <row r="25" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R25" s="11"/>
+    </row>
+    <row r="26" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R26" s="10"/>
+    </row>
+    <row r="27" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R27" s="10"/>
+    </row>
+    <row r="28" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R28" s="10"/>
+    </row>
+    <row r="29" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R29" s="10"/>
+    </row>
+    <row r="30" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R30" s="10"/>
+    </row>
+    <row r="31" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R31" s="11"/>
+    </row>
+    <row r="32" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R32" s="10"/>
+    </row>
+    <row r="33" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R33" s="10"/>
+    </row>
+    <row r="34" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R34" s="10"/>
+    </row>
+    <row r="35" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R35" s="10"/>
+    </row>
+    <row r="36" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R36" s="10"/>
+    </row>
+    <row r="37" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R37" s="10"/>
+    </row>
+    <row r="38" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R38" s="10"/>
+    </row>
+    <row r="39" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R39" s="10"/>
+    </row>
+    <row r="40" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R40" s="11"/>
+    </row>
+    <row r="41" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R41" s="10"/>
+    </row>
+    <row r="42" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R42" s="10"/>
+    </row>
+    <row r="43" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R43" s="10"/>
+    </row>
+    <row r="44" spans="18:18" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="R44" s="10"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0C8FA35-4843-4FEC-9720-CB1F6CC19C35}">
+  <dimension ref="A1:E29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="7" max="7" width="17.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B2">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>162</v>
+      </c>
+      <c r="D2" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B3">
+        <v>2.5026398888888901E-3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>162</v>
+      </c>
+      <c r="D3" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B4">
+        <v>2.5191576000000004E-3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>162</v>
+      </c>
+      <c r="D4" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>150</v>
+      </c>
+      <c r="B5">
+        <v>3.4014885333333339E-3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>162</v>
+      </c>
+      <c r="D5" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>151</v>
+      </c>
+      <c r="B6">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>162</v>
+      </c>
+      <c r="D6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>152</v>
+      </c>
+      <c r="B7">
+        <v>5.5000000000000003E-4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>162</v>
+      </c>
+      <c r="D7" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>153</v>
+      </c>
+      <c r="B8">
+        <v>5.5731720329999998E-4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>162</v>
+      </c>
+      <c r="D8" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9">
+        <v>2.8934473500000003E-3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>162</v>
+      </c>
+      <c r="D9" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10">
+        <v>2.5331492083333334E-3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>162</v>
+      </c>
+      <c r="D10" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>178</v>
+      </c>
+      <c r="B11">
+        <v>2.5165149883414934E-3</v>
+      </c>
+      <c r="C11" t="s">
+        <v>162</v>
+      </c>
+      <c r="D11" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>177</v>
+      </c>
+      <c r="B12">
+        <v>2.44344375E-3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>162</v>
+      </c>
+      <c r="D12" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>154</v>
+      </c>
+      <c r="B13">
+        <v>2.2090262539682538E-3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>162</v>
+      </c>
+      <c r="D13" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>155</v>
+      </c>
+      <c r="B14">
+        <v>5.8E-4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>163</v>
+      </c>
+      <c r="D14" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>156</v>
+      </c>
+      <c r="B15">
+        <v>5.5000000000000003E-4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>163</v>
+      </c>
+      <c r="D15" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>157</v>
+      </c>
+      <c r="B16">
+        <v>4.4999999999999999E-4</v>
+      </c>
+      <c r="C16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D16" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>158</v>
+      </c>
+      <c r="B17">
+        <v>7.5000000000000002E-4</v>
+      </c>
+      <c r="C17" t="s">
+        <v>163</v>
+      </c>
+      <c r="D17" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>159</v>
+      </c>
+      <c r="B18">
+        <v>2.0631828E-4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>163</v>
+      </c>
+      <c r="D18" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>160</v>
+      </c>
+      <c r="B19">
+        <v>5.4262139775921735E-4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>163</v>
+      </c>
+      <c r="D19" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>147</v>
+      </c>
+      <c r="B20">
+        <v>2.3440000000000003E-4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>163</v>
+      </c>
+      <c r="D20" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>145</v>
+      </c>
+      <c r="B21">
+        <v>2.9231999999999999E-4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>163</v>
+      </c>
+      <c r="D21" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>146</v>
+      </c>
+      <c r="B22">
+        <v>1.5964523839999997E-3</v>
+      </c>
+      <c r="C22" t="s">
+        <v>163</v>
+      </c>
+      <c r="D22" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>169</v>
+      </c>
+      <c r="B23">
+        <v>1.8285932799999999E-3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>163</v>
+      </c>
+      <c r="D23" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>170</v>
+      </c>
+      <c r="B24">
+        <v>3.6662312908139748E-4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>163</v>
+      </c>
+      <c r="D24" t="s">
+        <v>167</v>
+      </c>
+      <c r="E24" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>171</v>
+      </c>
+      <c r="B25">
+        <v>3.6662312908139748E-4</v>
+      </c>
+      <c r="C25" t="s">
+        <v>163</v>
+      </c>
+      <c r="D25" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>172</v>
+      </c>
+      <c r="B26">
+        <v>1.1635199999999999E-3</v>
+      </c>
+      <c r="C26" t="s">
+        <v>163</v>
+      </c>
+      <c r="D26" t="s">
+        <v>167</v>
+      </c>
+      <c r="E26" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>173</v>
+      </c>
+      <c r="B27">
+        <v>1.1635199999999999E-3</v>
+      </c>
+      <c r="C27" t="s">
+        <v>163</v>
+      </c>
+      <c r="D27" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>175</v>
+      </c>
+      <c r="B28">
+        <v>5.7248880000000007E-4</v>
+      </c>
+      <c r="C28" t="s">
+        <v>163</v>
+      </c>
+      <c r="D28" t="s">
+        <v>167</v>
+      </c>
+      <c r="E28" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>176</v>
+      </c>
+      <c r="B29">
+        <v>5.7248880000000007E-4</v>
+      </c>
+      <c r="C29" t="s">
+        <v>163</v>
+      </c>
+      <c r="D29" t="s">
+        <v>167</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3D8FFD4-4EA9-47C1-BA4E-47263EF1D3B0}">
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="25.08984375" customWidth="1"/>
+    <col min="2" max="2" width="29.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.90625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B1" t="s">
+        <v>182</v>
+      </c>
+      <c r="C1" t="s">
+        <v>89</v>
+      </c>
+      <c r="D1" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>185</v>
+      </c>
+      <c r="B2">
+        <v>6.7174054999999996E-4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>186</v>
+      </c>
+      <c r="B3">
+        <v>5.0052599999999992E-3</v>
+      </c>
+      <c r="C3" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B4">
+        <v>5.0052599999999992E-3</v>
+      </c>
+      <c r="C4" t="s">
+        <v>166</v>
+      </c>
+      <c r="D4" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>188</v>
+      </c>
+      <c r="B5">
+        <v>4.3945200000000007E-3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>189</v>
+      </c>
+      <c r="B6">
+        <v>1.1705850000000001E-4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>202</v>
+      </c>
+      <c r="B7">
+        <v>6.7174054999999996E-4</v>
+      </c>
+      <c r="C7" t="s">
+        <v>166</v>
+      </c>
+      <c r="D7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>194</v>
+      </c>
+      <c r="B8">
+        <v>2.0631828E-4</v>
+      </c>
+      <c r="C8" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>193</v>
+      </c>
+      <c r="B9">
+        <v>5.4262139775921735E-4</v>
+      </c>
+      <c r="C9" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>192</v>
+      </c>
+      <c r="B10">
+        <v>2.3440000000000003E-4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>195</v>
+      </c>
+      <c r="B11">
+        <v>2.9231999999999999E-4</v>
+      </c>
+      <c r="C11" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>196</v>
+      </c>
+      <c r="B12">
+        <v>1.5964523839999997E-3</v>
+      </c>
+      <c r="C12" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>197</v>
+      </c>
+      <c r="B13">
+        <v>1.8285932799999999E-3</v>
+      </c>
+      <c r="C13" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>198</v>
+      </c>
+      <c r="B14">
+        <v>3.6662312908139748E-4</v>
+      </c>
+      <c r="C14" t="s">
+        <v>167</v>
+      </c>
+      <c r="D14" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>199</v>
+      </c>
+      <c r="B15">
+        <v>3.6662312908139748E-4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>203</v>
+      </c>
+      <c r="B16">
+        <v>1.1635199999999999E-3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>167</v>
+      </c>
+      <c r="D16" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>204</v>
+      </c>
+      <c r="B17">
+        <v>1.1635199999999999E-3</v>
+      </c>
+      <c r="C17" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>200</v>
+      </c>
+      <c r="B18">
+        <v>5.7248880000000007E-4</v>
+      </c>
+      <c r="C18" t="s">
+        <v>167</v>
+      </c>
+      <c r="D18" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>201</v>
+      </c>
+      <c r="B19">
+        <v>5.7248880000000007E-4</v>
+      </c>
+      <c r="C19" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20">
+        <v>1.9282590170888892E-3</v>
+      </c>
+      <c r="C20" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21">
+        <v>7.789160266200002E-4</v>
+      </c>
+      <c r="C21" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>153</v>
+      </c>
+      <c r="B22">
+        <v>5.5731720329999998E-4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>32</v>
+      </c>
+      <c r="B23">
+        <v>2.5331492083333334E-3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>178</v>
+      </c>
+      <c r="B24">
+        <v>2.5165149883414934E-3</v>
+      </c>
+      <c r="C24" t="s">
+        <v>164</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDCA4DCB-FE4A-48BA-AD0E-D81C83744525}">
+  <dimension ref="A1:B10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="16.453125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>164</v>
+      </c>
+      <c r="B3">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>153</v>
+      </c>
+      <c r="B4">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>165</v>
+      </c>
+      <c r="B5">
+        <v>0.09</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>156</v>
+      </c>
+      <c r="B7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>157</v>
+      </c>
+      <c r="B8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>158</v>
+      </c>
+      <c r="B9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B10">
+        <v>0.79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B24DCEF-E7C2-4526-9D13-3C67B63444AD}">
+  <dimension ref="A1:AI3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>104</v>
+      </c>
+      <c r="B1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1" t="s">
+        <v>110</v>
+      </c>
+      <c r="H1" t="s">
+        <v>111</v>
+      </c>
+      <c r="I1" t="s">
+        <v>112</v>
+      </c>
+      <c r="J1" t="s">
+        <v>113</v>
+      </c>
+      <c r="K1" t="s">
+        <v>114</v>
+      </c>
+      <c r="L1" t="s">
+        <v>115</v>
+      </c>
+      <c r="M1" t="s">
+        <v>116</v>
+      </c>
+      <c r="N1" t="s">
+        <v>117</v>
+      </c>
+      <c r="O1" t="s">
+        <v>118</v>
+      </c>
+      <c r="P1" t="s">
+        <v>119</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>120</v>
+      </c>
+      <c r="R1" t="s">
+        <v>121</v>
+      </c>
+      <c r="S1" t="s">
+        <v>122</v>
+      </c>
+      <c r="T1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U1" t="s">
+        <v>124</v>
+      </c>
+      <c r="V1" t="s">
+        <v>125</v>
+      </c>
+      <c r="W1" t="s">
+        <v>126</v>
+      </c>
+      <c r="X1" t="s">
+        <v>127</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>128</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>129</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>130</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>131</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>132</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>133</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>134</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>136</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>137</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B2">
+        <v>92.113959999999992</v>
+      </c>
+      <c r="C2">
+        <v>9.3678999999999988</v>
+      </c>
+      <c r="D2">
+        <v>7.9292200000000008</v>
+      </c>
+      <c r="E2">
+        <v>32.702010000000001</v>
+      </c>
+      <c r="F2">
+        <v>28.21088000000001</v>
+      </c>
+      <c r="G2">
+        <v>97.652479999999954</v>
+      </c>
+      <c r="H2">
+        <v>15.820459999999995</v>
+      </c>
+      <c r="I2">
+        <v>66.401299999999992</v>
+      </c>
+      <c r="J2">
+        <v>35.252930000000006</v>
+      </c>
+      <c r="K2">
+        <v>14.638589999999997</v>
+      </c>
+      <c r="L2">
+        <v>44.824680000000001</v>
+      </c>
+      <c r="M2">
+        <v>31.32692999999999</v>
+      </c>
+      <c r="N2">
+        <v>160.72521</v>
+      </c>
+      <c r="O2">
+        <v>43.248719999999992</v>
+      </c>
+      <c r="P2">
+        <v>206.58865999999998</v>
+      </c>
+      <c r="Q2">
+        <v>32.781079999999989</v>
+      </c>
+      <c r="R2">
+        <v>58.299580000000006</v>
+      </c>
+      <c r="S2">
+        <v>8.6474600000000006</v>
+      </c>
+      <c r="T2">
+        <v>7.5009900000000016</v>
+      </c>
+      <c r="U2">
+        <v>24.510950000000001</v>
+      </c>
+      <c r="V2">
+        <v>1.1988499999999997</v>
+      </c>
+      <c r="W2">
+        <v>17.228110000000004</v>
+      </c>
+      <c r="X2">
+        <v>10.933770000000001</v>
+      </c>
+      <c r="Y2">
+        <v>27.44576</v>
+      </c>
+      <c r="Z2">
+        <v>48.051410000000011</v>
+      </c>
+      <c r="AA2">
+        <v>13.837059999999997</v>
+      </c>
+      <c r="AB2">
+        <v>10.718019999999999</v>
+      </c>
+      <c r="AC2">
+        <v>11.926820000000003</v>
+      </c>
+      <c r="AD2">
+        <v>12.789459999999996</v>
+      </c>
+      <c r="AE2">
+        <v>27.769340000000007</v>
+      </c>
+      <c r="AF2">
+        <v>5.3662799999999971</v>
+      </c>
+      <c r="AG2">
+        <v>11.832720000000002</v>
+      </c>
+      <c r="AH2">
+        <v>4.6259899999999998</v>
+      </c>
+      <c r="AI2">
+        <v>437.8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:35" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>139</v>
+      </c>
+      <c r="B3">
+        <v>58.260291000000002</v>
+      </c>
+      <c r="C3">
+        <v>43.361862000000002</v>
+      </c>
+      <c r="D3">
+        <v>30.468439999999994</v>
+      </c>
+      <c r="E3">
+        <v>91.869658000000001</v>
+      </c>
+      <c r="F3">
+        <v>23.830795000000002</v>
+      </c>
+      <c r="G3">
+        <v>125.05385200000001</v>
+      </c>
+      <c r="H3">
+        <v>7.2032819999999997</v>
+      </c>
+      <c r="I3">
+        <v>93.045423999999997</v>
+      </c>
+      <c r="J3">
+        <v>90.388374000000013</v>
+      </c>
+      <c r="K3">
+        <v>32.028894000000015</v>
+      </c>
+      <c r="L3">
+        <v>61.268584499999996</v>
+      </c>
+      <c r="M3">
+        <v>43.307626499999998</v>
+      </c>
+      <c r="N3">
+        <v>48.774823999999995</v>
+      </c>
+      <c r="O3">
+        <v>45.255763000000016</v>
+      </c>
+      <c r="P3">
+        <v>79.412431000000012</v>
+      </c>
+      <c r="Q3">
+        <v>93.641458999999998</v>
+      </c>
+      <c r="R3">
+        <v>47.56297</v>
+      </c>
+      <c r="S3">
+        <v>13.527467</v>
+      </c>
+      <c r="T3">
+        <v>4.7963090000000008</v>
+      </c>
+      <c r="U3">
+        <v>22.102628000000003</v>
+      </c>
+      <c r="V3">
+        <v>2.5489359999999999</v>
+      </c>
+      <c r="W3">
+        <v>19.579385000000002</v>
+      </c>
+      <c r="X3">
+        <v>3.6610950000000004</v>
+      </c>
+      <c r="Y3">
+        <v>59.672404000000043</v>
+      </c>
+      <c r="Z3">
+        <v>30.027981</v>
+      </c>
+      <c r="AA3">
+        <v>27.866744999999998</v>
+      </c>
+      <c r="AB3">
+        <v>20.721993000000001</v>
+      </c>
+      <c r="AC3">
+        <v>4.8341580000000004</v>
+      </c>
+      <c r="AD3">
+        <v>3.4297689999999998</v>
+      </c>
+      <c r="AE3">
+        <v>23.448231999999997</v>
+      </c>
+      <c r="AF3">
+        <v>1.181686</v>
+      </c>
+      <c r="AG3">
+        <v>24.802152999999997</v>
+      </c>
+      <c r="AH3">
+        <v>6.1657950000000001</v>
+      </c>
+      <c r="AI3">
+        <v>498.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E12223D9-0A39-4CC4-B45B-34CE66BF62BA}">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:O7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="22.36328125" customWidth="1"/>
@@ -1815,7 +3742,7 @@
     <col min="9" max="9" width="18.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>40</v>
       </c>
@@ -1855,8 +3782,14 @@
       <c r="M1" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N1" t="s">
+        <v>183</v>
+      </c>
+      <c r="O1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -1899,8 +3832,14 @@
       <c r="M2">
         <v>5.3E-3</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N2">
+        <v>0.49</v>
+      </c>
+      <c r="O2">
+        <v>0.38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -1943,8 +3882,14 @@
       <c r="M3">
         <v>9.4000000000000004E-3</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N3">
+        <v>0.7</v>
+      </c>
+      <c r="O3">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -1987,8 +3932,14 @@
       <c r="M4">
         <v>9.4000000000000004E-3</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N4">
+        <v>1.96</v>
+      </c>
+      <c r="O4">
+        <v>0.78</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -2031,8 +3982,14 @@
       <c r="M5">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N5">
+        <v>0.9</v>
+      </c>
+      <c r="O5">
+        <v>0.57999999999999996</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>45</v>
       </c>
@@ -2075,8 +4032,14 @@
       <c r="M6">
         <v>1.7899999999999999E-2</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="N6">
+        <v>3.95</v>
+      </c>
+      <c r="O6">
+        <v>3.68</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -2118,6 +4081,12 @@
       </c>
       <c r="M7">
         <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0.41</v>
+      </c>
+      <c r="O7">
+        <v>0.41</v>
       </c>
     </row>
   </sheetData>
@@ -2126,7 +4095,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D061B11-9C82-42EB-AFA7-28C01EBEFD7E}">
   <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>

<commit_message>
Transfert des données de carbone dans GRAFS_data.xslx
</commit_message>
<xml_diff>
--- a/src/grafs_e/data/GRAFS_data.xlsx
+++ b/src/grafs_e/data/GRAFS_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\faustega\Documents\These\isterre-dynamic-modeling\grafs-e-project\grafs-e\src\grafs_e\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4A4C28D-35CC-4E52-91E2-E4EC4192805F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBDA835C-E4AC-4C1C-ADE9-84D33511F05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15165" yWindow="-16680" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
+    <workbookView xWindow="15195" yWindow="-16065" windowWidth="25440" windowHeight="15390" activeTab="3" xr2:uid="{092E5AC7-17CB-4282-9989-CDCB089F75B9}"/>
   </bookViews>
   <sheets>
     <sheet name="crops" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="210">
   <si>
     <t>Culture</t>
   </si>
@@ -55,15 +55,9 @@
     <t>Oat</t>
   </si>
   <si>
-    <t>Grain maize</t>
-  </si>
-  <si>
     <t>Other cereals</t>
   </si>
   <si>
-    <t>Straw</t>
-  </si>
-  <si>
     <t>Rapeseed</t>
   </si>
   <si>
@@ -145,9 +139,6 @@
     <t>Note</t>
   </si>
   <si>
-    <t>Proche de blé…</t>
-  </si>
-  <si>
     <t>Entre beteraves et PDT</t>
   </si>
   <si>
@@ -592,12 +583,6 @@
     <t>Methanization power (GWh/tMB)</t>
   </si>
   <si>
-    <t>Manure nitrogen Content (%)</t>
-  </si>
-  <si>
-    <t>Slurry nitrogen Content (%)</t>
-  </si>
-  <si>
     <t>bovines waste</t>
   </si>
   <si>
@@ -656,13 +641,43 @@
   </si>
   <si>
     <t>equine manure</t>
+  </si>
+  <si>
+    <t>Carbon allocation to grain (%)</t>
+  </si>
+  <si>
+    <t>Carbon allocation to straw (%)</t>
+  </si>
+  <si>
+    <t>Maize</t>
+  </si>
+  <si>
+    <t>Wheat straw</t>
+  </si>
+  <si>
+    <t>Rye straw</t>
+  </si>
+  <si>
+    <t>Barley straw</t>
+  </si>
+  <si>
+    <t>Oat straw</t>
+  </si>
+  <si>
+    <t>Other cereals straw</t>
+  </si>
+  <si>
+    <t>Manure nitrogen Content (% N/MB)</t>
+  </si>
+  <si>
+    <t>Slurry nitrogen Content (% N/MB)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -696,6 +711,12 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -736,7 +757,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -760,6 +781,12 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1076,48 +1103,58 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{973E28D2-5D19-4409-920F-79B00DDA2ABC}">
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.7265625" customWidth="1"/>
     <col min="2" max="2" width="18.1796875" customWidth="1"/>
     <col min="5" max="5" width="19.6328125" customWidth="1"/>
     <col min="6" max="6" width="14.90625" customWidth="1"/>
+    <col min="8" max="8" width="22.7265625" customWidth="1"/>
+    <col min="9" max="9" width="19.7265625" customWidth="1"/>
+    <col min="10" max="10" width="23" customWidth="1"/>
+    <col min="11" max="11" width="25.90625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="F1" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="H1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="I1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="J1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
+        <v>95</v>
+      </c>
+      <c r="K1" t="s">
+        <v>200</v>
+      </c>
+      <c r="L1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1125,7 +1162,7 @@
         <v>0.12</v>
       </c>
       <c r="C2" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D2">
         <v>86.9</v>
@@ -1137,7 +1174,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H2" s="8">
         <v>0</v>
@@ -1148,12 +1185,17 @@
       <c r="J2" s="9">
         <v>0</v>
       </c>
-      <c r="K2" s="9"/>
-      <c r="L2" s="9"/>
-    </row>
-    <row r="3" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="K2" s="13">
+        <v>40.200000000000003</v>
+      </c>
+      <c r="L2" s="9">
+        <v>41.827100000000002</v>
+      </c>
+      <c r="N2" s="12"/>
+    </row>
+    <row r="3" spans="1:14" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B3">
         <v>0.03</v>
@@ -1168,7 +1210,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H3" s="8">
         <v>0</v>
@@ -1179,10 +1221,15 @@
       <c r="J3" s="9">
         <v>0</v>
       </c>
-      <c r="K3" s="9"/>
-      <c r="L3" s="9"/>
-    </row>
-    <row r="4" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="K3" s="9">
+        <v>40.200000000000003</v>
+      </c>
+      <c r="L3" s="9">
+        <v>41.827100000000002</v>
+      </c>
+      <c r="N3" s="12"/>
+    </row>
+    <row r="4" spans="1:14" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1199,7 +1246,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H4" s="8">
         <v>0</v>
@@ -1210,10 +1257,15 @@
       <c r="J4" s="9">
         <v>0</v>
       </c>
-      <c r="K4" s="9"/>
-      <c r="L4" s="9"/>
-    </row>
-    <row r="5" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="K4" s="9">
+        <v>44</v>
+      </c>
+      <c r="L4" s="9">
+        <v>42.311399999999999</v>
+      </c>
+      <c r="N4" s="12"/>
+    </row>
+    <row r="5" spans="1:14" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1230,7 +1282,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H5" s="8">
         <v>0</v>
@@ -1241,12 +1293,17 @@
       <c r="J5" s="9">
         <v>0</v>
       </c>
-      <c r="K5" s="9"/>
-      <c r="L5" s="9"/>
-    </row>
-    <row r="6" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="K5" s="9">
+        <v>33.1</v>
+      </c>
+      <c r="L5" s="9">
+        <v>29.4</v>
+      </c>
+      <c r="N5" s="12"/>
+    </row>
+    <row r="6" spans="1:14" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>4</v>
+        <v>202</v>
       </c>
       <c r="B6">
         <v>0.4</v>
@@ -1261,7 +1318,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H6" s="8">
         <v>0</v>
@@ -1272,12 +1329,17 @@
       <c r="J6" s="9">
         <v>0</v>
       </c>
-      <c r="K6" s="9"/>
-      <c r="L6" s="9"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K6" s="9">
+        <v>42.6</v>
+      </c>
+      <c r="L6" s="9">
+        <v>36.299999999999997</v>
+      </c>
+      <c r="N6" s="12"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B7">
         <v>0.03</v>
@@ -1292,7 +1354,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="H7" s="8">
         <v>0</v>
@@ -1303,12 +1365,17 @@
       <c r="J7" s="9">
         <v>125</v>
       </c>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-    </row>
-    <row r="8" spans="1:12" ht="37.5" x14ac:dyDescent="0.35">
+      <c r="K7" s="9">
+        <v>39.6</v>
+      </c>
+      <c r="L7" s="9">
+        <v>40.5794</v>
+      </c>
+      <c r="N7" s="12"/>
+    </row>
+    <row r="8" spans="1:14" ht="37.5" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8">
         <v>0.03</v>
@@ -1323,7 +1390,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="H8" s="8">
         <v>0</v>
@@ -1334,154 +1401,176 @@
       <c r="J8" s="9">
         <v>0</v>
       </c>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K8" s="9">
+        <v>39.6</v>
+      </c>
+      <c r="L8" s="9">
+        <v>40.5794</v>
+      </c>
+      <c r="N8" s="12"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9">
+        <v>0.33</v>
+      </c>
+      <c r="D9">
+        <v>92.4</v>
+      </c>
+      <c r="E9" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="F9" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="H9" s="8">
+        <v>0</v>
+      </c>
+      <c r="I9" s="3">
+        <v>7</v>
+      </c>
+      <c r="J9" s="9">
+        <v>0</v>
+      </c>
+      <c r="K9" s="9">
+        <v>16.3</v>
+      </c>
+      <c r="L9" s="9">
+        <v>60.234400000000001</v>
+      </c>
+      <c r="N9" s="12"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
         <v>6</v>
       </c>
-      <c r="B9">
-        <v>0.1</v>
-      </c>
-      <c r="C9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D9">
-        <v>90.3</v>
-      </c>
-      <c r="E9" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="F9" s="5">
-        <v>0</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="H9" s="8">
-        <v>0</v>
-      </c>
-      <c r="I9" s="3">
-        <v>3</v>
-      </c>
-      <c r="J9" s="9">
-        <v>0</v>
-      </c>
-      <c r="K9" s="9"/>
-      <c r="L9" s="9"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>7</v>
-      </c>
       <c r="B10">
-        <v>0.33</v>
+        <v>0.16</v>
       </c>
       <c r="D10">
-        <v>92.4</v>
+        <v>92.8</v>
       </c>
       <c r="E10" s="3">
-        <v>3.5</v>
+        <v>1.96</v>
       </c>
       <c r="F10" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="H10" s="8">
         <v>0</v>
       </c>
       <c r="I10" s="3">
+        <v>4.5</v>
+      </c>
+      <c r="J10" s="9">
+        <v>0</v>
+      </c>
+      <c r="K10" s="9">
+        <v>26</v>
+      </c>
+      <c r="L10" s="9">
+        <v>53.067</v>
+      </c>
+      <c r="N10" s="12"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
         <v>7</v>
       </c>
-      <c r="J10" s="9">
-        <v>0</v>
-      </c>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>8</v>
-      </c>
       <c r="B11">
-        <v>0.16</v>
+        <v>0</v>
       </c>
       <c r="D11">
-        <v>92.8</v>
-      </c>
-      <c r="E11" s="3">
-        <v>1.96</v>
+        <v>88.1</v>
+      </c>
+      <c r="E11" s="4">
+        <v>3.5</v>
       </c>
       <c r="F11" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="H11" s="8">
         <v>0</v>
       </c>
-      <c r="I11" s="3">
-        <v>4.5</v>
+      <c r="I11" s="9">
+        <v>5</v>
       </c>
       <c r="J11" s="9">
         <v>0</v>
       </c>
-      <c r="K11" s="9"/>
-      <c r="L11" s="9"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K11" s="9">
+        <v>25.2</v>
+      </c>
+      <c r="L11" s="9">
+        <v>52.439</v>
+      </c>
+      <c r="N11" s="12"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="D12">
+        <v>17.8</v>
+      </c>
+      <c r="E12" s="3">
+        <v>0.20799999999999999</v>
+      </c>
+      <c r="F12" s="5">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="H12" s="8">
+        <v>0</v>
+      </c>
+      <c r="I12" s="9">
+        <v>0</v>
+      </c>
+      <c r="J12" s="9">
+        <v>220</v>
+      </c>
+      <c r="K12" s="9">
+        <v>22.5</v>
+      </c>
+      <c r="L12" s="9">
+        <v>55.246799999999993</v>
+      </c>
+      <c r="N12" s="12"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
         <v>9</v>
       </c>
-      <c r="B12">
-        <v>0</v>
-      </c>
-      <c r="D12">
-        <v>88.1</v>
-      </c>
-      <c r="E12" s="4">
-        <v>3.5</v>
-      </c>
-      <c r="F12" s="5">
-        <v>2.7E-2</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>92</v>
-      </c>
-      <c r="H12" s="8">
-        <v>0</v>
-      </c>
-      <c r="I12" s="9">
-        <v>5</v>
-      </c>
-      <c r="J12" s="9">
-        <v>0</v>
-      </c>
-      <c r="K12" s="9"/>
-      <c r="L12" s="9"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>10</v>
-      </c>
       <c r="B13">
-        <v>0.56000000000000005</v>
+        <v>0.35</v>
       </c>
       <c r="D13">
-        <v>17.8</v>
+        <v>18.899999999999999</v>
       </c>
       <c r="E13" s="3">
-        <v>0.20799999999999999</v>
+        <v>0.25600000000000001</v>
       </c>
       <c r="F13" s="5">
         <v>5.6000000000000001E-2</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H13" s="8">
         <v>0</v>
@@ -1492,27 +1581,35 @@
       <c r="J13" s="9">
         <v>220</v>
       </c>
-      <c r="K13" s="9"/>
-      <c r="L13" s="9"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K13" s="9">
+        <v>38.6</v>
+      </c>
+      <c r="L13" s="9">
+        <v>34.144300000000001</v>
+      </c>
+      <c r="N13" s="12"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B14">
-        <v>0.35</v>
+        <v>0.45</v>
+      </c>
+      <c r="C14" t="s">
+        <v>32</v>
       </c>
       <c r="D14">
-        <v>18.899999999999999</v>
+        <v>17.8</v>
       </c>
       <c r="E14" s="3">
-        <v>0.25600000000000001</v>
+        <v>0.23</v>
       </c>
       <c r="F14" s="5">
         <v>5.6000000000000001E-2</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="H14" s="8">
         <v>0</v>
@@ -1523,64 +1620,71 @@
       <c r="J14" s="9">
         <v>220</v>
       </c>
-      <c r="K14" s="9"/>
-      <c r="L14" s="9"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K14" s="9">
+        <v>45.1</v>
+      </c>
+      <c r="L14" s="9">
+        <v>33.935500000000005</v>
+      </c>
+      <c r="N14" s="12"/>
+    </row>
+    <row r="15" spans="1:14" ht="25" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15">
+        <v>0</v>
+      </c>
+      <c r="C15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15">
+        <v>88.4</v>
+      </c>
+      <c r="E15" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="F15" s="5">
+        <v>2.7E-2</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="H15" s="8">
+        <v>0</v>
+      </c>
+      <c r="I15" s="9">
+        <v>0</v>
+      </c>
+      <c r="J15" s="9">
+        <v>50</v>
+      </c>
+      <c r="K15" s="9">
+        <v>41.9</v>
+      </c>
+      <c r="L15" s="9">
+        <v>34.039900000000003</v>
+      </c>
+      <c r="N15" s="12"/>
+    </row>
+    <row r="16" spans="1:14" ht="25" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
         <v>12</v>
       </c>
-      <c r="B15">
-        <v>0.45</v>
-      </c>
-      <c r="C15" t="s">
-        <v>35</v>
-      </c>
-      <c r="D15">
-        <v>17.8</v>
-      </c>
-      <c r="E15" s="3">
-        <v>0.23</v>
-      </c>
-      <c r="F15" s="5">
-        <v>5.6000000000000001E-2</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="H15" s="8">
-        <v>0</v>
-      </c>
-      <c r="I15" s="9">
-        <v>0</v>
-      </c>
-      <c r="J15" s="9">
-        <v>220</v>
-      </c>
-      <c r="K15" s="9"/>
-      <c r="L15" s="9"/>
-    </row>
-    <row r="16" spans="1:12" ht="25" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>13</v>
-      </c>
       <c r="B16">
         <v>0</v>
       </c>
-      <c r="C16" t="s">
-        <v>36</v>
-      </c>
       <c r="D16">
-        <v>88.4</v>
+        <v>80</v>
       </c>
       <c r="E16" s="3">
-        <v>3.6</v>
+        <v>2</v>
       </c>
       <c r="F16" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H16" s="8">
         <v>0</v>
@@ -1589,29 +1693,34 @@
         <v>0</v>
       </c>
       <c r="J16" s="9">
-        <v>50</v>
-      </c>
-      <c r="K16" s="9"/>
-      <c r="L16" s="9"/>
-    </row>
-    <row r="17" spans="1:12" ht="25" x14ac:dyDescent="0.35">
+        <v>100</v>
+      </c>
+      <c r="K16" s="9">
+        <v>59.099999999999994</v>
+      </c>
+      <c r="L16" s="9">
+        <v>15.103900000000001</v>
+      </c>
+      <c r="N16" s="12"/>
+    </row>
+    <row r="17" spans="1:14" ht="25" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="B17">
         <v>0</v>
       </c>
       <c r="D17">
-        <v>80</v>
+        <v>9.8000000000000007</v>
       </c>
       <c r="E17" s="3">
-        <v>2</v>
+        <v>0.18</v>
       </c>
       <c r="F17" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H17" s="8">
         <v>0</v>
@@ -1620,29 +1729,34 @@
         <v>0</v>
       </c>
       <c r="J17" s="9">
-        <v>100</v>
-      </c>
-      <c r="K17" s="9"/>
-      <c r="L17" s="9"/>
-    </row>
-    <row r="18" spans="1:12" ht="25" x14ac:dyDescent="0.35">
+        <v>180</v>
+      </c>
+      <c r="K17" s="9">
+        <v>82.699999999999989</v>
+      </c>
+      <c r="L17" s="9">
+        <v>15.0284</v>
+      </c>
+      <c r="N17" s="12"/>
+    </row>
+    <row r="18" spans="1:14" ht="25" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="B18">
         <v>0</v>
       </c>
       <c r="D18">
-        <v>9.8000000000000007</v>
+        <v>8.1</v>
       </c>
       <c r="E18" s="3">
-        <v>0.18</v>
+        <v>0.36</v>
       </c>
       <c r="F18" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H18" s="8">
         <v>0</v>
@@ -1651,29 +1765,34 @@
         <v>0</v>
       </c>
       <c r="J18" s="9">
-        <v>180</v>
-      </c>
-      <c r="K18" s="9"/>
-      <c r="L18" s="9"/>
-    </row>
-    <row r="19" spans="1:12" ht="25" x14ac:dyDescent="0.35">
+        <v>300</v>
+      </c>
+      <c r="K18" s="9">
+        <v>67</v>
+      </c>
+      <c r="L18" s="9">
+        <v>15.078700000000001</v>
+      </c>
+      <c r="N18" s="12"/>
+    </row>
+    <row r="19" spans="1:14" ht="25" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B19">
         <v>0</v>
       </c>
       <c r="D19">
-        <v>8.1</v>
+        <v>4.5</v>
       </c>
       <c r="E19" s="3">
-        <v>0.36</v>
+        <v>0.22</v>
       </c>
       <c r="F19" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="H19" s="8">
         <v>0</v>
@@ -1682,144 +1801,169 @@
         <v>0</v>
       </c>
       <c r="J19" s="9">
-        <v>300</v>
-      </c>
-      <c r="K19" s="9"/>
-      <c r="L19" s="9"/>
-    </row>
-    <row r="20" spans="1:12" ht="25" x14ac:dyDescent="0.35">
+        <v>150</v>
+      </c>
+      <c r="K19" s="9">
+        <v>41.9</v>
+      </c>
+      <c r="L19" s="9">
+        <v>34.039900000000003</v>
+      </c>
+      <c r="N19" s="12"/>
+    </row>
+    <row r="20" spans="1:14" ht="25" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>16.399999999999999</v>
+      </c>
+      <c r="E20" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="F20" s="5">
+        <v>0</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="H20" s="8">
+        <v>0</v>
+      </c>
+      <c r="I20" s="9">
+        <v>0</v>
+      </c>
+      <c r="J20" s="9">
+        <v>100</v>
+      </c>
+      <c r="K20" s="9">
+        <v>41.9</v>
+      </c>
+      <c r="L20" s="9">
+        <v>34.039900000000003</v>
+      </c>
+      <c r="N20" s="12"/>
+    </row>
+    <row r="21" spans="1:14" ht="25" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>16</v>
       </c>
-      <c r="B20">
-        <v>0</v>
-      </c>
-      <c r="D20">
-        <v>4.5</v>
-      </c>
-      <c r="E20" s="3">
-        <v>0.22</v>
-      </c>
-      <c r="F20" s="5">
+      <c r="B21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>24.7</v>
+      </c>
+      <c r="E21" s="3">
+        <v>0.67</v>
+      </c>
+      <c r="F21" s="5">
+        <v>0</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="H21" s="8">
+        <v>0</v>
+      </c>
+      <c r="I21" s="9">
+        <v>0</v>
+      </c>
+      <c r="J21" s="9">
+        <v>80</v>
+      </c>
+      <c r="K21" s="9">
+        <v>41.9</v>
+      </c>
+      <c r="L21" s="9">
+        <v>34.039900000000003</v>
+      </c>
+      <c r="N21" s="12"/>
+    </row>
+    <row r="22" spans="1:14" ht="25" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>17.5</v>
+      </c>
+      <c r="E22" s="3">
+        <v>0.18</v>
+      </c>
+      <c r="F22" s="5">
+        <v>0</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="H22" s="8">
+        <v>0</v>
+      </c>
+      <c r="I22" s="9">
+        <v>0</v>
+      </c>
+      <c r="J22" s="9">
+        <v>130</v>
+      </c>
+      <c r="K22" s="9">
+        <v>41.9</v>
+      </c>
+      <c r="L22" s="9">
+        <v>34.039900000000003</v>
+      </c>
+      <c r="N22" s="12"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>95</v>
+      </c>
+      <c r="E23" s="3">
+        <v>0.35</v>
+      </c>
+      <c r="F23" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="G20" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="H20" s="8">
-        <v>0</v>
-      </c>
-      <c r="I20" s="9">
-        <v>0</v>
-      </c>
-      <c r="J20" s="9">
-        <v>150</v>
-      </c>
-      <c r="K20" s="9"/>
-      <c r="L20" s="9"/>
-    </row>
-    <row r="21" spans="1:12" ht="25" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>17</v>
-      </c>
-      <c r="B21">
-        <v>0</v>
-      </c>
-      <c r="D21">
-        <v>16.399999999999999</v>
-      </c>
-      <c r="E21" s="3">
-        <v>0.1</v>
-      </c>
-      <c r="F21" s="5">
-        <v>0</v>
-      </c>
-      <c r="G21" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="H21" s="8">
-        <v>0</v>
-      </c>
-      <c r="I21" s="9">
-        <v>0</v>
-      </c>
-      <c r="J21" s="9">
-        <v>100</v>
-      </c>
-      <c r="K21" s="9"/>
-      <c r="L21" s="9"/>
-    </row>
-    <row r="22" spans="1:12" ht="25" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>18</v>
-      </c>
-      <c r="B22">
-        <v>0</v>
-      </c>
-      <c r="D22">
-        <v>24.7</v>
-      </c>
-      <c r="E22" s="3">
-        <v>0.67</v>
-      </c>
-      <c r="F22" s="5">
-        <v>0</v>
-      </c>
-      <c r="G22" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="H22" s="8">
-        <v>0</v>
-      </c>
-      <c r="I22" s="9">
-        <v>0</v>
-      </c>
-      <c r="J22" s="9">
-        <v>80</v>
-      </c>
-      <c r="K22" s="9"/>
-      <c r="L22" s="9"/>
-    </row>
-    <row r="23" spans="1:12" ht="25" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+      <c r="G23" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="H23" s="8">
+        <v>0</v>
+      </c>
+      <c r="I23" s="9">
+        <v>0</v>
+      </c>
+      <c r="J23" s="9">
+        <v>120</v>
+      </c>
+      <c r="K23" s="9">
+        <v>41.9</v>
+      </c>
+      <c r="L23" s="9">
+        <v>34.039900000000003</v>
+      </c>
+      <c r="N23" s="12"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>19</v>
       </c>
-      <c r="B23">
-        <v>0</v>
-      </c>
-      <c r="D23">
-        <v>17.5</v>
-      </c>
-      <c r="E23" s="3">
-        <v>0.18</v>
-      </c>
-      <c r="F23" s="5">
-        <v>0</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="H23" s="8">
-        <v>0</v>
-      </c>
-      <c r="I23" s="9">
-        <v>0</v>
-      </c>
-      <c r="J23" s="9">
-        <v>130</v>
-      </c>
-      <c r="K23" s="9"/>
-      <c r="L23" s="9"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>20</v>
-      </c>
       <c r="B24">
         <v>0</v>
       </c>
       <c r="D24">
-        <v>95</v>
+        <v>93.2</v>
       </c>
       <c r="E24" s="3">
         <v>0.35</v>
@@ -1828,7 +1972,7 @@
         <v>2.7E-2</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="H24" s="8">
         <v>0</v>
@@ -1837,23 +1981,28 @@
         <v>0</v>
       </c>
       <c r="J24" s="9">
-        <v>120</v>
-      </c>
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+      <c r="K24" s="9">
+        <v>41.699999999999996</v>
+      </c>
+      <c r="L24" s="9">
+        <v>8.3333000000000013</v>
+      </c>
+      <c r="N24" s="12"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>0.82</v>
       </c>
       <c r="D25">
-        <v>93.2</v>
+        <v>32</v>
       </c>
       <c r="E25" s="3">
-        <v>0.35</v>
+        <v>1</v>
       </c>
       <c r="F25" s="5">
         <v>2.7E-2</v>
@@ -1865,125 +2014,145 @@
         <v>0</v>
       </c>
       <c r="I25" s="9">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="J25" s="9">
-        <v>60</v>
-      </c>
-      <c r="K25" s="9"/>
-      <c r="L25" s="9"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+        <v>0</v>
+      </c>
+      <c r="K25" s="9">
+        <v>41.699999999999996</v>
+      </c>
+      <c r="L25" s="9">
+        <v>8.3333000000000013</v>
+      </c>
+      <c r="N25" s="12"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B26">
-        <v>0.82</v>
+        <v>0</v>
       </c>
       <c r="D26">
-        <v>32</v>
+        <v>7.8</v>
       </c>
       <c r="E26" s="3">
-        <v>1</v>
+        <v>0.36</v>
       </c>
       <c r="F26" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="H26" s="8">
         <v>0</v>
       </c>
       <c r="I26" s="9">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="J26" s="9">
-        <v>0</v>
-      </c>
-      <c r="K26" s="9"/>
-      <c r="L26" s="9"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+        <v>300</v>
+      </c>
+      <c r="K26" s="9">
+        <v>41.699999999999996</v>
+      </c>
+      <c r="L26" s="9">
+        <v>8.3333000000000013</v>
+      </c>
+      <c r="N26" s="12"/>
+    </row>
+    <row r="27" spans="1:14" ht="25" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27">
+        <v>0.38</v>
+      </c>
+      <c r="D27">
+        <v>17</v>
+      </c>
+      <c r="E27" s="3">
+        <v>1.25</v>
+      </c>
+      <c r="F27" s="6">
+        <v>0</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="H27" s="8">
+        <v>0</v>
+      </c>
+      <c r="I27" s="9">
+        <v>0</v>
+      </c>
+      <c r="J27" s="9">
+        <v>150</v>
+      </c>
+      <c r="K27" s="9">
+        <v>41.699999999999996</v>
+      </c>
+      <c r="L27" s="9">
+        <v>8.3333000000000013</v>
+      </c>
+      <c r="N27" s="12"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>23</v>
       </c>
-      <c r="B27">
-        <v>0</v>
-      </c>
-      <c r="D27">
-        <v>7.8</v>
-      </c>
-      <c r="E27" s="3">
-        <v>0.36</v>
-      </c>
-      <c r="F27" s="5">
+      <c r="B28">
+        <v>0</v>
+      </c>
+      <c r="D28">
+        <v>88</v>
+      </c>
+      <c r="E28" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="F28" s="5">
         <v>2.7E-2</v>
       </c>
-      <c r="G27" s="7" t="s">
-        <v>95</v>
-      </c>
-      <c r="H27" s="8">
-        <v>0</v>
-      </c>
-      <c r="I27" s="9">
-        <v>0</v>
-      </c>
-      <c r="J27" s="9">
-        <v>300</v>
-      </c>
-      <c r="K27" s="9"/>
-      <c r="L27" s="9"/>
-    </row>
-    <row r="28" spans="1:12" ht="25" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="G28" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="H28" s="8">
+        <v>1.23</v>
+      </c>
+      <c r="I28" s="9">
+        <v>0</v>
+      </c>
+      <c r="J28" s="9">
+        <v>0</v>
+      </c>
+      <c r="K28" s="9">
+        <v>41.699999999999996</v>
+      </c>
+      <c r="L28" s="9">
+        <v>8.3333000000000013</v>
+      </c>
+      <c r="N28" s="12"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>24</v>
       </c>
-      <c r="B28">
-        <v>0.38</v>
-      </c>
-      <c r="D28">
-        <v>17</v>
-      </c>
-      <c r="E28" s="3">
-        <v>1.25</v>
-      </c>
-      <c r="F28" s="6">
-        <v>0</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="H28" s="8">
-        <v>0</v>
-      </c>
-      <c r="I28" s="9">
-        <v>0</v>
-      </c>
-      <c r="J28" s="9">
-        <v>150</v>
-      </c>
-      <c r="K28" s="9"/>
-      <c r="L28" s="9"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>25</v>
-      </c>
       <c r="B29">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="D29">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E29" s="3">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="F29" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H29" s="8">
         <v>1.23</v>
@@ -1994,10 +2163,15 @@
       <c r="J29" s="9">
         <v>0</v>
       </c>
-      <c r="K29" s="9"/>
-      <c r="L29" s="9"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K29" s="9">
+        <v>41.699999999999996</v>
+      </c>
+      <c r="L29" s="9">
+        <v>8.3333000000000013</v>
+      </c>
+      <c r="N29" s="12"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>26</v>
       </c>
@@ -2005,16 +2179,16 @@
         <v>0.08</v>
       </c>
       <c r="D30">
-        <v>87</v>
+        <v>18</v>
       </c>
       <c r="E30" s="3">
-        <v>3.6</v>
+        <v>0.5</v>
       </c>
       <c r="F30" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H30" s="8">
         <v>1.23</v>
@@ -2025,27 +2199,32 @@
       <c r="J30" s="9">
         <v>0</v>
       </c>
-      <c r="K30" s="9"/>
-      <c r="L30" s="9"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K30" s="9">
+        <v>41.699999999999996</v>
+      </c>
+      <c r="L30" s="9">
+        <v>8.3333000000000013</v>
+      </c>
+      <c r="N30" s="12"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B31">
-        <v>0.08</v>
+        <v>0</v>
       </c>
       <c r="D31">
-        <v>18</v>
+        <v>88</v>
       </c>
       <c r="E31" s="3">
-        <v>0.5</v>
+        <v>3.6</v>
       </c>
       <c r="F31" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G31" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H31" s="8">
         <v>1.23</v>
@@ -2056,10 +2235,15 @@
       <c r="J31" s="9">
         <v>0</v>
       </c>
-      <c r="K31" s="9"/>
-      <c r="L31" s="9"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K31" s="9">
+        <v>41.699999999999996</v>
+      </c>
+      <c r="L31" s="9">
+        <v>8.3333000000000013</v>
+      </c>
+      <c r="N31" s="12"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>27</v>
       </c>
@@ -2067,16 +2251,16 @@
         <v>0</v>
       </c>
       <c r="D32">
-        <v>88</v>
+        <v>87.7</v>
       </c>
       <c r="E32" s="3">
-        <v>3.6</v>
+        <v>1.5</v>
       </c>
       <c r="F32" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H32" s="8">
         <v>1.23</v>
@@ -2087,27 +2271,32 @@
       <c r="J32" s="9">
         <v>0</v>
       </c>
-      <c r="K32" s="9"/>
-      <c r="L32" s="9"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K32" s="9">
+        <v>75.900000000000006</v>
+      </c>
+      <c r="L32" s="9">
+        <v>2.9558999999999997</v>
+      </c>
+      <c r="N32" s="12"/>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B33">
         <v>0</v>
       </c>
       <c r="D33">
-        <v>87.7</v>
+        <v>10.3</v>
       </c>
       <c r="E33" s="3">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="F33" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H33" s="8">
         <v>1.23</v>
@@ -2118,27 +2307,32 @@
       <c r="J33" s="9">
         <v>0</v>
       </c>
-      <c r="K33" s="9"/>
-      <c r="L33" s="9"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K33" s="9">
+        <v>41.666699999999999</v>
+      </c>
+      <c r="L33" s="9">
+        <v>8.3333000000000013</v>
+      </c>
+      <c r="N33" s="12"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B34">
         <v>0</v>
       </c>
       <c r="D34">
-        <v>10.3</v>
+        <v>90</v>
       </c>
       <c r="E34" s="3">
-        <v>0.5</v>
+        <v>6</v>
       </c>
       <c r="F34" s="5">
         <v>2.7E-2</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="H34" s="8">
         <v>1.23</v>
@@ -2149,30 +2343,35 @@
       <c r="J34" s="9">
         <v>0</v>
       </c>
-      <c r="K34" s="9"/>
-      <c r="L34" s="9"/>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="K34" s="9">
+        <v>47.571100000000001</v>
+      </c>
+      <c r="L34" s="9">
+        <v>7.1374999999999993</v>
+      </c>
+      <c r="N34" s="12"/>
+    </row>
+    <row r="35" spans="1:14" ht="25" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B35">
         <v>0</v>
       </c>
       <c r="D35">
-        <v>90</v>
+        <v>17.7</v>
       </c>
       <c r="E35" s="3">
-        <v>6</v>
+        <v>2.8</v>
       </c>
       <c r="F35" s="5">
-        <v>2.7E-2</v>
+        <v>0</v>
       </c>
       <c r="G35" s="7" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="H35" s="8">
-        <v>1.23</v>
+        <v>1.47</v>
       </c>
       <c r="I35" s="9">
         <v>0</v>
@@ -2180,70 +2379,52 @@
       <c r="J35" s="9">
         <v>0</v>
       </c>
-      <c r="K35" s="9"/>
-      <c r="L35" s="9"/>
-    </row>
-    <row r="36" spans="1:12" ht="25" x14ac:dyDescent="0.35">
+      <c r="K35" s="9">
+        <v>41.666699999999999</v>
+      </c>
+      <c r="L35" s="9">
+        <v>8.3333000000000013</v>
+      </c>
+      <c r="N35" s="12"/>
+    </row>
+    <row r="36" spans="1:14" ht="25" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B36">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="D36">
-        <v>17.7</v>
+        <v>86</v>
       </c>
       <c r="E36" s="3">
-        <v>2.8</v>
-      </c>
-      <c r="F36" s="5">
+        <v>2.0499999999999998</v>
+      </c>
+      <c r="F36" s="6">
         <v>0</v>
       </c>
       <c r="G36" s="7" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="H36" s="8">
-        <v>1.47</v>
+        <v>0.36749999999999999</v>
       </c>
       <c r="I36" s="9">
         <v>0</v>
       </c>
       <c r="J36" s="9">
-        <v>0</v>
-      </c>
-      <c r="K36" s="9"/>
-      <c r="L36" s="9"/>
-    </row>
-    <row r="37" spans="1:12" ht="25" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>39</v>
-      </c>
-      <c r="B37">
-        <v>0.25</v>
-      </c>
-      <c r="D37">
-        <v>86</v>
-      </c>
-      <c r="E37" s="3">
-        <v>2.0499999999999998</v>
-      </c>
-      <c r="F37" s="6">
-        <v>0</v>
-      </c>
-      <c r="G37" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="H37" s="8">
-        <v>0.36749999999999999</v>
-      </c>
-      <c r="I37" s="9">
-        <v>0</v>
-      </c>
-      <c r="J37" s="9">
         <v>150</v>
       </c>
-      <c r="K37" s="9"/>
-      <c r="L37" s="9"/>
+      <c r="K36" s="9">
+        <v>44.618900000000004</v>
+      </c>
+      <c r="L36" s="9">
+        <v>7.7354000000000003</v>
+      </c>
+      <c r="N36" s="12"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="N37" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2257,114 +2438,114 @@
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" t="s">
         <v>104</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>105</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>106</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>107</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>108</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>109</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>110</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>111</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>112</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>113</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>114</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>115</v>
       </c>
-      <c r="M1" t="s">
+      <c r="P1" t="s">
         <v>116</v>
       </c>
-      <c r="N1" t="s">
+      <c r="Q1" t="s">
         <v>117</v>
       </c>
-      <c r="O1" t="s">
+      <c r="R1" t="s">
         <v>118</v>
       </c>
-      <c r="P1" t="s">
+      <c r="S1" t="s">
         <v>119</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="T1" t="s">
         <v>120</v>
       </c>
-      <c r="R1" t="s">
+      <c r="U1" t="s">
         <v>121</v>
       </c>
-      <c r="S1" t="s">
+      <c r="V1" t="s">
         <v>122</v>
       </c>
-      <c r="T1" t="s">
+      <c r="W1" t="s">
         <v>123</v>
       </c>
-      <c r="U1" t="s">
+      <c r="X1" t="s">
         <v>124</v>
       </c>
-      <c r="V1" t="s">
+      <c r="Y1" t="s">
         <v>125</v>
       </c>
-      <c r="W1" t="s">
+      <c r="Z1" t="s">
         <v>126</v>
       </c>
-      <c r="X1" t="s">
+      <c r="AA1" t="s">
         <v>127</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="AB1" t="s">
         <v>128</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AC1" t="s">
         <v>129</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AD1" t="s">
         <v>130</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AE1" t="s">
         <v>131</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AF1" t="s">
         <v>132</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AG1" t="s">
         <v>133</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AH1" t="s">
         <v>134</v>
       </c>
-      <c r="AF1" t="s">
-        <v>135</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>136</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>137</v>
-      </c>
       <c r="AI1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B2">
         <v>877</v>
@@ -2588,417 +2769,417 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B1" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B2">
         <v>3.0999999999999999E-3</v>
       </c>
       <c r="C2" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D2" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B3">
         <v>2.5026398888888901E-3</v>
       </c>
       <c r="C3" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="B4">
         <v>2.5191576000000004E-3</v>
       </c>
       <c r="C4" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D4" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B5">
         <v>3.4014885333333339E-3</v>
       </c>
       <c r="C5" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D5" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B6">
         <v>8.9999999999999998E-4</v>
       </c>
       <c r="C6" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D6" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B7">
         <v>5.5000000000000003E-4</v>
       </c>
       <c r="C7" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D7" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B8">
         <v>5.5731720329999998E-4</v>
       </c>
       <c r="C8" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D8" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B9">
         <v>2.8934473500000003E-3</v>
       </c>
       <c r="C9" t="s">
+        <v>159</v>
+      </c>
+      <c r="D9" t="s">
         <v>162</v>
-      </c>
-      <c r="D9" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B10">
         <v>2.5331492083333334E-3</v>
       </c>
       <c r="C10" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D10" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B11">
         <v>2.5165149883414934E-3</v>
       </c>
       <c r="C11" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D11" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B12">
         <v>2.44344375E-3</v>
       </c>
       <c r="C12" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D12" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="B13">
         <v>2.2090262539682538E-3</v>
       </c>
       <c r="C13" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D13" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="B14">
         <v>5.8E-4</v>
       </c>
       <c r="C14" t="s">
+        <v>160</v>
+      </c>
+      <c r="D14" t="s">
         <v>163</v>
-      </c>
-      <c r="D14" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B15">
         <v>5.5000000000000003E-4</v>
       </c>
       <c r="C15" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D15" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B16">
         <v>4.4999999999999999E-4</v>
       </c>
       <c r="C16" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D16" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B17">
         <v>7.5000000000000002E-4</v>
       </c>
       <c r="C17" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D17" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B18">
         <v>2.0631828E-4</v>
       </c>
       <c r="C18" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D18" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="B19">
         <v>5.4262139775921735E-4</v>
       </c>
       <c r="C19" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D19" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B20">
         <v>2.3440000000000003E-4</v>
       </c>
       <c r="C20" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D20" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B21">
         <v>2.9231999999999999E-4</v>
       </c>
       <c r="C21" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D21" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B22">
         <v>1.5964523839999997E-3</v>
       </c>
       <c r="C22" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D22" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B23">
         <v>1.8285932799999999E-3</v>
       </c>
       <c r="C23" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D23" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B24">
         <v>3.6662312908139748E-4</v>
       </c>
       <c r="C24" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D24" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E24" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="B25">
         <v>3.6662312908139748E-4</v>
       </c>
       <c r="C25" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D25" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B26">
         <v>1.1635199999999999E-3</v>
       </c>
       <c r="C26" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D26" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E26" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B27">
         <v>1.1635199999999999E-3</v>
       </c>
       <c r="C27" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D27" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B28">
         <v>5.7248880000000007E-4</v>
       </c>
       <c r="C28" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D28" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E28" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B29">
         <v>5.7248880000000007E-4</v>
       </c>
       <c r="C29" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D29" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -3008,7 +3189,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3D8FFD4-4EA9-47C1-BA4E-47263EF1D3B0}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="25.08984375" customWidth="1"/>
@@ -3018,284 +3199,339 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B1" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D1" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="B2">
         <v>6.7174054999999996E-4</v>
       </c>
       <c r="C2" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B3">
         <v>5.0052599999999992E-3</v>
       </c>
       <c r="C3" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="B4">
         <v>5.0052599999999992E-3</v>
       </c>
       <c r="C4" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D4" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="B5">
         <v>4.3945200000000007E-3</v>
       </c>
       <c r="C5" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="B6">
         <v>1.1705850000000001E-4</v>
       </c>
       <c r="C6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="B7">
         <v>6.7174054999999996E-4</v>
       </c>
       <c r="C7" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D7" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="B8">
-        <v>2.0631828E-4</v>
+        <v>2.0569932516000002E-4</v>
       </c>
       <c r="C8" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="B9">
-        <v>5.4262139775921735E-4</v>
+        <v>6.5601400315309921E-4</v>
       </c>
       <c r="C9" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B10">
-        <v>2.3440000000000003E-4</v>
+        <v>2.3369680000000001E-4</v>
       </c>
       <c r="C10" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="B11">
-        <v>2.9231999999999999E-4</v>
+        <v>3.9241920000000004E-4</v>
       </c>
       <c r="C11" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B12">
-        <v>1.5964523839999997E-3</v>
+        <v>1.5916630268479996E-3</v>
       </c>
       <c r="C12" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="B13">
-        <v>1.8285932799999999E-3</v>
+        <v>1.8231075001599998E-3</v>
       </c>
       <c r="C13" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="B14">
-        <v>3.6662312908139748E-4</v>
+        <v>3.795876976509448E-4</v>
       </c>
       <c r="C14" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D14" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="B15">
-        <v>3.6662312908139748E-4</v>
+        <v>3.795876976509448E-4</v>
       </c>
       <c r="C15" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="B16">
-        <v>1.1635199999999999E-3</v>
+        <v>1.1600294399999999E-3</v>
       </c>
       <c r="C16" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D16" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="B17">
-        <v>1.1635199999999999E-3</v>
+        <v>1.1600294399999999E-3</v>
       </c>
       <c r="C17" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="B18">
-        <v>5.7248880000000007E-4</v>
+        <v>5.7077133360000014E-4</v>
       </c>
       <c r="C18" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="D18" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="B19">
-        <v>5.7248880000000007E-4</v>
+        <v>5.7077133360000014E-4</v>
       </c>
       <c r="C19" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>6</v>
+        <v>203</v>
       </c>
       <c r="B20">
         <v>1.9282590170888892E-3</v>
       </c>
       <c r="C20" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>204</v>
       </c>
       <c r="B21">
-        <v>7.789160266200002E-4</v>
+        <v>1.9282590170888892E-3</v>
       </c>
       <c r="C21" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>153</v>
+        <v>205</v>
       </c>
       <c r="B22">
-        <v>5.5731720329999998E-4</v>
+        <v>1.9282590170888892E-3</v>
       </c>
       <c r="C22" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>206</v>
       </c>
       <c r="B23">
-        <v>2.5331492083333334E-3</v>
+        <v>1.9282590170888892E-3</v>
       </c>
       <c r="C23" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>178</v>
+        <v>141</v>
       </c>
       <c r="B24">
+        <v>1.9282590170888892E-3</v>
+      </c>
+      <c r="C24" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>207</v>
+      </c>
+      <c r="B25">
+        <v>1.9282590170888892E-3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26">
+        <v>7.789160266200002E-4</v>
+      </c>
+      <c r="C26" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>150</v>
+      </c>
+      <c r="B27">
+        <v>5.5731720329999998E-4</v>
+      </c>
+      <c r="C27" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28">
+        <v>2.5331492083333334E-3</v>
+      </c>
+      <c r="C28" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>175</v>
+      </c>
+      <c r="B29">
         <v>2.5165149883414934E-3</v>
       </c>
-      <c r="C24" t="s">
-        <v>164</v>
+      <c r="C29" t="s">
+        <v>161</v>
       </c>
     </row>
   </sheetData>
@@ -3313,15 +3549,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B2">
         <v>0</v>
@@ -3329,7 +3565,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B3">
         <v>0.06</v>
@@ -3337,7 +3573,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B4">
         <v>0.02</v>
@@ -3345,7 +3581,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="B5">
         <v>0.09</v>
@@ -3353,7 +3589,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="B6">
         <v>0.04</v>
@@ -3361,7 +3597,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -3369,7 +3605,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B8">
         <v>0</v>
@@ -3377,7 +3613,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -3385,7 +3621,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B10">
         <v>0.79</v>
@@ -3403,114 +3639,114 @@
   <sheetData>
     <row r="1" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D1" t="s">
         <v>104</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>105</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" t="s">
         <v>106</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>107</v>
       </c>
-      <c r="E1" t="s">
+      <c r="H1" t="s">
         <v>108</v>
       </c>
-      <c r="F1" t="s">
+      <c r="I1" t="s">
         <v>109</v>
       </c>
-      <c r="G1" t="s">
+      <c r="J1" t="s">
         <v>110</v>
       </c>
-      <c r="H1" t="s">
+      <c r="K1" t="s">
         <v>111</v>
       </c>
-      <c r="I1" t="s">
+      <c r="L1" t="s">
         <v>112</v>
       </c>
-      <c r="J1" t="s">
+      <c r="M1" t="s">
         <v>113</v>
       </c>
-      <c r="K1" t="s">
+      <c r="N1" t="s">
         <v>114</v>
       </c>
-      <c r="L1" t="s">
+      <c r="O1" t="s">
         <v>115</v>
       </c>
-      <c r="M1" t="s">
+      <c r="P1" t="s">
         <v>116</v>
       </c>
-      <c r="N1" t="s">
+      <c r="Q1" t="s">
         <v>117</v>
       </c>
-      <c r="O1" t="s">
+      <c r="R1" t="s">
         <v>118</v>
       </c>
-      <c r="P1" t="s">
+      <c r="S1" t="s">
         <v>119</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="T1" t="s">
         <v>120</v>
       </c>
-      <c r="R1" t="s">
+      <c r="U1" t="s">
         <v>121</v>
       </c>
-      <c r="S1" t="s">
+      <c r="V1" t="s">
         <v>122</v>
       </c>
-      <c r="T1" t="s">
+      <c r="W1" t="s">
         <v>123</v>
       </c>
-      <c r="U1" t="s">
+      <c r="X1" t="s">
         <v>124</v>
       </c>
-      <c r="V1" t="s">
+      <c r="Y1" t="s">
         <v>125</v>
       </c>
-      <c r="W1" t="s">
+      <c r="Z1" t="s">
         <v>126</v>
       </c>
-      <c r="X1" t="s">
+      <c r="AA1" t="s">
         <v>127</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="AB1" t="s">
         <v>128</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AC1" t="s">
         <v>129</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AD1" t="s">
         <v>130</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AE1" t="s">
         <v>131</v>
       </c>
-      <c r="AC1" t="s">
+      <c r="AF1" t="s">
         <v>132</v>
       </c>
-      <c r="AD1" t="s">
+      <c r="AG1" t="s">
         <v>133</v>
       </c>
-      <c r="AE1" t="s">
+      <c r="AH1" t="s">
         <v>134</v>
       </c>
-      <c r="AF1" t="s">
-        <v>135</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>136</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>137</v>
-      </c>
       <c r="AI1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B2">
         <v>92.113959999999992</v>
@@ -3617,7 +3853,7 @@
     </row>
     <row r="3" spans="1:35" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B3">
         <v>58.260291000000002</v>
@@ -3740,58 +3976,59 @@
     <col min="7" max="7" width="24.453125" customWidth="1"/>
     <col min="8" max="8" width="18.1796875" customWidth="1"/>
     <col min="9" max="9" width="18.453125" customWidth="1"/>
+    <col min="14" max="14" width="18.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" t="s">
+        <v>80</v>
+      </c>
+      <c r="F1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G1" t="s">
+        <v>78</v>
+      </c>
+      <c r="H1" t="s">
+        <v>75</v>
+      </c>
+      <c r="I1" t="s">
+        <v>76</v>
+      </c>
+      <c r="J1" t="s">
         <v>77</v>
       </c>
-      <c r="D1" t="s">
-        <v>48</v>
-      </c>
-      <c r="E1" t="s">
+      <c r="K1" t="s">
+        <v>82</v>
+      </c>
+      <c r="L1" t="s">
         <v>83</v>
       </c>
-      <c r="F1" t="s">
-        <v>82</v>
-      </c>
-      <c r="G1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H1" t="s">
-        <v>78</v>
-      </c>
-      <c r="I1" t="s">
-        <v>79</v>
-      </c>
-      <c r="J1" t="s">
-        <v>80</v>
-      </c>
-      <c r="K1" t="s">
-        <v>85</v>
-      </c>
-      <c r="L1" t="s">
-        <v>86</v>
-      </c>
       <c r="M1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="N1" t="s">
-        <v>183</v>
+        <v>208</v>
       </c>
       <c r="O1" t="s">
-        <v>184</v>
+        <v>209</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B2">
         <f>1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -3841,7 +4078,7 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B3">
         <f>1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -3891,7 +4128,7 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B4">
         <f t="shared" ref="B4:B7" si="2">1-(1-0.3)*(1-0.05)*(1-0.2)</f>
@@ -3941,7 +4178,7 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B5">
         <f t="shared" si="2"/>
@@ -3991,7 +4228,7 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B6">
         <f>1-(1-0.5)*(1-0.2)*(1-0.2)</f>
@@ -4041,7 +4278,7 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B7">
         <f t="shared" si="2"/>
@@ -4109,31 +4346,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" t="s">
         <v>49</v>
       </c>
-      <c r="B1" t="s">
+      <c r="E1" t="s">
         <v>50</v>
       </c>
-      <c r="C1" t="s">
+      <c r="F1" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" t="s">
+      <c r="G1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" t="s">
-        <v>53</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="G1" t="s">
-        <v>55</v>
-      </c>
       <c r="H1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -4159,7 +4396,7 @@
         <v>54417</v>
       </c>
       <c r="H2" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I2" s="1">
         <f>2*14/(2*14+16)*(0.01164*B2+0.00594*C2+0.00594*F2)/(B2+C2+F2)*100</f>
@@ -4189,7 +4426,7 @@
         <v>266265</v>
       </c>
       <c r="H3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="I3" s="1">
         <f t="shared" ref="I3:I24" si="0">2*14/(2*14+16)*(0.01164*B3+0.00594*C3+0.00594*F3)/(B3+C3+F3)*100</f>
@@ -4219,7 +4456,7 @@
         <v>168251</v>
       </c>
       <c r="H4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I4" s="1">
         <f t="shared" si="0"/>
@@ -4249,7 +4486,7 @@
         <v>80548</v>
       </c>
       <c r="H5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="I5" s="1">
         <f t="shared" si="0"/>
@@ -4279,7 +4516,7 @@
         <v>256528</v>
       </c>
       <c r="H6" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="I6" s="1">
         <f t="shared" si="0"/>
@@ -4309,7 +4546,7 @@
         <v>74606</v>
       </c>
       <c r="H7" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I7" s="1">
         <f t="shared" si="0"/>
@@ -4339,7 +4576,7 @@
         <v>96358</v>
       </c>
       <c r="H8" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I8" s="1">
         <f t="shared" si="0"/>
@@ -4369,7 +4606,7 @@
         <v>87002</v>
       </c>
       <c r="H9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="I9" s="1">
         <f t="shared" si="0"/>
@@ -4399,7 +4636,7 @@
         <v>116150</v>
       </c>
       <c r="H10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="I10" s="1">
         <f t="shared" si="0"/>
@@ -4429,7 +4666,7 @@
         <v>35716</v>
       </c>
       <c r="H11" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="I11" s="1">
         <f t="shared" si="0"/>
@@ -4459,7 +4696,7 @@
         <v>29157</v>
       </c>
       <c r="H12" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="I12" s="1">
         <f t="shared" si="0"/>
@@ -4489,7 +4726,7 @@
         <v>141243</v>
       </c>
       <c r="H13" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="I13" s="1">
         <f t="shared" si="0"/>
@@ -4519,7 +4756,7 @@
         <v>111801</v>
       </c>
       <c r="H14" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I14" s="1">
         <f t="shared" si="0"/>
@@ -4549,7 +4786,7 @@
         <v>184174</v>
       </c>
       <c r="H15" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I15" s="1">
         <f t="shared" si="0"/>
@@ -4579,7 +4816,7 @@
         <v>133267</v>
       </c>
       <c r="H16" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I16" s="1">
         <f t="shared" si="0"/>
@@ -4609,7 +4846,7 @@
         <v>135672</v>
       </c>
       <c r="H17" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I17" s="1">
         <f t="shared" si="0"/>
@@ -4639,7 +4876,7 @@
         <v>18541</v>
       </c>
       <c r="H18" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I18" s="1">
         <f t="shared" si="0"/>
@@ -4669,7 +4906,7 @@
         <v>66736</v>
       </c>
       <c r="H19" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="I19" s="1">
         <f t="shared" si="0"/>
@@ -4699,7 +4936,7 @@
         <v>50349</v>
       </c>
       <c r="H20" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I20" s="1">
         <f>2*14/(2*14+16)*(0.01164*B20+0.00594*C20+0.00594*F20)/(B20+C20+F20)*100</f>
@@ -4729,7 +4966,7 @@
         <v>31445</v>
       </c>
       <c r="H21" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I21" s="1">
         <f t="shared" si="0"/>
@@ -4759,7 +4996,7 @@
         <v>21502</v>
       </c>
       <c r="H22" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="I22" s="1">
         <f t="shared" si="0"/>
@@ -4778,7 +5015,7 @@
       </c>
       <c r="F23" s="2"/>
       <c r="H23" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I23" s="1">
         <f t="shared" si="0"/>
@@ -4787,7 +5024,7 @@
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B24">
         <v>924490</v>
@@ -4808,7 +5045,7 @@
         <v>2205890</v>
       </c>
       <c r="H24" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="I24" s="1">
         <f t="shared" si="0"/>

</xml_diff>